<commit_message>
Reformatted some radial field plots for report
</commit_message>
<xml_diff>
--- a/Sheets/ErrorTableRun1.xlsx
+++ b/Sheets/ErrorTableRun1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8ECD9E4-0F55-3847-AC0E-913590430E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62108EEF-619C-244A-8143-4D51FFFE6C4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-1000" yWindow="-19500" windowWidth="13120" windowHeight="16940" xr2:uid="{C29EF40E-6384-C447-AF4D-92516C1B0710}"/>
   </bookViews>
@@ -54,6 +54,9 @@
     <t xml:space="preserve">Dilution correction </t>
   </si>
   <si>
+    <t xml:space="preserve">Weighted fit  </t>
+  </si>
+  <si>
     <t>Total</t>
   </si>
   <si>
@@ -64,9 +67,6 @@
   </si>
   <si>
     <t>Average</t>
-  </si>
-  <si>
-    <t>Fit to delta'(p) (stat)</t>
   </si>
 </sst>
 </file>
@@ -449,7 +449,7 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G1" s="3"/>
       <c r="I1" s="3"/>
@@ -498,7 +498,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2">
         <v>2.4563299999999999E-19</v>
@@ -519,7 +519,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" s="1">
         <v>2.6240419999999998E-19</v>
@@ -540,7 +540,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8" s="1">
         <v>1.060207E-19</v>
@@ -548,7 +548,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1">
         <f>SQRT(B5^2+C5^2+D5^2+E5^2)/4</f>

</xml_diff>

<commit_message>
Work on alignment and dilution prior to 8th Feb EDM meeting
</commit_message>
<xml_diff>
--- a/Sheets/ErrorTableRun1.xlsx
+++ b/Sheets/ErrorTableRun1.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED92E986-E6B2-7A4A-92A3-97ADFC3C9EF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C59DC84-61E9-9548-9089-53C975EE2EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{C29EF40E-6384-C447-AF4D-92516C1B0710}"/>
   </bookViews>
   <sheets>
-    <sheet name="Run-1 (v2) (HS refit)" sheetId="14" r:id="rId1"/>
-    <sheet name="Run-1 (v2) (HS reweight refit)" sheetId="13" r:id="rId2"/>
-    <sheet name="Run-1 (v2) (HS reweight)" sheetId="12" r:id="rId3"/>
+    <sheet name="Run-1 (v2) (HS reweight refit)" sheetId="13" r:id="rId1"/>
+    <sheet name="Run-1 (v2) (HS reweight)" sheetId="12" r:id="rId2"/>
+    <sheet name="Run-1 (v2) (HS refit)" sheetId="14" r:id="rId3"/>
     <sheet name="Run-1 (v2) (HS)" sheetId="11" r:id="rId4"/>
     <sheet name="Run-1 (v2)" sheetId="6" r:id="rId5"/>
     <sheet name="Run-1 (v1)" sheetId="1" r:id="rId6"/>
@@ -706,6 +706,2100 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2695A833-57C4-DC4E-AC5C-0BDB90378BCB}">
+  <dimension ref="A1:R29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="22">
+        <f>N6</f>
+        <v>1.49629E-18</v>
+      </c>
+      <c r="C2" s="22">
+        <f>N12</f>
+        <v>1.37313E-18</v>
+      </c>
+      <c r="D2" s="22">
+        <f>N18</f>
+        <v>2.2958900000000001E-18</v>
+      </c>
+      <c r="E2" s="22">
+        <f>N24</f>
+        <v>1.8930599999999998E-18</v>
+      </c>
+      <c r="F2" s="1">
+        <f>SQRT(B2^2+C2^2+D2^2+E2^2)/4</f>
+        <v>9.0066492162388003E-19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="24">
+        <f>R6</f>
+        <v>2.8764699999999999E-19</v>
+      </c>
+      <c r="C3" s="24">
+        <f>R12</f>
+        <v>2.4680000000000001E-19</v>
+      </c>
+      <c r="D3" s="24">
+        <f>R18</f>
+        <v>2.3704400000000001E-19</v>
+      </c>
+      <c r="E3" s="24">
+        <f>R24</f>
+        <v>1.8167600000000001E-19</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F4" si="0">SQRT(B3^2+C3^2+D3^2+E3^2)/4</f>
+        <v>1.2063557298766603E-19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="23">
+        <f>B3/B2</f>
+        <v>0.19224014061445308</v>
+      </c>
+      <c r="C4" s="23">
+        <f t="shared" ref="C4:E4" si="1">C3/C2</f>
+        <v>0.17973534916577455</v>
+      </c>
+      <c r="D4" s="23">
+        <f t="shared" si="1"/>
+        <v>0.10324710678647496</v>
+      </c>
+      <c r="E4" s="28">
+        <f t="shared" si="1"/>
+        <v>9.5969488552924906E-2</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
+        <v>7.4637111745806173E-2</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4">
+        <v>0.654451</v>
+      </c>
+      <c r="J4">
+        <v>0.111583</v>
+      </c>
+      <c r="K4">
+        <v>4.8462999999999999E-2</v>
+      </c>
+      <c r="L4">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M4">
+        <v>0.121836</v>
+      </c>
+      <c r="N4" s="1">
+        <v>2.0242400000000001E-18</v>
+      </c>
+      <c r="O4" s="1">
+        <v>3.5619899999999999E-19</v>
+      </c>
+      <c r="P4" s="1">
+        <v>1.54705E-19</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R4" s="1">
+        <v>3.8892800000000001E-19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" s="37"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="H5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5">
+        <v>0.30299100000000001</v>
+      </c>
+      <c r="J5">
+        <v>0.126971</v>
+      </c>
+      <c r="K5">
+        <v>5.0055000000000002E-2</v>
+      </c>
+      <c r="L5">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M5">
+        <v>0.13664499999999999</v>
+      </c>
+      <c r="N5" s="1">
+        <v>9.0230500000000007E-19</v>
+      </c>
+      <c r="O5" s="1">
+        <v>4.0532099999999998E-19</v>
+      </c>
+      <c r="P5" s="1">
+        <v>1.5978799999999999E-19</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R5" s="1">
+        <v>4.3620000000000004E-19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A6" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="38"/>
+      <c r="F6" s="1"/>
+      <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6">
+        <v>0.489064</v>
+      </c>
+      <c r="J6">
+        <v>8.4459999999999993E-2</v>
+      </c>
+      <c r="K6">
+        <v>3.0686000000000001E-2</v>
+      </c>
+      <c r="L6">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M6">
+        <v>9.0108999999999995E-2</v>
+      </c>
+      <c r="N6" s="1">
+        <v>1.49629E-18</v>
+      </c>
+      <c r="O6" s="1">
+        <v>2.69614E-19</v>
+      </c>
+      <c r="P6" s="1">
+        <v>9.7956499999999994E-20</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R6" s="1">
+        <v>2.8764699999999999E-19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A8" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="22">
+        <f>L4</f>
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="C8" s="22">
+        <f>L12</f>
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="D8" s="22">
+        <f>L18</f>
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="E8" s="22">
+        <f>L24</f>
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="F8" s="1">
+        <f>SQRT(B10^2+C10^2+D10^2+E10^2)/4</f>
+        <v>7.0562593169518437E-3</v>
+      </c>
+      <c r="I8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A9" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="24">
+        <f>Q6</f>
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="C9" s="24">
+        <f>Q12</f>
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="D9" s="24">
+        <f>Q18</f>
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="E9" s="24">
+        <f>Q24</f>
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="F9" s="1">
+        <f>SQRT(B11^2+C11^2+D11^2+E11^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" t="s">
+        <v>25</v>
+      </c>
+      <c r="J9" t="s">
+        <v>26</v>
+      </c>
+      <c r="K9" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" t="s">
+        <v>28</v>
+      </c>
+      <c r="M9" t="s">
+        <v>29</v>
+      </c>
+      <c r="N9" t="s">
+        <v>25</v>
+      </c>
+      <c r="O9" t="s">
+        <v>26</v>
+      </c>
+      <c r="P9" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>28</v>
+      </c>
+      <c r="R9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A10" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="28">
+        <f>B9/B2</f>
+        <v>1.4232601968869671E-2</v>
+      </c>
+      <c r="C10" s="28">
+        <f>C9/C2</f>
+        <v>1.7521938927850967E-2</v>
+      </c>
+      <c r="D10" s="28">
+        <f>D9/D2</f>
+        <v>1.0540966683943918E-2</v>
+      </c>
+      <c r="E10" s="28">
+        <f>E9/E2</f>
+        <v>1.3264819921185805E-2</v>
+      </c>
+      <c r="F10" s="3">
+        <f>SQRT(B12^2+C12^2+D12^2+E12^2)/4</f>
+        <v>1.7168382695379316E-2</v>
+      </c>
+      <c r="H10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10">
+        <v>0.37874000000000002</v>
+      </c>
+      <c r="J10">
+        <v>9.5302999999999999E-2</v>
+      </c>
+      <c r="K10">
+        <v>2.8292999999999999E-2</v>
+      </c>
+      <c r="L10">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M10">
+        <v>9.9699999999999997E-2</v>
+      </c>
+      <c r="N10" s="1">
+        <v>1.14197E-18</v>
+      </c>
+      <c r="O10" s="1">
+        <v>3.0422899999999999E-19</v>
+      </c>
+      <c r="P10" s="1">
+        <v>9.0318600000000001E-20</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R10" s="1">
+        <v>3.1826299999999998E-19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A11" s="36"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="H11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11">
+        <v>0.51285000000000003</v>
+      </c>
+      <c r="J11">
+        <v>0.108587</v>
+      </c>
+      <c r="K11">
+        <v>5.8909000000000003E-2</v>
+      </c>
+      <c r="L11">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M11">
+        <v>0.123767</v>
+      </c>
+      <c r="N11" s="1">
+        <v>1.57008E-18</v>
+      </c>
+      <c r="O11" s="1">
+        <v>3.4663400000000001E-19</v>
+      </c>
+      <c r="P11" s="1">
+        <v>1.88051E-19</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R11" s="1">
+        <v>3.9509099999999998E-19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A12" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="24">
+        <f>K6</f>
+        <v>3.0686000000000001E-2</v>
+      </c>
+      <c r="C12" s="22">
+        <f>K12</f>
+        <v>2.6641000000000001E-2</v>
+      </c>
+      <c r="D12" s="22">
+        <f>K18</f>
+        <v>4.2286999999999998E-2</v>
+      </c>
+      <c r="E12" s="22">
+        <f>K24</f>
+        <v>3.5728000000000003E-2</v>
+      </c>
+      <c r="F12" s="1">
+        <f>SQRT(B14^2+C14^2+D14^2+E14^2)/4</f>
+        <v>3.0830559026828703E-2</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12">
+        <v>0.45115100000000002</v>
+      </c>
+      <c r="J12">
+        <v>7.2184999999999999E-2</v>
+      </c>
+      <c r="K12">
+        <v>2.6641000000000001E-2</v>
+      </c>
+      <c r="L12">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M12">
+        <v>7.7313000000000007E-2</v>
+      </c>
+      <c r="N12" s="1">
+        <v>1.37313E-18</v>
+      </c>
+      <c r="O12" s="1">
+        <v>2.3043099999999998E-19</v>
+      </c>
+      <c r="P12" s="1">
+        <v>8.5044799999999996E-20</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R12" s="1">
+        <v>2.4680000000000001E-19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A13" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="24">
+        <f>P6</f>
+        <v>9.7956499999999994E-20</v>
+      </c>
+      <c r="C13" s="24">
+        <f>P12</f>
+        <v>8.5044799999999996E-20</v>
+      </c>
+      <c r="D13" s="24">
+        <f>P18</f>
+        <v>1.3498799999999999E-19</v>
+      </c>
+      <c r="E13" s="24">
+        <f>P24</f>
+        <v>1.14051E-19</v>
+      </c>
+      <c r="F13" s="1">
+        <f>SQRT(B15^2+C15^2+D15^2+E15^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="28">
+        <f>B13/B2</f>
+        <v>6.5466253199580299E-2</v>
+      </c>
+      <c r="C14" s="28">
+        <f>C13/C2</f>
+        <v>6.1934995229876263E-2</v>
+      </c>
+      <c r="D14" s="28">
+        <f>D13/D2</f>
+        <v>5.8795499784397326E-2</v>
+      </c>
+      <c r="E14" s="28">
+        <f>E13/E2</f>
+        <v>6.024690184146303E-2</v>
+      </c>
+      <c r="F14" s="3">
+        <f>SQRT(B16^2+C16^2+D16^2+E16^2)/4</f>
+        <v>3.3460106530949656E-2</v>
+      </c>
+      <c r="I14" t="s">
+        <v>39</v>
+      </c>
+      <c r="J14" t="s">
+        <v>40</v>
+      </c>
+      <c r="K14" t="s">
+        <v>41</v>
+      </c>
+      <c r="L14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A15" s="36"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="H15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" t="s">
+        <v>28</v>
+      </c>
+      <c r="M15" t="s">
+        <v>29</v>
+      </c>
+      <c r="N15" t="s">
+        <v>25</v>
+      </c>
+      <c r="O15" t="s">
+        <v>26</v>
+      </c>
+      <c r="P15" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>28</v>
+      </c>
+      <c r="R15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A16" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="22">
+        <f>J6</f>
+        <v>8.4459999999999993E-2</v>
+      </c>
+      <c r="C16" s="22">
+        <f>J12</f>
+        <v>7.2184999999999999E-2</v>
+      </c>
+      <c r="D16" s="22">
+        <f>J18</f>
+        <v>6.0567999999999997E-2</v>
+      </c>
+      <c r="E16" s="22">
+        <f>J24</f>
+        <v>4.3596000000000003E-2</v>
+      </c>
+      <c r="F16" s="1">
+        <f>SQRT(B18^2+C18^2+D18^2+E18^2)/4</f>
+        <v>6.7604520390212017E-2</v>
+      </c>
+      <c r="H16" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16">
+        <v>0.683056</v>
+      </c>
+      <c r="J16">
+        <v>7.9561000000000007E-2</v>
+      </c>
+      <c r="K16">
+        <v>4.9695999999999997E-2</v>
+      </c>
+      <c r="L16">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M16">
+        <v>9.4112000000000001E-2</v>
+      </c>
+      <c r="N16" s="1">
+        <v>2.0930800000000002E-18</v>
+      </c>
+      <c r="O16" s="1">
+        <v>2.5397600000000002E-19</v>
+      </c>
+      <c r="P16" s="1">
+        <v>1.5863999999999999E-19</v>
+      </c>
+      <c r="Q16" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R16" s="1">
+        <v>3.0042700000000002E-19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A17" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="24">
+        <f>O6</f>
+        <v>2.69614E-19</v>
+      </c>
+      <c r="C17" s="24">
+        <f>O12</f>
+        <v>2.3043099999999998E-19</v>
+      </c>
+      <c r="D17" s="24">
+        <f>O18</f>
+        <v>1.93345E-19</v>
+      </c>
+      <c r="E17" s="24">
+        <f>O24</f>
+        <v>1.3916899999999999E-19</v>
+      </c>
+      <c r="F17" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17">
+        <v>0.80426799999999998</v>
+      </c>
+      <c r="J17">
+        <v>9.1606000000000007E-2</v>
+      </c>
+      <c r="K17">
+        <v>7.0844000000000004E-2</v>
+      </c>
+      <c r="L17">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M17">
+        <v>0.116051</v>
+      </c>
+      <c r="N17" s="1">
+        <v>2.48001E-18</v>
+      </c>
+      <c r="O17" s="1">
+        <v>2.92426E-19</v>
+      </c>
+      <c r="P17" s="1">
+        <v>2.26149E-19</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R17" s="1">
+        <v>3.7046199999999999E-19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A18" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="23">
+        <f>B17/B2</f>
+        <v>0.18018833247565647</v>
+      </c>
+      <c r="C18" s="23">
+        <f>C17/C2</f>
+        <v>0.16781440941498618</v>
+      </c>
+      <c r="D18" s="28">
+        <f>D17/D2</f>
+        <v>8.4213529393829839E-2</v>
+      </c>
+      <c r="E18" s="28">
+        <f>E17/E2</f>
+        <v>7.3515366655045267E-2</v>
+      </c>
+      <c r="F18" s="3">
+        <f>SQRT(B20^2+C20^2+D20^2+E20^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18">
+        <v>0.74658800000000003</v>
+      </c>
+      <c r="J18">
+        <v>6.0567999999999997E-2</v>
+      </c>
+      <c r="K18">
+        <v>4.2286999999999998E-2</v>
+      </c>
+      <c r="L18">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M18">
+        <v>7.4257000000000004E-2</v>
+      </c>
+      <c r="N18" s="1">
+        <v>2.2958900000000001E-18</v>
+      </c>
+      <c r="O18" s="1">
+        <v>1.93345E-19</v>
+      </c>
+      <c r="P18" s="1">
+        <v>1.3498799999999999E-19</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R18" s="1">
+        <v>2.3704400000000001E-19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A19" s="36"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A20" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="I20" t="s">
+        <v>39</v>
+      </c>
+      <c r="J20" t="s">
+        <v>40</v>
+      </c>
+      <c r="K20" t="s">
+        <v>41</v>
+      </c>
+      <c r="L20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A21" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="22">
+        <f>SQRT(B17^2+B13^2+B9^2)</f>
+        <v>2.8764684730318183E-19</v>
+      </c>
+      <c r="C21" s="22">
+        <f>SQRT(C17^2+C13^2+C9^2)</f>
+        <v>2.4679939739806901E-19</v>
+      </c>
+      <c r="D21" s="22">
+        <f>SQRT(D17^2+D13^2+D9^2)</f>
+        <v>2.3704373590080372E-19</v>
+      </c>
+      <c r="E21" s="22">
+        <f>SQRT(E17^2+E13^2+E9^2)</f>
+        <v>1.8167610879036902E-19</v>
+      </c>
+      <c r="H21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I21" t="s">
+        <v>25</v>
+      </c>
+      <c r="J21" t="s">
+        <v>26</v>
+      </c>
+      <c r="K21" t="s">
+        <v>27</v>
+      </c>
+      <c r="L21" t="s">
+        <v>28</v>
+      </c>
+      <c r="M21" t="s">
+        <v>29</v>
+      </c>
+      <c r="N21" t="s">
+        <v>25</v>
+      </c>
+      <c r="O21" t="s">
+        <v>26</v>
+      </c>
+      <c r="P21" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>28</v>
+      </c>
+      <c r="R21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A22" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="23">
+        <f>B21/B2</f>
+        <v>0.19224003856416993</v>
+      </c>
+      <c r="C22" s="23">
+        <f>C21/C2</f>
+        <v>0.17973491031298494</v>
+      </c>
+      <c r="D22" s="23">
+        <f>D21/D2</f>
+        <v>0.10324699175518152</v>
+      </c>
+      <c r="E22" s="28">
+        <f>E21/E2</f>
+        <v>9.596954602092328E-2</v>
+      </c>
+      <c r="H22" t="s">
+        <v>30</v>
+      </c>
+      <c r="I22">
+        <v>0.59173600000000004</v>
+      </c>
+      <c r="J22">
+        <v>5.6980999999999997E-2</v>
+      </c>
+      <c r="K22">
+        <v>4.3527000000000003E-2</v>
+      </c>
+      <c r="L22">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M22">
+        <v>7.2134000000000004E-2</v>
+      </c>
+      <c r="N22" s="1">
+        <v>1.78864E-18</v>
+      </c>
+      <c r="O22" s="1">
+        <v>1.81896E-19</v>
+      </c>
+      <c r="P22" s="1">
+        <v>1.3894599999999999E-19</v>
+      </c>
+      <c r="Q22" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R22" s="1">
+        <v>2.3026700000000002E-19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A23" s="6"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="H23" t="s">
+        <v>31</v>
+      </c>
+      <c r="I23">
+        <v>0.653752</v>
+      </c>
+      <c r="J23">
+        <v>6.6333000000000003E-2</v>
+      </c>
+      <c r="K23">
+        <v>6.4299999999999996E-2</v>
+      </c>
+      <c r="L23">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M23">
+        <v>9.2716999999999994E-2</v>
+      </c>
+      <c r="N23" s="1">
+        <v>1.98661E-18</v>
+      </c>
+      <c r="O23" s="1">
+        <v>2.1175E-19</v>
+      </c>
+      <c r="P23" s="1">
+        <v>2.0526000000000001E-19</v>
+      </c>
+      <c r="Q23" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R23" s="1">
+        <v>2.9597299999999999E-19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A24" s="6"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="5"/>
+      <c r="H24" t="s">
+        <v>32</v>
+      </c>
+      <c r="I24">
+        <v>0.62444599999999995</v>
+      </c>
+      <c r="J24">
+        <v>4.3596000000000003E-2</v>
+      </c>
+      <c r="K24">
+        <v>3.5728000000000003E-2</v>
+      </c>
+      <c r="L24">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M24">
+        <v>5.6911999999999997E-2</v>
+      </c>
+      <c r="N24" s="1">
+        <v>1.8930599999999998E-18</v>
+      </c>
+      <c r="O24" s="1">
+        <v>1.3916899999999999E-19</v>
+      </c>
+      <c r="P24" s="1">
+        <v>1.14051E-19</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R24" s="1">
+        <v>1.8167600000000001E-19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="C25" s="1"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="1">
+        <f>B3-B21</f>
+        <v>1.5269681816184276E-25</v>
+      </c>
+      <c r="C26" s="1">
+        <f>C3-C21</f>
+        <v>6.0260193099454558E-25</v>
+      </c>
+      <c r="D26" s="1">
+        <f>D3-D21</f>
+        <v>2.6409919629228419E-25</v>
+      </c>
+      <c r="E26" s="1">
+        <f>E3-E21</f>
+        <v>-1.0879036901010252E-25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B27" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2389C22-199B-564C-BB09-6A12BD67C173}">
+  <dimension ref="A1:R29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="22">
+        <f>N6</f>
+        <v>1.46642E-18</v>
+      </c>
+      <c r="C2" s="22">
+        <f>N12</f>
+        <v>1.3471599999999999E-18</v>
+      </c>
+      <c r="D2" s="22">
+        <f>N18</f>
+        <v>2.2857000000000001E-18</v>
+      </c>
+      <c r="E2" s="22">
+        <f>N24</f>
+        <v>1.88991E-18</v>
+      </c>
+      <c r="F2" s="1">
+        <f>SQRT(B2^2+C2^2+D2^2+E2^2)/4</f>
+        <v>8.9307796342550629E-19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="24">
+        <f>R6</f>
+        <v>2.8112400000000002E-19</v>
+      </c>
+      <c r="C3" s="24">
+        <f>R12</f>
+        <v>2.4182999999999998E-19</v>
+      </c>
+      <c r="D3" s="24">
+        <f>R18</f>
+        <v>2.2777700000000001E-19</v>
+      </c>
+      <c r="E3" s="24">
+        <f>R24</f>
+        <v>1.7349099999999999E-19</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F4" si="0">SQRT(B3^2+C3^2+D3^2+E3^2)/4</f>
+        <v>1.1712545119603595E-19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="23">
+        <f>B3/B2</f>
+        <v>0.19170769629437678</v>
+      </c>
+      <c r="C4" s="23">
+        <f t="shared" ref="C4:E4" si="1">C3/C2</f>
+        <v>0.17951097122836188</v>
+      </c>
+      <c r="D4" s="23">
+        <f t="shared" si="1"/>
+        <v>9.9653060331627075E-2</v>
+      </c>
+      <c r="E4" s="28">
+        <f t="shared" si="1"/>
+        <v>9.1798551253763405E-2</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
+        <v>7.3880704541001221E-2</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4">
+        <v>0.62288500000000002</v>
+      </c>
+      <c r="J4">
+        <v>0.109403</v>
+      </c>
+      <c r="K4">
+        <v>4.5337000000000002E-2</v>
+      </c>
+      <c r="L4">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M4">
+        <v>0.118612</v>
+      </c>
+      <c r="N4" s="1">
+        <v>1.92348E-18</v>
+      </c>
+      <c r="O4" s="1">
+        <v>3.4923800000000002E-19</v>
+      </c>
+      <c r="P4" s="1">
+        <v>1.44727E-19</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R4" s="1">
+        <v>3.7863699999999999E-19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" s="37"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="H5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5">
+        <v>0.30293599999999998</v>
+      </c>
+      <c r="J5">
+        <v>0.12731100000000001</v>
+      </c>
+      <c r="K5">
+        <v>2.3862999999999999E-2</v>
+      </c>
+      <c r="L5">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M5">
+        <v>0.12970000000000001</v>
+      </c>
+      <c r="N5" s="1">
+        <v>9.0212999999999999E-19</v>
+      </c>
+      <c r="O5" s="1">
+        <v>4.0640499999999998E-19</v>
+      </c>
+      <c r="P5" s="1">
+        <v>7.6175300000000001E-20</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R5" s="1">
+        <v>4.1403100000000001E-19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A6" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="38"/>
+      <c r="F6" s="1"/>
+      <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6">
+        <v>0.47970600000000002</v>
+      </c>
+      <c r="J6">
+        <v>8.3918999999999994E-2</v>
+      </c>
+      <c r="K6">
+        <v>2.5856000000000001E-2</v>
+      </c>
+      <c r="L6">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M6">
+        <v>8.8065000000000004E-2</v>
+      </c>
+      <c r="N6" s="1">
+        <v>1.46642E-18</v>
+      </c>
+      <c r="O6" s="1">
+        <v>2.6788900000000001E-19</v>
+      </c>
+      <c r="P6" s="1">
+        <v>8.2538800000000001E-20</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R6" s="1">
+        <v>2.8112400000000002E-19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A8" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="22">
+        <f>L4</f>
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="C8" s="22">
+        <f>L12</f>
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="D8" s="22">
+        <f>L18</f>
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="E8" s="22">
+        <f>L24</f>
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="F8" s="1">
+        <f>SQRT(B10^2+C10^2+D10^2+E10^2)/4</f>
+        <v>7.1524483572727388E-3</v>
+      </c>
+      <c r="I8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A9" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="24">
+        <f>Q6</f>
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="C9" s="24">
+        <f>Q12</f>
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="D9" s="24">
+        <f>Q18</f>
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="E9" s="24">
+        <f>Q24</f>
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="F9" s="1">
+        <f>SQRT(B11^2+C11^2+D11^2+E11^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" t="s">
+        <v>25</v>
+      </c>
+      <c r="J9" t="s">
+        <v>26</v>
+      </c>
+      <c r="K9" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" t="s">
+        <v>28</v>
+      </c>
+      <c r="M9" t="s">
+        <v>29</v>
+      </c>
+      <c r="N9" t="s">
+        <v>25</v>
+      </c>
+      <c r="O9" t="s">
+        <v>26</v>
+      </c>
+      <c r="P9" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>28</v>
+      </c>
+      <c r="R9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A10" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="28">
+        <f>B9/B2</f>
+        <v>1.4522510604056137E-2</v>
+      </c>
+      <c r="C10" s="28">
+        <f>C9/C2</f>
+        <v>1.7859719706642123E-2</v>
+      </c>
+      <c r="D10" s="28">
+        <f>D9/D2</f>
+        <v>1.058795992474953E-2</v>
+      </c>
+      <c r="E10" s="28">
+        <f>E9/E2</f>
+        <v>1.32869290072014E-2</v>
+      </c>
+      <c r="F10" s="3">
+        <f>SQRT(B12^2+C12^2+D12^2+E12^2)/4</f>
+        <v>1.5068494933552588E-2</v>
+      </c>
+      <c r="H10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10">
+        <v>0.360288</v>
+      </c>
+      <c r="J10">
+        <v>9.3454999999999996E-2</v>
+      </c>
+      <c r="K10">
+        <v>2.6723E-2</v>
+      </c>
+      <c r="L10">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M10">
+        <v>9.7491999999999995E-2</v>
+      </c>
+      <c r="N10" s="1">
+        <v>1.08307E-18</v>
+      </c>
+      <c r="O10" s="1">
+        <v>2.9832799999999999E-19</v>
+      </c>
+      <c r="P10" s="1">
+        <v>8.5305099999999998E-20</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R10" s="1">
+        <v>3.1121600000000002E-19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A11" s="36"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="H11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11">
+        <v>0.50922900000000004</v>
+      </c>
+      <c r="J11">
+        <v>0.108885</v>
+      </c>
+      <c r="K11">
+        <v>3.9389E-2</v>
+      </c>
+      <c r="L11">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M11">
+        <v>0.116036</v>
+      </c>
+      <c r="N11" s="1">
+        <v>1.5585200000000001E-18</v>
+      </c>
+      <c r="O11" s="1">
+        <v>3.4758499999999999E-19</v>
+      </c>
+      <c r="P11" s="1">
+        <v>1.2573900000000001E-19</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R11" s="1">
+        <v>3.7041199999999999E-19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A12" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="24">
+        <f>K6</f>
+        <v>2.5856000000000001E-2</v>
+      </c>
+      <c r="C12" s="22">
+        <f>K12</f>
+        <v>2.3181E-2</v>
+      </c>
+      <c r="D12" s="22">
+        <f>K18</f>
+        <v>3.7580000000000002E-2</v>
+      </c>
+      <c r="E12" s="22">
+        <f>K24</f>
+        <v>3.1856000000000002E-2</v>
+      </c>
+      <c r="F12" s="1">
+        <f>SQRT(B14^2+C14^2+D14^2+E14^2)/4</f>
+        <v>2.7197361727229023E-2</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12">
+        <v>0.44301800000000002</v>
+      </c>
+      <c r="J12">
+        <v>7.1726999999999999E-2</v>
+      </c>
+      <c r="K12">
+        <v>2.3181E-2</v>
+      </c>
+      <c r="L12">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M12">
+        <v>7.5756000000000004E-2</v>
+      </c>
+      <c r="N12" s="1">
+        <v>1.3471599999999999E-18</v>
+      </c>
+      <c r="O12" s="1">
+        <v>2.2897E-19</v>
+      </c>
+      <c r="P12" s="1">
+        <v>7.3998099999999995E-20</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R12" s="1">
+        <v>2.4182999999999998E-19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A13" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="24">
+        <f>P6</f>
+        <v>8.2538800000000001E-20</v>
+      </c>
+      <c r="C13" s="24">
+        <f>P12</f>
+        <v>7.3998099999999995E-20</v>
+      </c>
+      <c r="D13" s="24">
+        <f>P18</f>
+        <v>1.1996500000000001E-19</v>
+      </c>
+      <c r="E13" s="24">
+        <f>P24</f>
+        <v>1.0169E-19</v>
+      </c>
+      <c r="F13" s="1">
+        <f>SQRT(B15^2+C15^2+D15^2+E15^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="28">
+        <f>B13/B2</f>
+        <v>5.6285920813955073E-2</v>
+      </c>
+      <c r="C14" s="28">
+        <f>C13/C2</f>
+        <v>5.4928961667507943E-2</v>
+      </c>
+      <c r="D14" s="28">
+        <f>D13/D2</f>
+        <v>5.2485015531347073E-2</v>
+      </c>
+      <c r="E14" s="28">
+        <f>E13/E2</f>
+        <v>5.3806795032567689E-2</v>
+      </c>
+      <c r="F14" s="3">
+        <f>SQRT(B16^2+C16^2+D16^2+E16^2)/4</f>
+        <v>3.3247038510031232E-2</v>
+      </c>
+      <c r="I14" t="s">
+        <v>39</v>
+      </c>
+      <c r="J14" t="s">
+        <v>40</v>
+      </c>
+      <c r="K14" t="s">
+        <v>41</v>
+      </c>
+      <c r="L14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A15" s="36"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="H15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" t="s">
+        <v>28</v>
+      </c>
+      <c r="M15" t="s">
+        <v>29</v>
+      </c>
+      <c r="N15" t="s">
+        <v>25</v>
+      </c>
+      <c r="O15" t="s">
+        <v>26</v>
+      </c>
+      <c r="P15" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>28</v>
+      </c>
+      <c r="R15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A16" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="22">
+        <f>J6</f>
+        <v>8.3918999999999994E-2</v>
+      </c>
+      <c r="C16" s="22">
+        <f>J12</f>
+        <v>7.1726999999999999E-2</v>
+      </c>
+      <c r="D16" s="22">
+        <f>J18</f>
+        <v>6.0179999999999997E-2</v>
+      </c>
+      <c r="E16" s="22">
+        <f>J24</f>
+        <v>4.3325000000000002E-2</v>
+      </c>
+      <c r="F16" s="1">
+        <f>SQRT(B18^2+C18^2+D18^2+E18^2)/4</f>
+        <v>6.8319166755937813E-2</v>
+      </c>
+      <c r="H16" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16">
+        <v>0.677844</v>
+      </c>
+      <c r="J16">
+        <v>7.8012999999999999E-2</v>
+      </c>
+      <c r="K16">
+        <v>4.6717000000000002E-2</v>
+      </c>
+      <c r="L16">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M16">
+        <v>9.1246999999999995E-2</v>
+      </c>
+      <c r="N16" s="1">
+        <v>2.0764400000000001E-18</v>
+      </c>
+      <c r="O16" s="1">
+        <v>2.4903599999999998E-19</v>
+      </c>
+      <c r="P16" s="1">
+        <v>1.49131E-19</v>
+      </c>
+      <c r="Q16" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R16" s="1">
+        <v>2.9128100000000002E-19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A17" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="24">
+        <f>O6</f>
+        <v>2.6788900000000001E-19</v>
+      </c>
+      <c r="C17" s="24">
+        <f>O12</f>
+        <v>2.2897E-19</v>
+      </c>
+      <c r="D17" s="24">
+        <f>O18</f>
+        <v>1.92107E-19</v>
+      </c>
+      <c r="E17" s="24">
+        <f>O24</f>
+        <v>1.38303E-19</v>
+      </c>
+      <c r="F17" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17">
+        <v>0.80456499999999997</v>
+      </c>
+      <c r="J17">
+        <v>9.1906000000000002E-2</v>
+      </c>
+      <c r="K17">
+        <v>5.8146999999999997E-2</v>
+      </c>
+      <c r="L17">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M17">
+        <v>0.109019</v>
+      </c>
+      <c r="N17" s="1">
+        <v>2.48096E-18</v>
+      </c>
+      <c r="O17" s="1">
+        <v>2.9338299999999998E-19</v>
+      </c>
+      <c r="P17" s="1">
+        <v>1.85618E-19</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R17" s="1">
+        <v>3.4801300000000001E-19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A18" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="23">
+        <f>B17/B2</f>
+        <v>0.18268231475293573</v>
+      </c>
+      <c r="C18" s="23">
+        <f>C17/C2</f>
+        <v>0.16996496333026517</v>
+      </c>
+      <c r="D18" s="28">
+        <f>D17/D2</f>
+        <v>8.4047337795861224E-2</v>
+      </c>
+      <c r="E18" s="28">
+        <f>E17/E2</f>
+        <v>7.317967522262965E-2</v>
+      </c>
+      <c r="F18" s="3">
+        <f>SQRT(B20^2+C20^2+D20^2+E20^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18">
+        <v>0.74339699999999997</v>
+      </c>
+      <c r="J18">
+        <v>6.0179999999999997E-2</v>
+      </c>
+      <c r="K18">
+        <v>3.7580000000000002E-2</v>
+      </c>
+      <c r="L18">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M18">
+        <v>7.1354000000000001E-2</v>
+      </c>
+      <c r="N18" s="1">
+        <v>2.2857000000000001E-18</v>
+      </c>
+      <c r="O18" s="1">
+        <v>1.92107E-19</v>
+      </c>
+      <c r="P18" s="1">
+        <v>1.1996500000000001E-19</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R18" s="1">
+        <v>2.2777700000000001E-19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A19" s="36"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A20" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="I20" t="s">
+        <v>39</v>
+      </c>
+      <c r="J20" t="s">
+        <v>40</v>
+      </c>
+      <c r="K20" t="s">
+        <v>41</v>
+      </c>
+      <c r="L20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A21" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="22">
+        <f>SQRT(B17^2+B13^2+B9^2)</f>
+        <v>2.8112398279344651E-19</v>
+      </c>
+      <c r="C21" s="22">
+        <f>SQRT(C17^2+C13^2+C9^2)</f>
+        <v>2.4183022658803429E-19</v>
+      </c>
+      <c r="D21" s="22">
+        <f>SQRT(D17^2+D13^2+D9^2)</f>
+        <v>2.2777704940316089E-19</v>
+      </c>
+      <c r="E21" s="22">
+        <f>SQRT(E17^2+E13^2+E9^2)</f>
+        <v>1.7349104660532197E-19</v>
+      </c>
+      <c r="H21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I21" t="s">
+        <v>25</v>
+      </c>
+      <c r="J21" t="s">
+        <v>26</v>
+      </c>
+      <c r="K21" t="s">
+        <v>27</v>
+      </c>
+      <c r="L21" t="s">
+        <v>28</v>
+      </c>
+      <c r="M21" t="s">
+        <v>29</v>
+      </c>
+      <c r="N21" t="s">
+        <v>25</v>
+      </c>
+      <c r="O21" t="s">
+        <v>26</v>
+      </c>
+      <c r="P21" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>28</v>
+      </c>
+      <c r="R21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A22" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="23">
+        <f>B21/B2</f>
+        <v>0.19170768456066237</v>
+      </c>
+      <c r="C22" s="23">
+        <f>C21/C2</f>
+        <v>0.17951113942518654</v>
+      </c>
+      <c r="D22" s="23">
+        <f>D21/D2</f>
+        <v>9.9653081945645039E-2</v>
+      </c>
+      <c r="E22" s="28">
+        <f>E21/E2</f>
+        <v>9.1798575913838207E-2</v>
+      </c>
+      <c r="H22" t="s">
+        <v>30</v>
+      </c>
+      <c r="I22">
+        <v>0.57918899999999995</v>
+      </c>
+      <c r="J22">
+        <v>5.5905999999999997E-2</v>
+      </c>
+      <c r="K22">
+        <v>4.0346E-2</v>
+      </c>
+      <c r="L22">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M22">
+        <v>6.9390999999999994E-2</v>
+      </c>
+      <c r="N22" s="1">
+        <v>1.74859E-18</v>
+      </c>
+      <c r="O22" s="1">
+        <v>1.78465E-19</v>
+      </c>
+      <c r="P22" s="1">
+        <v>1.2879299999999999E-19</v>
+      </c>
+      <c r="Q22" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R22" s="1">
+        <v>2.21513E-19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A23" s="6"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="H23" t="s">
+        <v>31</v>
+      </c>
+      <c r="I23">
+        <v>0.65437100000000004</v>
+      </c>
+      <c r="J23">
+        <v>6.6559999999999994E-2</v>
+      </c>
+      <c r="K23">
+        <v>4.9153000000000002E-2</v>
+      </c>
+      <c r="L23">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M23">
+        <v>8.3114999999999994E-2</v>
+      </c>
+      <c r="N23" s="1">
+        <v>1.9885899999999998E-18</v>
+      </c>
+      <c r="O23" s="1">
+        <v>2.1247599999999999E-19</v>
+      </c>
+      <c r="P23" s="1">
+        <v>1.5690700000000001E-19</v>
+      </c>
+      <c r="Q23" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R23" s="1">
+        <v>2.6532299999999999E-19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A24" s="6"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="5"/>
+      <c r="H24" t="s">
+        <v>32</v>
+      </c>
+      <c r="I24">
+        <v>0.62345799999999996</v>
+      </c>
+      <c r="J24">
+        <v>4.3325000000000002E-2</v>
+      </c>
+      <c r="K24">
+        <v>3.1856000000000002E-2</v>
+      </c>
+      <c r="L24">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M24">
+        <v>5.4348E-2</v>
+      </c>
+      <c r="N24" s="1">
+        <v>1.88991E-18</v>
+      </c>
+      <c r="O24" s="1">
+        <v>1.38303E-19</v>
+      </c>
+      <c r="P24" s="1">
+        <v>1.0169E-19</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R24" s="1">
+        <v>1.7349099999999999E-19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="C25" s="1"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="1">
+        <f>B3-B21</f>
+        <v>1.7206553512660786E-26</v>
+      </c>
+      <c r="C26" s="1">
+        <f>C3-C21</f>
+        <v>-2.2658803431396843E-25</v>
+      </c>
+      <c r="D26" s="1">
+        <f>D3-D21</f>
+        <v>-4.9403160872505303E-26</v>
+      </c>
+      <c r="E26" s="1">
+        <f>E3-E21</f>
+        <v>-4.6605321973691009E-26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B27" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92994925-A506-0B4B-AB86-443EF5CF787E}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1737,2104 +3831,7 @@
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B27" s="1">
-        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2695A833-57C4-DC4E-AC5C-0BDB90378BCB}">
-  <dimension ref="A1:R29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.1640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="22">
-        <f>N6</f>
-        <v>1.49629E-18</v>
-      </c>
-      <c r="C2" s="22">
-        <f>N12</f>
-        <v>1.37313E-18</v>
-      </c>
-      <c r="D2" s="22">
-        <f>N18</f>
-        <v>2.2958900000000001E-18</v>
-      </c>
-      <c r="E2" s="22">
-        <f>N24</f>
-        <v>1.8930599999999998E-18</v>
-      </c>
-      <c r="F2" s="1">
-        <f>SQRT(B2^2+C2^2+D2^2+E2^2)/4</f>
-        <v>9.0066492162388003E-19</v>
-      </c>
-      <c r="I2" t="s">
-        <v>39</v>
-      </c>
-      <c r="J2" t="s">
-        <v>40</v>
-      </c>
-      <c r="K2" t="s">
-        <v>41</v>
-      </c>
-      <c r="L2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A3" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="24">
-        <f>R6</f>
-        <v>2.8764699999999999E-19</v>
-      </c>
-      <c r="C3" s="24">
-        <f>R12</f>
-        <v>2.4680000000000001E-19</v>
-      </c>
-      <c r="D3" s="24">
-        <f>R18</f>
-        <v>2.3704400000000001E-19</v>
-      </c>
-      <c r="E3" s="24">
-        <f>R24</f>
-        <v>1.8167600000000001E-19</v>
-      </c>
-      <c r="F3" s="1">
-        <f t="shared" ref="F3:F4" si="0">SQRT(B3^2+C3^2+D3^2+E3^2)/4</f>
-        <v>1.2063557298766603E-19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" t="s">
-        <v>27</v>
-      </c>
-      <c r="L3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N3" t="s">
-        <v>25</v>
-      </c>
-      <c r="O3" t="s">
-        <v>26</v>
-      </c>
-      <c r="P3" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>28</v>
-      </c>
-      <c r="R3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="23">
-        <f>B3/B2</f>
-        <v>0.19224014061445308</v>
-      </c>
-      <c r="C4" s="23">
-        <f t="shared" ref="C4:E4" si="1">C3/C2</f>
-        <v>0.17973534916577455</v>
-      </c>
-      <c r="D4" s="23">
-        <f t="shared" si="1"/>
-        <v>0.10324710678647496</v>
-      </c>
-      <c r="E4" s="28">
-        <f t="shared" si="1"/>
-        <v>9.5969488552924906E-2</v>
-      </c>
-      <c r="F4" s="1">
-        <f t="shared" si="0"/>
-        <v>7.4637111745806173E-2</v>
-      </c>
-      <c r="H4" t="s">
-        <v>30</v>
-      </c>
-      <c r="I4">
-        <v>0.654451</v>
-      </c>
-      <c r="J4">
-        <v>0.111583</v>
-      </c>
-      <c r="K4">
-        <v>4.8462999999999999E-2</v>
-      </c>
-      <c r="L4">
-        <v>6.6709999999999998E-3</v>
-      </c>
-      <c r="M4">
-        <v>0.121836</v>
-      </c>
-      <c r="N4" s="1">
-        <v>2.0242400000000001E-18</v>
-      </c>
-      <c r="O4" s="1">
-        <v>3.5619899999999999E-19</v>
-      </c>
-      <c r="P4" s="1">
-        <v>1.54705E-19</v>
-      </c>
-      <c r="Q4" s="1">
-        <v>2.1296100000000001E-20</v>
-      </c>
-      <c r="R4" s="1">
-        <v>3.8892800000000001E-19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" s="37"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="H5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5">
-        <v>0.30299100000000001</v>
-      </c>
-      <c r="J5">
-        <v>0.126971</v>
-      </c>
-      <c r="K5">
-        <v>5.0055000000000002E-2</v>
-      </c>
-      <c r="L5">
-        <v>6.6709999999999998E-3</v>
-      </c>
-      <c r="M5">
-        <v>0.13664499999999999</v>
-      </c>
-      <c r="N5" s="1">
-        <v>9.0230500000000007E-19</v>
-      </c>
-      <c r="O5" s="1">
-        <v>4.0532099999999998E-19</v>
-      </c>
-      <c r="P5" s="1">
-        <v>1.5978799999999999E-19</v>
-      </c>
-      <c r="Q5" s="1">
-        <v>2.1296100000000001E-20</v>
-      </c>
-      <c r="R5" s="1">
-        <v>4.3620000000000004E-19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="38"/>
-      <c r="F6" s="1"/>
-      <c r="H6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I6">
-        <v>0.489064</v>
-      </c>
-      <c r="J6">
-        <v>8.4459999999999993E-2</v>
-      </c>
-      <c r="K6">
-        <v>3.0686000000000001E-2</v>
-      </c>
-      <c r="L6">
-        <v>6.6709999999999998E-3</v>
-      </c>
-      <c r="M6">
-        <v>9.0108999999999995E-2</v>
-      </c>
-      <c r="N6" s="1">
-        <v>1.49629E-18</v>
-      </c>
-      <c r="O6" s="1">
-        <v>2.69614E-19</v>
-      </c>
-      <c r="P6" s="1">
-        <v>9.7956499999999994E-20</v>
-      </c>
-      <c r="Q6" s="1">
-        <v>2.1296100000000001E-20</v>
-      </c>
-      <c r="R6" s="1">
-        <v>2.8764699999999999E-19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A8" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="22">
-        <f>L4</f>
-        <v>6.6709999999999998E-3</v>
-      </c>
-      <c r="C8" s="22">
-        <f>L12</f>
-        <v>7.5370000000000003E-3</v>
-      </c>
-      <c r="D8" s="22">
-        <f>L18</f>
-        <v>7.5810000000000001E-3</v>
-      </c>
-      <c r="E8" s="22">
-        <f>L24</f>
-        <v>7.8659999999999997E-3</v>
-      </c>
-      <c r="F8" s="1">
-        <f>SQRT(B10^2+C10^2+D10^2+E10^2)/4</f>
-        <v>7.0562593169518437E-3</v>
-      </c>
-      <c r="I8" t="s">
-        <v>39</v>
-      </c>
-      <c r="J8" t="s">
-        <v>40</v>
-      </c>
-      <c r="K8" t="s">
-        <v>41</v>
-      </c>
-      <c r="L8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A9" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="24">
-        <f>Q6</f>
-        <v>2.1296100000000001E-20</v>
-      </c>
-      <c r="C9" s="24">
-        <f>Q12</f>
-        <v>2.4059899999999999E-20</v>
-      </c>
-      <c r="D9" s="24">
-        <f>Q18</f>
-        <v>2.4200900000000001E-20</v>
-      </c>
-      <c r="E9" s="24">
-        <f>Q24</f>
-        <v>2.5111099999999999E-20</v>
-      </c>
-      <c r="F9" s="1">
-        <f>SQRT(B11^2+C11^2+D11^2+E11^2)/4</f>
-        <v>0</v>
-      </c>
-      <c r="H9" t="s">
-        <v>24</v>
-      </c>
-      <c r="I9" t="s">
-        <v>25</v>
-      </c>
-      <c r="J9" t="s">
-        <v>26</v>
-      </c>
-      <c r="K9" t="s">
-        <v>27</v>
-      </c>
-      <c r="L9" t="s">
-        <v>28</v>
-      </c>
-      <c r="M9" t="s">
-        <v>29</v>
-      </c>
-      <c r="N9" t="s">
-        <v>25</v>
-      </c>
-      <c r="O9" t="s">
-        <v>26</v>
-      </c>
-      <c r="P9" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>28</v>
-      </c>
-      <c r="R9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A10" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="28">
-        <f>B9/B2</f>
-        <v>1.4232601968869671E-2</v>
-      </c>
-      <c r="C10" s="28">
-        <f>C9/C2</f>
-        <v>1.7521938927850967E-2</v>
-      </c>
-      <c r="D10" s="28">
-        <f>D9/D2</f>
-        <v>1.0540966683943918E-2</v>
-      </c>
-      <c r="E10" s="28">
-        <f>E9/E2</f>
-        <v>1.3264819921185805E-2</v>
-      </c>
-      <c r="F10" s="3">
-        <f>SQRT(B12^2+C12^2+D12^2+E12^2)/4</f>
-        <v>1.7168382695379316E-2</v>
-      </c>
-      <c r="H10" t="s">
-        <v>30</v>
-      </c>
-      <c r="I10">
-        <v>0.37874000000000002</v>
-      </c>
-      <c r="J10">
-        <v>9.5302999999999999E-2</v>
-      </c>
-      <c r="K10">
-        <v>2.8292999999999999E-2</v>
-      </c>
-      <c r="L10">
-        <v>7.5370000000000003E-3</v>
-      </c>
-      <c r="M10">
-        <v>9.9699999999999997E-2</v>
-      </c>
-      <c r="N10" s="1">
-        <v>1.14197E-18</v>
-      </c>
-      <c r="O10" s="1">
-        <v>3.0422899999999999E-19</v>
-      </c>
-      <c r="P10" s="1">
-        <v>9.0318600000000001E-20</v>
-      </c>
-      <c r="Q10" s="1">
-        <v>2.4059899999999999E-20</v>
-      </c>
-      <c r="R10" s="1">
-        <v>3.1826299999999998E-19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A11" s="36"/>
-      <c r="B11" s="40"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="H11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I11">
-        <v>0.51285000000000003</v>
-      </c>
-      <c r="J11">
-        <v>0.108587</v>
-      </c>
-      <c r="K11">
-        <v>5.8909000000000003E-2</v>
-      </c>
-      <c r="L11">
-        <v>7.5370000000000003E-3</v>
-      </c>
-      <c r="M11">
-        <v>0.123767</v>
-      </c>
-      <c r="N11" s="1">
-        <v>1.57008E-18</v>
-      </c>
-      <c r="O11" s="1">
-        <v>3.4663400000000001E-19</v>
-      </c>
-      <c r="P11" s="1">
-        <v>1.88051E-19</v>
-      </c>
-      <c r="Q11" s="1">
-        <v>2.4059899999999999E-20</v>
-      </c>
-      <c r="R11" s="1">
-        <v>3.9509099999999998E-19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A12" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="24">
-        <f>K6</f>
-        <v>3.0686000000000001E-2</v>
-      </c>
-      <c r="C12" s="22">
-        <f>K12</f>
-        <v>2.6641000000000001E-2</v>
-      </c>
-      <c r="D12" s="22">
-        <f>K18</f>
-        <v>4.2286999999999998E-2</v>
-      </c>
-      <c r="E12" s="22">
-        <f>K24</f>
-        <v>3.5728000000000003E-2</v>
-      </c>
-      <c r="F12" s="1">
-        <f>SQRT(B14^2+C14^2+D14^2+E14^2)/4</f>
-        <v>3.0830559026828703E-2</v>
-      </c>
-      <c r="H12" t="s">
-        <v>32</v>
-      </c>
-      <c r="I12">
-        <v>0.45115100000000002</v>
-      </c>
-      <c r="J12">
-        <v>7.2184999999999999E-2</v>
-      </c>
-      <c r="K12">
-        <v>2.6641000000000001E-2</v>
-      </c>
-      <c r="L12">
-        <v>7.5370000000000003E-3</v>
-      </c>
-      <c r="M12">
-        <v>7.7313000000000007E-2</v>
-      </c>
-      <c r="N12" s="1">
-        <v>1.37313E-18</v>
-      </c>
-      <c r="O12" s="1">
-        <v>2.3043099999999998E-19</v>
-      </c>
-      <c r="P12" s="1">
-        <v>8.5044799999999996E-20</v>
-      </c>
-      <c r="Q12" s="1">
-        <v>2.4059899999999999E-20</v>
-      </c>
-      <c r="R12" s="1">
-        <v>2.4680000000000001E-19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A13" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="24">
-        <f>P6</f>
-        <v>9.7956499999999994E-20</v>
-      </c>
-      <c r="C13" s="24">
-        <f>P12</f>
-        <v>8.5044799999999996E-20</v>
-      </c>
-      <c r="D13" s="24">
-        <f>P18</f>
-        <v>1.3498799999999999E-19</v>
-      </c>
-      <c r="E13" s="24">
-        <f>P24</f>
-        <v>1.14051E-19</v>
-      </c>
-      <c r="F13" s="1">
-        <f>SQRT(B15^2+C15^2+D15^2+E15^2)/4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A14" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="28">
-        <f>B13/B2</f>
-        <v>6.5466253199580299E-2</v>
-      </c>
-      <c r="C14" s="28">
-        <f>C13/C2</f>
-        <v>6.1934995229876263E-2</v>
-      </c>
-      <c r="D14" s="28">
-        <f>D13/D2</f>
-        <v>5.8795499784397326E-2</v>
-      </c>
-      <c r="E14" s="28">
-        <f>E13/E2</f>
-        <v>6.024690184146303E-2</v>
-      </c>
-      <c r="F14" s="3">
-        <f>SQRT(B16^2+C16^2+D16^2+E16^2)/4</f>
-        <v>3.3460106530949656E-2</v>
-      </c>
-      <c r="I14" t="s">
-        <v>39</v>
-      </c>
-      <c r="J14" t="s">
-        <v>40</v>
-      </c>
-      <c r="K14" t="s">
-        <v>41</v>
-      </c>
-      <c r="L14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A15" s="36"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="H15" t="s">
-        <v>24</v>
-      </c>
-      <c r="I15" t="s">
-        <v>25</v>
-      </c>
-      <c r="J15" t="s">
-        <v>26</v>
-      </c>
-      <c r="K15" t="s">
-        <v>27</v>
-      </c>
-      <c r="L15" t="s">
-        <v>28</v>
-      </c>
-      <c r="M15" t="s">
-        <v>29</v>
-      </c>
-      <c r="N15" t="s">
-        <v>25</v>
-      </c>
-      <c r="O15" t="s">
-        <v>26</v>
-      </c>
-      <c r="P15" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>28</v>
-      </c>
-      <c r="R15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A16" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="22">
-        <f>J6</f>
-        <v>8.4459999999999993E-2</v>
-      </c>
-      <c r="C16" s="22">
-        <f>J12</f>
-        <v>7.2184999999999999E-2</v>
-      </c>
-      <c r="D16" s="22">
-        <f>J18</f>
-        <v>6.0567999999999997E-2</v>
-      </c>
-      <c r="E16" s="22">
-        <f>J24</f>
-        <v>4.3596000000000003E-2</v>
-      </c>
-      <c r="F16" s="1">
-        <f>SQRT(B18^2+C18^2+D18^2+E18^2)/4</f>
-        <v>6.7604520390212017E-2</v>
-      </c>
-      <c r="H16" t="s">
-        <v>30</v>
-      </c>
-      <c r="I16">
-        <v>0.683056</v>
-      </c>
-      <c r="J16">
-        <v>7.9561000000000007E-2</v>
-      </c>
-      <c r="K16">
-        <v>4.9695999999999997E-2</v>
-      </c>
-      <c r="L16">
-        <v>7.5810000000000001E-3</v>
-      </c>
-      <c r="M16">
-        <v>9.4112000000000001E-2</v>
-      </c>
-      <c r="N16" s="1">
-        <v>2.0930800000000002E-18</v>
-      </c>
-      <c r="O16" s="1">
-        <v>2.5397600000000002E-19</v>
-      </c>
-      <c r="P16" s="1">
-        <v>1.5863999999999999E-19</v>
-      </c>
-      <c r="Q16" s="1">
-        <v>2.4200900000000001E-20</v>
-      </c>
-      <c r="R16" s="1">
-        <v>3.0042700000000002E-19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A17" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="24">
-        <f>O6</f>
-        <v>2.69614E-19</v>
-      </c>
-      <c r="C17" s="24">
-        <f>O12</f>
-        <v>2.3043099999999998E-19</v>
-      </c>
-      <c r="D17" s="24">
-        <f>O18</f>
-        <v>1.93345E-19</v>
-      </c>
-      <c r="E17" s="24">
-        <f>O24</f>
-        <v>1.3916899999999999E-19</v>
-      </c>
-      <c r="F17" s="1">
-        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
-        <v>0</v>
-      </c>
-      <c r="H17" t="s">
-        <v>31</v>
-      </c>
-      <c r="I17">
-        <v>0.80426799999999998</v>
-      </c>
-      <c r="J17">
-        <v>9.1606000000000007E-2</v>
-      </c>
-      <c r="K17">
-        <v>7.0844000000000004E-2</v>
-      </c>
-      <c r="L17">
-        <v>7.5810000000000001E-3</v>
-      </c>
-      <c r="M17">
-        <v>0.116051</v>
-      </c>
-      <c r="N17" s="1">
-        <v>2.48001E-18</v>
-      </c>
-      <c r="O17" s="1">
-        <v>2.92426E-19</v>
-      </c>
-      <c r="P17" s="1">
-        <v>2.26149E-19</v>
-      </c>
-      <c r="Q17" s="1">
-        <v>2.4200900000000001E-20</v>
-      </c>
-      <c r="R17" s="1">
-        <v>3.7046199999999999E-19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A18" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="23">
-        <f>B17/B2</f>
-        <v>0.18018833247565647</v>
-      </c>
-      <c r="C18" s="23">
-        <f>C17/C2</f>
-        <v>0.16781440941498618</v>
-      </c>
-      <c r="D18" s="28">
-        <f>D17/D2</f>
-        <v>8.4213529393829839E-2</v>
-      </c>
-      <c r="E18" s="28">
-        <f>E17/E2</f>
-        <v>7.3515366655045267E-2</v>
-      </c>
-      <c r="F18" s="3">
-        <f>SQRT(B20^2+C20^2+D20^2+E20^2)/4</f>
-        <v>0</v>
-      </c>
-      <c r="H18" t="s">
-        <v>32</v>
-      </c>
-      <c r="I18">
-        <v>0.74658800000000003</v>
-      </c>
-      <c r="J18">
-        <v>6.0567999999999997E-2</v>
-      </c>
-      <c r="K18">
-        <v>4.2286999999999998E-2</v>
-      </c>
-      <c r="L18">
-        <v>7.5810000000000001E-3</v>
-      </c>
-      <c r="M18">
-        <v>7.4257000000000004E-2</v>
-      </c>
-      <c r="N18" s="1">
-        <v>2.2958900000000001E-18</v>
-      </c>
-      <c r="O18" s="1">
-        <v>1.93345E-19</v>
-      </c>
-      <c r="P18" s="1">
-        <v>1.3498799999999999E-19</v>
-      </c>
-      <c r="Q18" s="1">
-        <v>2.4200900000000001E-20</v>
-      </c>
-      <c r="R18" s="1">
-        <v>2.3704400000000001E-19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A19" s="36"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A20" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="I20" t="s">
-        <v>39</v>
-      </c>
-      <c r="J20" t="s">
-        <v>40</v>
-      </c>
-      <c r="K20" t="s">
-        <v>41</v>
-      </c>
-      <c r="L20" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="22">
-        <f>SQRT(B17^2+B13^2+B9^2)</f>
-        <v>2.8764684730318183E-19</v>
-      </c>
-      <c r="C21" s="22">
-        <f>SQRT(C17^2+C13^2+C9^2)</f>
-        <v>2.4679939739806901E-19</v>
-      </c>
-      <c r="D21" s="22">
-        <f>SQRT(D17^2+D13^2+D9^2)</f>
-        <v>2.3704373590080372E-19</v>
-      </c>
-      <c r="E21" s="22">
-        <f>SQRT(E17^2+E13^2+E9^2)</f>
-        <v>1.8167610879036902E-19</v>
-      </c>
-      <c r="H21" t="s">
-        <v>24</v>
-      </c>
-      <c r="I21" t="s">
-        <v>25</v>
-      </c>
-      <c r="J21" t="s">
-        <v>26</v>
-      </c>
-      <c r="K21" t="s">
-        <v>27</v>
-      </c>
-      <c r="L21" t="s">
-        <v>28</v>
-      </c>
-      <c r="M21" t="s">
-        <v>29</v>
-      </c>
-      <c r="N21" t="s">
-        <v>25</v>
-      </c>
-      <c r="O21" t="s">
-        <v>26</v>
-      </c>
-      <c r="P21" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>28</v>
-      </c>
-      <c r="R21" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A22" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="23">
-        <f>B21/B2</f>
-        <v>0.19224003856416993</v>
-      </c>
-      <c r="C22" s="23">
-        <f>C21/C2</f>
-        <v>0.17973491031298494</v>
-      </c>
-      <c r="D22" s="23">
-        <f>D21/D2</f>
-        <v>0.10324699175518152</v>
-      </c>
-      <c r="E22" s="28">
-        <f>E21/E2</f>
-        <v>9.596954602092328E-2</v>
-      </c>
-      <c r="H22" t="s">
-        <v>30</v>
-      </c>
-      <c r="I22">
-        <v>0.59173600000000004</v>
-      </c>
-      <c r="J22">
-        <v>5.6980999999999997E-2</v>
-      </c>
-      <c r="K22">
-        <v>4.3527000000000003E-2</v>
-      </c>
-      <c r="L22">
-        <v>7.8659999999999997E-3</v>
-      </c>
-      <c r="M22">
-        <v>7.2134000000000004E-2</v>
-      </c>
-      <c r="N22" s="1">
-        <v>1.78864E-18</v>
-      </c>
-      <c r="O22" s="1">
-        <v>1.81896E-19</v>
-      </c>
-      <c r="P22" s="1">
-        <v>1.3894599999999999E-19</v>
-      </c>
-      <c r="Q22" s="1">
-        <v>2.5111099999999999E-20</v>
-      </c>
-      <c r="R22" s="1">
-        <v>2.3026700000000002E-19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A23" s="6"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="H23" t="s">
-        <v>31</v>
-      </c>
-      <c r="I23">
-        <v>0.653752</v>
-      </c>
-      <c r="J23">
-        <v>6.6333000000000003E-2</v>
-      </c>
-      <c r="K23">
-        <v>6.4299999999999996E-2</v>
-      </c>
-      <c r="L23">
-        <v>7.8659999999999997E-3</v>
-      </c>
-      <c r="M23">
-        <v>9.2716999999999994E-2</v>
-      </c>
-      <c r="N23" s="1">
-        <v>1.98661E-18</v>
-      </c>
-      <c r="O23" s="1">
-        <v>2.1175E-19</v>
-      </c>
-      <c r="P23" s="1">
-        <v>2.0526000000000001E-19</v>
-      </c>
-      <c r="Q23" s="1">
-        <v>2.5111099999999999E-20</v>
-      </c>
-      <c r="R23" s="1">
-        <v>2.9597299999999999E-19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A24" s="6"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="5"/>
-      <c r="H24" t="s">
-        <v>32</v>
-      </c>
-      <c r="I24">
-        <v>0.62444599999999995</v>
-      </c>
-      <c r="J24">
-        <v>4.3596000000000003E-2</v>
-      </c>
-      <c r="K24">
-        <v>3.5728000000000003E-2</v>
-      </c>
-      <c r="L24">
-        <v>7.8659999999999997E-3</v>
-      </c>
-      <c r="M24">
-        <v>5.6911999999999997E-2</v>
-      </c>
-      <c r="N24" s="1">
-        <v>1.8930599999999998E-18</v>
-      </c>
-      <c r="O24" s="1">
-        <v>1.3916899999999999E-19</v>
-      </c>
-      <c r="P24" s="1">
-        <v>1.14051E-19</v>
-      </c>
-      <c r="Q24" s="1">
-        <v>2.5111099999999999E-20</v>
-      </c>
-      <c r="R24" s="1">
-        <v>1.8167600000000001E-19</v>
-      </c>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="C25" s="1"/>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A26" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="1">
-        <f>B3-B21</f>
-        <v>1.5269681816184276E-25</v>
-      </c>
-      <c r="C26" s="1">
-        <f>C3-C21</f>
-        <v>6.0260193099454558E-25</v>
-      </c>
-      <c r="D26" s="1">
-        <f>D3-D21</f>
-        <v>2.6409919629228419E-25</v>
-      </c>
-      <c r="E26" s="1">
-        <f>E3-E21</f>
-        <v>-1.0879036901010252E-25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B27" s="1">
-        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2389C22-199B-564C-BB09-6A12BD67C173}">
-  <dimension ref="A1:R29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.1640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="22">
-        <f>N6</f>
-        <v>1.46642E-18</v>
-      </c>
-      <c r="C2" s="22">
-        <f>N12</f>
-        <v>1.3471599999999999E-18</v>
-      </c>
-      <c r="D2" s="22">
-        <f>N18</f>
-        <v>2.2857000000000001E-18</v>
-      </c>
-      <c r="E2" s="22">
-        <f>N24</f>
-        <v>1.88991E-18</v>
-      </c>
-      <c r="F2" s="1">
-        <f>SQRT(B2^2+C2^2+D2^2+E2^2)/4</f>
-        <v>8.9307796342550629E-19</v>
-      </c>
-      <c r="I2" t="s">
-        <v>39</v>
-      </c>
-      <c r="J2" t="s">
-        <v>40</v>
-      </c>
-      <c r="K2" t="s">
-        <v>41</v>
-      </c>
-      <c r="L2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A3" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="24">
-        <f>R6</f>
-        <v>2.8112400000000002E-19</v>
-      </c>
-      <c r="C3" s="24">
-        <f>R12</f>
-        <v>2.4182999999999998E-19</v>
-      </c>
-      <c r="D3" s="24">
-        <f>R18</f>
-        <v>2.2777700000000001E-19</v>
-      </c>
-      <c r="E3" s="24">
-        <f>R24</f>
-        <v>1.7349099999999999E-19</v>
-      </c>
-      <c r="F3" s="1">
-        <f t="shared" ref="F3:F4" si="0">SQRT(B3^2+C3^2+D3^2+E3^2)/4</f>
-        <v>1.1712545119603595E-19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" t="s">
-        <v>27</v>
-      </c>
-      <c r="L3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N3" t="s">
-        <v>25</v>
-      </c>
-      <c r="O3" t="s">
-        <v>26</v>
-      </c>
-      <c r="P3" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>28</v>
-      </c>
-      <c r="R3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="23">
-        <f>B3/B2</f>
-        <v>0.19170769629437678</v>
-      </c>
-      <c r="C4" s="23">
-        <f t="shared" ref="C4:E4" si="1">C3/C2</f>
-        <v>0.17951097122836188</v>
-      </c>
-      <c r="D4" s="23">
-        <f t="shared" si="1"/>
-        <v>9.9653060331627075E-2</v>
-      </c>
-      <c r="E4" s="28">
-        <f t="shared" si="1"/>
-        <v>9.1798551253763405E-2</v>
-      </c>
-      <c r="F4" s="1">
-        <f t="shared" si="0"/>
-        <v>7.3880704541001221E-2</v>
-      </c>
-      <c r="H4" t="s">
-        <v>30</v>
-      </c>
-      <c r="I4">
-        <v>0.62288500000000002</v>
-      </c>
-      <c r="J4">
-        <v>0.109403</v>
-      </c>
-      <c r="K4">
-        <v>4.5337000000000002E-2</v>
-      </c>
-      <c r="L4">
-        <v>6.6709999999999998E-3</v>
-      </c>
-      <c r="M4">
-        <v>0.118612</v>
-      </c>
-      <c r="N4" s="1">
-        <v>1.92348E-18</v>
-      </c>
-      <c r="O4" s="1">
-        <v>3.4923800000000002E-19</v>
-      </c>
-      <c r="P4" s="1">
-        <v>1.44727E-19</v>
-      </c>
-      <c r="Q4" s="1">
-        <v>2.1296100000000001E-20</v>
-      </c>
-      <c r="R4" s="1">
-        <v>3.7863699999999999E-19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" s="37"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="H5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5">
-        <v>0.30293599999999998</v>
-      </c>
-      <c r="J5">
-        <v>0.12731100000000001</v>
-      </c>
-      <c r="K5">
-        <v>2.3862999999999999E-2</v>
-      </c>
-      <c r="L5">
-        <v>6.6709999999999998E-3</v>
-      </c>
-      <c r="M5">
-        <v>0.12970000000000001</v>
-      </c>
-      <c r="N5" s="1">
-        <v>9.0212999999999999E-19</v>
-      </c>
-      <c r="O5" s="1">
-        <v>4.0640499999999998E-19</v>
-      </c>
-      <c r="P5" s="1">
-        <v>7.6175300000000001E-20</v>
-      </c>
-      <c r="Q5" s="1">
-        <v>2.1296100000000001E-20</v>
-      </c>
-      <c r="R5" s="1">
-        <v>4.1403100000000001E-19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="38"/>
-      <c r="F6" s="1"/>
-      <c r="H6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I6">
-        <v>0.47970600000000002</v>
-      </c>
-      <c r="J6">
-        <v>8.3918999999999994E-2</v>
-      </c>
-      <c r="K6">
-        <v>2.5856000000000001E-2</v>
-      </c>
-      <c r="L6">
-        <v>6.6709999999999998E-3</v>
-      </c>
-      <c r="M6">
-        <v>8.8065000000000004E-2</v>
-      </c>
-      <c r="N6" s="1">
-        <v>1.46642E-18</v>
-      </c>
-      <c r="O6" s="1">
-        <v>2.6788900000000001E-19</v>
-      </c>
-      <c r="P6" s="1">
-        <v>8.2538800000000001E-20</v>
-      </c>
-      <c r="Q6" s="1">
-        <v>2.1296100000000001E-20</v>
-      </c>
-      <c r="R6" s="1">
-        <v>2.8112400000000002E-19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A8" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="22">
-        <f>L4</f>
-        <v>6.6709999999999998E-3</v>
-      </c>
-      <c r="C8" s="22">
-        <f>L12</f>
-        <v>7.5370000000000003E-3</v>
-      </c>
-      <c r="D8" s="22">
-        <f>L18</f>
-        <v>7.5810000000000001E-3</v>
-      </c>
-      <c r="E8" s="22">
-        <f>L24</f>
-        <v>7.8659999999999997E-3</v>
-      </c>
-      <c r="F8" s="1">
-        <f>SQRT(B10^2+C10^2+D10^2+E10^2)/4</f>
-        <v>7.1524483572727388E-3</v>
-      </c>
-      <c r="I8" t="s">
-        <v>39</v>
-      </c>
-      <c r="J8" t="s">
-        <v>40</v>
-      </c>
-      <c r="K8" t="s">
-        <v>41</v>
-      </c>
-      <c r="L8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A9" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="24">
-        <f>Q6</f>
-        <v>2.1296100000000001E-20</v>
-      </c>
-      <c r="C9" s="24">
-        <f>Q12</f>
-        <v>2.4059899999999999E-20</v>
-      </c>
-      <c r="D9" s="24">
-        <f>Q18</f>
-        <v>2.4200900000000001E-20</v>
-      </c>
-      <c r="E9" s="24">
-        <f>Q24</f>
-        <v>2.5111099999999999E-20</v>
-      </c>
-      <c r="F9" s="1">
-        <f>SQRT(B11^2+C11^2+D11^2+E11^2)/4</f>
-        <v>0</v>
-      </c>
-      <c r="H9" t="s">
-        <v>24</v>
-      </c>
-      <c r="I9" t="s">
-        <v>25</v>
-      </c>
-      <c r="J9" t="s">
-        <v>26</v>
-      </c>
-      <c r="K9" t="s">
-        <v>27</v>
-      </c>
-      <c r="L9" t="s">
-        <v>28</v>
-      </c>
-      <c r="M9" t="s">
-        <v>29</v>
-      </c>
-      <c r="N9" t="s">
-        <v>25</v>
-      </c>
-      <c r="O9" t="s">
-        <v>26</v>
-      </c>
-      <c r="P9" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>28</v>
-      </c>
-      <c r="R9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A10" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="28">
-        <f>B9/B2</f>
-        <v>1.4522510604056137E-2</v>
-      </c>
-      <c r="C10" s="28">
-        <f>C9/C2</f>
-        <v>1.7859719706642123E-2</v>
-      </c>
-      <c r="D10" s="28">
-        <f>D9/D2</f>
-        <v>1.058795992474953E-2</v>
-      </c>
-      <c r="E10" s="28">
-        <f>E9/E2</f>
-        <v>1.32869290072014E-2</v>
-      </c>
-      <c r="F10" s="3">
-        <f>SQRT(B12^2+C12^2+D12^2+E12^2)/4</f>
-        <v>1.5068494933552588E-2</v>
-      </c>
-      <c r="H10" t="s">
-        <v>30</v>
-      </c>
-      <c r="I10">
-        <v>0.360288</v>
-      </c>
-      <c r="J10">
-        <v>9.3454999999999996E-2</v>
-      </c>
-      <c r="K10">
-        <v>2.6723E-2</v>
-      </c>
-      <c r="L10">
-        <v>7.5370000000000003E-3</v>
-      </c>
-      <c r="M10">
-        <v>9.7491999999999995E-2</v>
-      </c>
-      <c r="N10" s="1">
-        <v>1.08307E-18</v>
-      </c>
-      <c r="O10" s="1">
-        <v>2.9832799999999999E-19</v>
-      </c>
-      <c r="P10" s="1">
-        <v>8.5305099999999998E-20</v>
-      </c>
-      <c r="Q10" s="1">
-        <v>2.4059899999999999E-20</v>
-      </c>
-      <c r="R10" s="1">
-        <v>3.1121600000000002E-19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A11" s="36"/>
-      <c r="B11" s="40"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="H11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I11">
-        <v>0.50922900000000004</v>
-      </c>
-      <c r="J11">
-        <v>0.108885</v>
-      </c>
-      <c r="K11">
-        <v>3.9389E-2</v>
-      </c>
-      <c r="L11">
-        <v>7.5370000000000003E-3</v>
-      </c>
-      <c r="M11">
-        <v>0.116036</v>
-      </c>
-      <c r="N11" s="1">
-        <v>1.5585200000000001E-18</v>
-      </c>
-      <c r="O11" s="1">
-        <v>3.4758499999999999E-19</v>
-      </c>
-      <c r="P11" s="1">
-        <v>1.2573900000000001E-19</v>
-      </c>
-      <c r="Q11" s="1">
-        <v>2.4059899999999999E-20</v>
-      </c>
-      <c r="R11" s="1">
-        <v>3.7041199999999999E-19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A12" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="24">
-        <f>K6</f>
-        <v>2.5856000000000001E-2</v>
-      </c>
-      <c r="C12" s="22">
-        <f>K12</f>
-        <v>2.3181E-2</v>
-      </c>
-      <c r="D12" s="22">
-        <f>K18</f>
-        <v>3.7580000000000002E-2</v>
-      </c>
-      <c r="E12" s="22">
-        <f>K24</f>
-        <v>3.1856000000000002E-2</v>
-      </c>
-      <c r="F12" s="1">
-        <f>SQRT(B14^2+C14^2+D14^2+E14^2)/4</f>
-        <v>2.7197361727229023E-2</v>
-      </c>
-      <c r="H12" t="s">
-        <v>32</v>
-      </c>
-      <c r="I12">
-        <v>0.44301800000000002</v>
-      </c>
-      <c r="J12">
-        <v>7.1726999999999999E-2</v>
-      </c>
-      <c r="K12">
-        <v>2.3181E-2</v>
-      </c>
-      <c r="L12">
-        <v>7.5370000000000003E-3</v>
-      </c>
-      <c r="M12">
-        <v>7.5756000000000004E-2</v>
-      </c>
-      <c r="N12" s="1">
-        <v>1.3471599999999999E-18</v>
-      </c>
-      <c r="O12" s="1">
-        <v>2.2897E-19</v>
-      </c>
-      <c r="P12" s="1">
-        <v>7.3998099999999995E-20</v>
-      </c>
-      <c r="Q12" s="1">
-        <v>2.4059899999999999E-20</v>
-      </c>
-      <c r="R12" s="1">
-        <v>2.4182999999999998E-19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A13" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="24">
-        <f>P6</f>
-        <v>8.2538800000000001E-20</v>
-      </c>
-      <c r="C13" s="24">
-        <f>P12</f>
-        <v>7.3998099999999995E-20</v>
-      </c>
-      <c r="D13" s="24">
-        <f>P18</f>
-        <v>1.1996500000000001E-19</v>
-      </c>
-      <c r="E13" s="24">
-        <f>P24</f>
-        <v>1.0169E-19</v>
-      </c>
-      <c r="F13" s="1">
-        <f>SQRT(B15^2+C15^2+D15^2+E15^2)/4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A14" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="28">
-        <f>B13/B2</f>
-        <v>5.6285920813955073E-2</v>
-      </c>
-      <c r="C14" s="28">
-        <f>C13/C2</f>
-        <v>5.4928961667507943E-2</v>
-      </c>
-      <c r="D14" s="28">
-        <f>D13/D2</f>
-        <v>5.2485015531347073E-2</v>
-      </c>
-      <c r="E14" s="28">
-        <f>E13/E2</f>
-        <v>5.3806795032567689E-2</v>
-      </c>
-      <c r="F14" s="3">
-        <f>SQRT(B16^2+C16^2+D16^2+E16^2)/4</f>
-        <v>3.3247038510031232E-2</v>
-      </c>
-      <c r="I14" t="s">
-        <v>39</v>
-      </c>
-      <c r="J14" t="s">
-        <v>40</v>
-      </c>
-      <c r="K14" t="s">
-        <v>41</v>
-      </c>
-      <c r="L14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A15" s="36"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="H15" t="s">
-        <v>24</v>
-      </c>
-      <c r="I15" t="s">
-        <v>25</v>
-      </c>
-      <c r="J15" t="s">
-        <v>26</v>
-      </c>
-      <c r="K15" t="s">
-        <v>27</v>
-      </c>
-      <c r="L15" t="s">
-        <v>28</v>
-      </c>
-      <c r="M15" t="s">
-        <v>29</v>
-      </c>
-      <c r="N15" t="s">
-        <v>25</v>
-      </c>
-      <c r="O15" t="s">
-        <v>26</v>
-      </c>
-      <c r="P15" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>28</v>
-      </c>
-      <c r="R15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A16" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="22">
-        <f>J6</f>
-        <v>8.3918999999999994E-2</v>
-      </c>
-      <c r="C16" s="22">
-        <f>J12</f>
-        <v>7.1726999999999999E-2</v>
-      </c>
-      <c r="D16" s="22">
-        <f>J18</f>
-        <v>6.0179999999999997E-2</v>
-      </c>
-      <c r="E16" s="22">
-        <f>J24</f>
-        <v>4.3325000000000002E-2</v>
-      </c>
-      <c r="F16" s="1">
-        <f>SQRT(B18^2+C18^2+D18^2+E18^2)/4</f>
-        <v>6.8319166755937813E-2</v>
-      </c>
-      <c r="H16" t="s">
-        <v>30</v>
-      </c>
-      <c r="I16">
-        <v>0.677844</v>
-      </c>
-      <c r="J16">
-        <v>7.8012999999999999E-2</v>
-      </c>
-      <c r="K16">
-        <v>4.6717000000000002E-2</v>
-      </c>
-      <c r="L16">
-        <v>7.5810000000000001E-3</v>
-      </c>
-      <c r="M16">
-        <v>9.1246999999999995E-2</v>
-      </c>
-      <c r="N16" s="1">
-        <v>2.0764400000000001E-18</v>
-      </c>
-      <c r="O16" s="1">
-        <v>2.4903599999999998E-19</v>
-      </c>
-      <c r="P16" s="1">
-        <v>1.49131E-19</v>
-      </c>
-      <c r="Q16" s="1">
-        <v>2.4200900000000001E-20</v>
-      </c>
-      <c r="R16" s="1">
-        <v>2.9128100000000002E-19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A17" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="24">
-        <f>O6</f>
-        <v>2.6788900000000001E-19</v>
-      </c>
-      <c r="C17" s="24">
-        <f>O12</f>
-        <v>2.2897E-19</v>
-      </c>
-      <c r="D17" s="24">
-        <f>O18</f>
-        <v>1.92107E-19</v>
-      </c>
-      <c r="E17" s="24">
-        <f>O24</f>
-        <v>1.38303E-19</v>
-      </c>
-      <c r="F17" s="1">
-        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
-        <v>0</v>
-      </c>
-      <c r="H17" t="s">
-        <v>31</v>
-      </c>
-      <c r="I17">
-        <v>0.80456499999999997</v>
-      </c>
-      <c r="J17">
-        <v>9.1906000000000002E-2</v>
-      </c>
-      <c r="K17">
-        <v>5.8146999999999997E-2</v>
-      </c>
-      <c r="L17">
-        <v>7.5810000000000001E-3</v>
-      </c>
-      <c r="M17">
-        <v>0.109019</v>
-      </c>
-      <c r="N17" s="1">
-        <v>2.48096E-18</v>
-      </c>
-      <c r="O17" s="1">
-        <v>2.9338299999999998E-19</v>
-      </c>
-      <c r="P17" s="1">
-        <v>1.85618E-19</v>
-      </c>
-      <c r="Q17" s="1">
-        <v>2.4200900000000001E-20</v>
-      </c>
-      <c r="R17" s="1">
-        <v>3.4801300000000001E-19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A18" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="23">
-        <f>B17/B2</f>
-        <v>0.18268231475293573</v>
-      </c>
-      <c r="C18" s="23">
-        <f>C17/C2</f>
-        <v>0.16996496333026517</v>
-      </c>
-      <c r="D18" s="28">
-        <f>D17/D2</f>
-        <v>8.4047337795861224E-2</v>
-      </c>
-      <c r="E18" s="28">
-        <f>E17/E2</f>
-        <v>7.317967522262965E-2</v>
-      </c>
-      <c r="F18" s="3">
-        <f>SQRT(B20^2+C20^2+D20^2+E20^2)/4</f>
-        <v>0</v>
-      </c>
-      <c r="H18" t="s">
-        <v>32</v>
-      </c>
-      <c r="I18">
-        <v>0.74339699999999997</v>
-      </c>
-      <c r="J18">
-        <v>6.0179999999999997E-2</v>
-      </c>
-      <c r="K18">
-        <v>3.7580000000000002E-2</v>
-      </c>
-      <c r="L18">
-        <v>7.5810000000000001E-3</v>
-      </c>
-      <c r="M18">
-        <v>7.1354000000000001E-2</v>
-      </c>
-      <c r="N18" s="1">
-        <v>2.2857000000000001E-18</v>
-      </c>
-      <c r="O18" s="1">
-        <v>1.92107E-19</v>
-      </c>
-      <c r="P18" s="1">
-        <v>1.1996500000000001E-19</v>
-      </c>
-      <c r="Q18" s="1">
-        <v>2.4200900000000001E-20</v>
-      </c>
-      <c r="R18" s="1">
-        <v>2.2777700000000001E-19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A19" s="36"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A20" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="I20" t="s">
-        <v>39</v>
-      </c>
-      <c r="J20" t="s">
-        <v>40</v>
-      </c>
-      <c r="K20" t="s">
-        <v>41</v>
-      </c>
-      <c r="L20" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="22">
-        <f>SQRT(B17^2+B13^2+B9^2)</f>
-        <v>2.8112398279344651E-19</v>
-      </c>
-      <c r="C21" s="22">
-        <f>SQRT(C17^2+C13^2+C9^2)</f>
-        <v>2.4183022658803429E-19</v>
-      </c>
-      <c r="D21" s="22">
-        <f>SQRT(D17^2+D13^2+D9^2)</f>
-        <v>2.2777704940316089E-19</v>
-      </c>
-      <c r="E21" s="22">
-        <f>SQRT(E17^2+E13^2+E9^2)</f>
-        <v>1.7349104660532197E-19</v>
-      </c>
-      <c r="H21" t="s">
-        <v>24</v>
-      </c>
-      <c r="I21" t="s">
-        <v>25</v>
-      </c>
-      <c r="J21" t="s">
-        <v>26</v>
-      </c>
-      <c r="K21" t="s">
-        <v>27</v>
-      </c>
-      <c r="L21" t="s">
-        <v>28</v>
-      </c>
-      <c r="M21" t="s">
-        <v>29</v>
-      </c>
-      <c r="N21" t="s">
-        <v>25</v>
-      </c>
-      <c r="O21" t="s">
-        <v>26</v>
-      </c>
-      <c r="P21" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>28</v>
-      </c>
-      <c r="R21" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A22" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="23">
-        <f>B21/B2</f>
-        <v>0.19170768456066237</v>
-      </c>
-      <c r="C22" s="23">
-        <f>C21/C2</f>
-        <v>0.17951113942518654</v>
-      </c>
-      <c r="D22" s="23">
-        <f>D21/D2</f>
-        <v>9.9653081945645039E-2</v>
-      </c>
-      <c r="E22" s="28">
-        <f>E21/E2</f>
-        <v>9.1798575913838207E-2</v>
-      </c>
-      <c r="H22" t="s">
-        <v>30</v>
-      </c>
-      <c r="I22">
-        <v>0.57918899999999995</v>
-      </c>
-      <c r="J22">
-        <v>5.5905999999999997E-2</v>
-      </c>
-      <c r="K22">
-        <v>4.0346E-2</v>
-      </c>
-      <c r="L22">
-        <v>7.8659999999999997E-3</v>
-      </c>
-      <c r="M22">
-        <v>6.9390999999999994E-2</v>
-      </c>
-      <c r="N22" s="1">
-        <v>1.74859E-18</v>
-      </c>
-      <c r="O22" s="1">
-        <v>1.78465E-19</v>
-      </c>
-      <c r="P22" s="1">
-        <v>1.2879299999999999E-19</v>
-      </c>
-      <c r="Q22" s="1">
-        <v>2.5111099999999999E-20</v>
-      </c>
-      <c r="R22" s="1">
-        <v>2.21513E-19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A23" s="6"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="H23" t="s">
-        <v>31</v>
-      </c>
-      <c r="I23">
-        <v>0.65437100000000004</v>
-      </c>
-      <c r="J23">
-        <v>6.6559999999999994E-2</v>
-      </c>
-      <c r="K23">
-        <v>4.9153000000000002E-2</v>
-      </c>
-      <c r="L23">
-        <v>7.8659999999999997E-3</v>
-      </c>
-      <c r="M23">
-        <v>8.3114999999999994E-2</v>
-      </c>
-      <c r="N23" s="1">
-        <v>1.9885899999999998E-18</v>
-      </c>
-      <c r="O23" s="1">
-        <v>2.1247599999999999E-19</v>
-      </c>
-      <c r="P23" s="1">
-        <v>1.5690700000000001E-19</v>
-      </c>
-      <c r="Q23" s="1">
-        <v>2.5111099999999999E-20</v>
-      </c>
-      <c r="R23" s="1">
-        <v>2.6532299999999999E-19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A24" s="6"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="5"/>
-      <c r="H24" t="s">
-        <v>32</v>
-      </c>
-      <c r="I24">
-        <v>0.62345799999999996</v>
-      </c>
-      <c r="J24">
-        <v>4.3325000000000002E-2</v>
-      </c>
-      <c r="K24">
-        <v>3.1856000000000002E-2</v>
-      </c>
-      <c r="L24">
-        <v>7.8659999999999997E-3</v>
-      </c>
-      <c r="M24">
-        <v>5.4348E-2</v>
-      </c>
-      <c r="N24" s="1">
-        <v>1.88991E-18</v>
-      </c>
-      <c r="O24" s="1">
-        <v>1.38303E-19</v>
-      </c>
-      <c r="P24" s="1">
-        <v>1.0169E-19</v>
-      </c>
-      <c r="Q24" s="1">
-        <v>2.5111099999999999E-20</v>
-      </c>
-      <c r="R24" s="1">
-        <v>1.7349099999999999E-19</v>
-      </c>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="C25" s="1"/>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A26" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="1">
-        <f>B3-B21</f>
-        <v>1.7206553512660786E-26</v>
-      </c>
-      <c r="C26" s="1">
-        <f>C3-C21</f>
-        <v>-2.2658803431396843E-25</v>
-      </c>
-      <c r="D26" s="1">
-        <f>D3-D21</f>
-        <v>-4.9403160872505303E-26</v>
-      </c>
-      <c r="E26" s="1">
-        <f>E3-E21</f>
-        <v>-4.6605321973691009E-26</v>
-      </c>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B27" s="1">
-        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
-        <v>0</v>
-      </c>
+      <c r="B27" s="1"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B29" s="1"/>

</xml_diff>

<commit_message>
Attempting to run acceptance correction in reverse
</commit_message>
<xml_diff>
--- a/Sheets/ErrorTableRun1.xlsx
+++ b/Sheets/ErrorTableRun1.xlsx
@@ -1,24 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10313"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6531C75-D5E3-544D-B8C6-F5382597B09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B557F89-AE0D-0A48-B0FE-6FC17BE9A720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{C29EF40E-6384-C447-AF4D-92516C1B0710}"/>
   </bookViews>
   <sheets>
-    <sheet name="Run-1 (v2) (HS refit)" sheetId="14" r:id="rId1"/>
-    <sheet name="Run-1 (v2) (HS reweight refit)" sheetId="13" r:id="rId2"/>
-    <sheet name="Run-1 (v2) (HS reweight)" sheetId="12" r:id="rId3"/>
-    <sheet name="Run-1 (v2) (HS)" sheetId="11" r:id="rId4"/>
-    <sheet name="Run-1 (v2)" sheetId="6" r:id="rId5"/>
-    <sheet name="Run-1 (v1)" sheetId="1" r:id="rId6"/>
+    <sheet name="Run-1 (v2) (acceptance reweigh)" sheetId="16" r:id="rId1"/>
+    <sheet name="Run-1 (v2) (HS refit)" sheetId="14" r:id="rId2"/>
+    <sheet name="Run-1 (v2) (HS reweight refit)" sheetId="13" r:id="rId3"/>
+    <sheet name="Run-1 (v2) (HS reweight)" sheetId="12" r:id="rId4"/>
+    <sheet name="Run-1 (v2) (HS)" sheetId="11" r:id="rId5"/>
+    <sheet name="Run-1 (v2)" sheetId="6" r:id="rId6"/>
+    <sheet name="Run-1 (v1)" sheetId="1" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="15" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="55">
   <si>
     <t>Run-1a</t>
   </si>
@@ -166,6 +168,45 @@
   <si>
     <t xml:space="preserve"> dMu [ecm]</t>
   </si>
+  <si>
+    <t> value</t>
+  </si>
+  <si>
+    <t> fit_error</t>
+  </si>
+  <si>
+    <t> dil_error</t>
+  </si>
+  <si>
+    <t> Br_error</t>
+  </si>
+  <si>
+    <t> tot_error</t>
+  </si>
+  <si>
+    <t>NEW</t>
+  </si>
+  <si>
+    <t>OLD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No acceptance weighting </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acceptance weighting </t>
+  </si>
+  <si>
+    <t>Blind tilt angles [mrad]</t>
+  </si>
+  <si>
+    <t>pol0 fit error [mrad]</t>
+  </si>
+  <si>
+    <t>pol0 error [ecm]</t>
+  </si>
+  <si>
+    <t>pol0 error  [%]</t>
+  </si>
 </sst>
 </file>
 
@@ -179,7 +220,7 @@
     <numFmt numFmtId="168" formatCode="0.000%"/>
     <numFmt numFmtId="169" formatCode="0.0000E+00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -207,6 +248,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -348,7 +396,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
@@ -392,6 +440,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -706,6 +760,1053 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2482EF7A-1157-4D44-B170-DFD4B5A9AC0F}">
+  <dimension ref="A1:R29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="22">
+        <f>N6</f>
+        <v>1.39568E-18</v>
+      </c>
+      <c r="C2" s="22">
+        <f>N12</f>
+        <v>1.2767600000000001E-18</v>
+      </c>
+      <c r="D2" s="22">
+        <f>N18</f>
+        <v>2.1938800000000001E-18</v>
+      </c>
+      <c r="E2" s="22">
+        <f>N24</f>
+        <v>1.8048900000000002E-18</v>
+      </c>
+      <c r="F2" s="1">
+        <f>SQRT(B2^2+C2^2+D2^2+E2^2)/4</f>
+        <v>8.5325758590606748E-19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="24">
+        <f>R6</f>
+        <v>2.5917300000000002E-19</v>
+      </c>
+      <c r="C3" s="24">
+        <f>R12</f>
+        <v>2.2214800000000002E-19</v>
+      </c>
+      <c r="D3" s="24">
+        <f>R18</f>
+        <v>1.8957E-19</v>
+      </c>
+      <c r="E3" s="24">
+        <f>R24</f>
+        <v>1.38575E-19</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F4" si="0">SQRT(B3^2+C3^2+D3^2+E3^2)/4</f>
+        <v>1.0357973781041832E-19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="23">
+        <f>B3/B2</f>
+        <v>0.18569657801215181</v>
+      </c>
+      <c r="C4" s="23">
+        <f t="shared" ref="C4:E4" si="1">C3/C2</f>
+        <v>0.17399354616372695</v>
+      </c>
+      <c r="D4" s="23">
+        <f t="shared" si="1"/>
+        <v>8.6408554706729632E-2</v>
+      </c>
+      <c r="E4" s="28">
+        <f t="shared" si="1"/>
+        <v>7.67775321487736E-2</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
+        <v>6.9874083608218965E-2</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4">
+        <v>0.62104700000000002</v>
+      </c>
+      <c r="J4">
+        <v>0.11122700000000001</v>
+      </c>
+      <c r="K4">
+        <v>1.0704999999999999E-2</v>
+      </c>
+      <c r="L4">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M4">
+        <v>0.11194</v>
+      </c>
+      <c r="N4" s="1">
+        <v>1.9176099999999998E-18</v>
+      </c>
+      <c r="O4" s="1">
+        <v>3.5506200000000001E-19</v>
+      </c>
+      <c r="P4" s="1">
+        <v>3.4172699999999998E-20</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R4" s="1">
+        <v>3.57338E-19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" s="37"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="H5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5">
+        <v>0.27496999999999999</v>
+      </c>
+      <c r="J5">
+        <v>0.11677899999999999</v>
+      </c>
+      <c r="K5">
+        <v>4.4889999999999999E-3</v>
+      </c>
+      <c r="L5">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M5">
+        <v>0.11705500000000001</v>
+      </c>
+      <c r="N5" s="1">
+        <v>8.1285600000000003E-19</v>
+      </c>
+      <c r="O5" s="1">
+        <v>3.7278300000000002E-19</v>
+      </c>
+      <c r="P5" s="1">
+        <v>1.43292E-20</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R5" s="1">
+        <v>3.7366600000000002E-19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A6" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="38"/>
+      <c r="F6" s="1"/>
+      <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6">
+        <v>0.45754600000000001</v>
+      </c>
+      <c r="J6">
+        <v>8.0547999999999995E-2</v>
+      </c>
+      <c r="K6">
+        <v>7.6949999999999996E-3</v>
+      </c>
+      <c r="L6">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M6">
+        <v>8.1188999999999997E-2</v>
+      </c>
+      <c r="N6" s="1">
+        <v>1.39568E-18</v>
+      </c>
+      <c r="O6" s="1">
+        <v>2.5712599999999998E-19</v>
+      </c>
+      <c r="P6" s="1">
+        <v>2.45649E-20</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R6" s="1">
+        <v>2.5917300000000002E-19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A8" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="22">
+        <f>L4</f>
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="C8" s="22">
+        <f>L12</f>
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="D8" s="22">
+        <f>L18</f>
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="E8" s="22">
+        <f>L24</f>
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="F8" s="1">
+        <f>SQRT(B10^2+C10^2+D10^2+E10^2)/4</f>
+        <v>7.5132837478750717E-3</v>
+      </c>
+      <c r="I8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A9" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="24">
+        <f>Q6</f>
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="C9" s="24">
+        <f>Q12</f>
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="D9" s="24">
+        <f>Q18</f>
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="E9" s="24">
+        <f>Q24</f>
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="F9" s="1">
+        <f>SQRT(B11^2+C11^2+D11^2+E11^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="K9" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="L9" s="42" t="s">
+        <v>45</v>
+      </c>
+      <c r="M9" s="42" t="s">
+        <v>46</v>
+      </c>
+      <c r="N9" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="O9" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="P9" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q9" s="42" t="s">
+        <v>45</v>
+      </c>
+      <c r="R9" s="42" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A10" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="28">
+        <f>B9/B2</f>
+        <v>1.525858362948527E-2</v>
+      </c>
+      <c r="C10" s="28">
+        <f>C9/C2</f>
+        <v>1.8844497008051627E-2</v>
+      </c>
+      <c r="D10" s="28">
+        <f>D9/D2</f>
+        <v>1.1031095593195617E-2</v>
+      </c>
+      <c r="E10" s="28">
+        <f>E9/E2</f>
+        <v>1.3912814631362574E-2</v>
+      </c>
+      <c r="F10" s="3">
+        <f>SQRT(B12^2+C12^2+D12^2+E12^2)/4</f>
+        <v>4.568095329292067E-3</v>
+      </c>
+      <c r="H10" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="42">
+        <v>0.37762099999999998</v>
+      </c>
+      <c r="J10" s="42">
+        <v>9.5033000000000006E-2</v>
+      </c>
+      <c r="K10" s="42">
+        <v>6.1419999999999999E-3</v>
+      </c>
+      <c r="L10" s="42">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M10" s="42">
+        <v>9.5529000000000003E-2</v>
+      </c>
+      <c r="N10" s="43">
+        <v>1.1384E-18</v>
+      </c>
+      <c r="O10" s="43">
+        <v>3.03366E-19</v>
+      </c>
+      <c r="P10" s="43">
+        <v>1.9606999999999999E-20</v>
+      </c>
+      <c r="Q10" s="43">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R10" s="43">
+        <v>3.0495000000000001E-19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A11" s="36"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="H11" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="42">
+        <v>0.46899299999999999</v>
+      </c>
+      <c r="J11" s="42">
+        <v>9.9851999999999996E-2</v>
+      </c>
+      <c r="K11" s="42">
+        <v>7.7409999999999996E-3</v>
+      </c>
+      <c r="L11" s="42">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M11" s="42">
+        <v>0.100435</v>
+      </c>
+      <c r="N11" s="43">
+        <v>1.4300799999999999E-18</v>
+      </c>
+      <c r="O11" s="43">
+        <v>3.1875099999999998E-19</v>
+      </c>
+      <c r="P11" s="43">
+        <v>2.4710800000000001E-20</v>
+      </c>
+      <c r="Q11" s="43">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R11" s="43">
+        <v>3.2061099999999998E-19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A12" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="24">
+        <f>K6</f>
+        <v>7.6949999999999996E-3</v>
+      </c>
+      <c r="C12" s="22">
+        <f>K12</f>
+        <v>6.8310000000000003E-3</v>
+      </c>
+      <c r="D12" s="22">
+        <f>K18</f>
+        <v>1.1578E-2</v>
+      </c>
+      <c r="E12" s="22">
+        <f>K24</f>
+        <v>9.6930000000000002E-3</v>
+      </c>
+      <c r="F12" s="1">
+        <f>SQRT(B14^2+C14^2+D14^2+E14^2)/4</f>
+        <v>8.5848174442298506E-3</v>
+      </c>
+      <c r="H12" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12" s="42">
+        <v>0.42096299999999998</v>
+      </c>
+      <c r="J12" s="42">
+        <v>6.8843000000000001E-2</v>
+      </c>
+      <c r="K12" s="42">
+        <v>6.8310000000000003E-3</v>
+      </c>
+      <c r="L12" s="42">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M12" s="42">
+        <v>6.9589999999999999E-2</v>
+      </c>
+      <c r="N12" s="43">
+        <v>1.2767600000000001E-18</v>
+      </c>
+      <c r="O12" s="43">
+        <v>2.1976199999999999E-19</v>
+      </c>
+      <c r="P12" s="43">
+        <v>2.1807E-20</v>
+      </c>
+      <c r="Q12" s="43">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R12" s="43">
+        <v>2.2214800000000002E-19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A13" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="24">
+        <f>P6</f>
+        <v>2.45649E-20</v>
+      </c>
+      <c r="C13" s="24">
+        <f>P12</f>
+        <v>2.1807E-20</v>
+      </c>
+      <c r="D13" s="24">
+        <f>P18</f>
+        <v>3.6958099999999998E-20</v>
+      </c>
+      <c r="E13" s="24">
+        <f>P24</f>
+        <v>3.0941599999999999E-20</v>
+      </c>
+      <c r="F13" s="1">
+        <f>SQRT(B15^2+C15^2+D15^2+E15^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="28">
+        <f>B13/B2</f>
+        <v>1.7600667774848103E-2</v>
+      </c>
+      <c r="C14" s="28">
+        <f>C13/C2</f>
+        <v>1.7079952379460507E-2</v>
+      </c>
+      <c r="D14" s="28">
+        <f>D13/D2</f>
+        <v>1.6845998869582657E-2</v>
+      </c>
+      <c r="E14" s="28">
+        <f>E13/E2</f>
+        <v>1.7143205403099354E-2</v>
+      </c>
+      <c r="F14" s="3">
+        <f>SQRT(B16^2+C16^2+D16^2+E16^2)/4</f>
+        <v>3.1909097822956381E-2</v>
+      </c>
+      <c r="I14" t="s">
+        <v>39</v>
+      </c>
+      <c r="J14" t="s">
+        <v>40</v>
+      </c>
+      <c r="K14" t="s">
+        <v>41</v>
+      </c>
+      <c r="L14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A15" s="36"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="H15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" t="s">
+        <v>28</v>
+      </c>
+      <c r="M15" t="s">
+        <v>29</v>
+      </c>
+      <c r="N15" t="s">
+        <v>25</v>
+      </c>
+      <c r="O15" t="s">
+        <v>26</v>
+      </c>
+      <c r="P15" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>28</v>
+      </c>
+      <c r="R15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A16" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="22">
+        <f>J6</f>
+        <v>8.0547999999999995E-2</v>
+      </c>
+      <c r="C16" s="22">
+        <f>J12</f>
+        <v>6.8843000000000001E-2</v>
+      </c>
+      <c r="D16" s="22">
+        <f>J18</f>
+        <v>5.7750000000000003E-2</v>
+      </c>
+      <c r="E16" s="22">
+        <f>J24</f>
+        <v>4.1577000000000003E-2</v>
+      </c>
+      <c r="F16" s="1">
+        <f>SQRT(B18^2+C18^2+D18^2+E18^2)/4</f>
+        <v>6.893649549188427E-2</v>
+      </c>
+      <c r="H16" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16">
+        <v>0.69755699999999998</v>
+      </c>
+      <c r="J16">
+        <v>7.9378000000000004E-2</v>
+      </c>
+      <c r="K16">
+        <v>1.1298000000000001E-2</v>
+      </c>
+      <c r="L16">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M16">
+        <v>8.0534999999999995E-2</v>
+      </c>
+      <c r="N16" s="1">
+        <v>2.13937E-18</v>
+      </c>
+      <c r="O16" s="1">
+        <v>2.53391E-19</v>
+      </c>
+      <c r="P16" s="1">
+        <v>3.6065799999999998E-20</v>
+      </c>
+      <c r="Q16" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R16" s="1">
+        <v>2.57087E-19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A17" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="24">
+        <f>O6</f>
+        <v>2.5712599999999998E-19</v>
+      </c>
+      <c r="C17" s="24">
+        <f>O12</f>
+        <v>2.1976199999999999E-19</v>
+      </c>
+      <c r="D17" s="24">
+        <f>O18</f>
+        <v>1.8435000000000001E-19</v>
+      </c>
+      <c r="E17" s="24">
+        <f>O24</f>
+        <v>1.32722E-19</v>
+      </c>
+      <c r="F17" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17">
+        <v>0.73346999999999996</v>
+      </c>
+      <c r="J17">
+        <v>8.4167000000000006E-2</v>
+      </c>
+      <c r="K17">
+        <v>1.1897E-2</v>
+      </c>
+      <c r="L17">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M17">
+        <v>8.5341E-2</v>
+      </c>
+      <c r="N17" s="1">
+        <v>2.2540099999999998E-18</v>
+      </c>
+      <c r="O17" s="1">
+        <v>2.6867900000000001E-19</v>
+      </c>
+      <c r="P17" s="1">
+        <v>3.7977600000000002E-20</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R17" s="1">
+        <v>2.72427E-19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A18" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="23">
+        <f>B17/B2</f>
+        <v>0.18422990943482745</v>
+      </c>
+      <c r="C18" s="23">
+        <f>C17/C2</f>
+        <v>0.1721247532817444</v>
+      </c>
+      <c r="D18" s="28">
+        <f>D17/D2</f>
+        <v>8.4029208525534665E-2</v>
+      </c>
+      <c r="E18" s="28">
+        <f>E17/E2</f>
+        <v>7.3534675243366626E-2</v>
+      </c>
+      <c r="F18" s="3">
+        <f>SQRT(B20^2+C20^2+D20^2+E20^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18">
+        <v>0.71463399999999999</v>
+      </c>
+      <c r="J18">
+        <v>5.7750000000000003E-2</v>
+      </c>
+      <c r="K18">
+        <v>1.1578E-2</v>
+      </c>
+      <c r="L18">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M18">
+        <v>5.9385E-2</v>
+      </c>
+      <c r="N18" s="1">
+        <v>2.1938800000000001E-18</v>
+      </c>
+      <c r="O18" s="1">
+        <v>1.8435000000000001E-19</v>
+      </c>
+      <c r="P18" s="1">
+        <v>3.6958099999999998E-20</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R18" s="1">
+        <v>1.8957E-19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A19" s="36"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A20" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="I20" t="s">
+        <v>39</v>
+      </c>
+      <c r="J20" t="s">
+        <v>40</v>
+      </c>
+      <c r="K20" t="s">
+        <v>41</v>
+      </c>
+      <c r="L20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A21" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="22">
+        <f>SQRT(B17^2+B13^2+B9^2)</f>
+        <v>2.5917318160492607E-19</v>
+      </c>
+      <c r="C21" s="22">
+        <f>SQRT(C17^2+C13^2+C9^2)</f>
+        <v>2.2214806026839396E-19</v>
+      </c>
+      <c r="D21" s="22">
+        <f>SQRT(D17^2+D13^2+D9^2)</f>
+        <v>1.8956926759477655E-19</v>
+      </c>
+      <c r="E21" s="22">
+        <f>SQRT(E17^2+E13^2+E9^2)</f>
+        <v>1.3857517540227036E-19</v>
+      </c>
+      <c r="H21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I21" t="s">
+        <v>25</v>
+      </c>
+      <c r="J21" t="s">
+        <v>26</v>
+      </c>
+      <c r="K21" t="s">
+        <v>27</v>
+      </c>
+      <c r="L21" t="s">
+        <v>28</v>
+      </c>
+      <c r="M21" t="s">
+        <v>29</v>
+      </c>
+      <c r="N21" t="s">
+        <v>25</v>
+      </c>
+      <c r="O21" t="s">
+        <v>26</v>
+      </c>
+      <c r="P21" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>28</v>
+      </c>
+      <c r="R21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A22" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="23">
+        <f>B21/B2</f>
+        <v>0.18569670813146716</v>
+      </c>
+      <c r="C22" s="23">
+        <f>C21/C2</f>
+        <v>0.17399359336789524</v>
+      </c>
+      <c r="D22" s="23">
+        <f>D21/D2</f>
+        <v>8.6408220866581828E-2</v>
+      </c>
+      <c r="E22" s="28">
+        <f>E21/E2</f>
+        <v>7.6777629330469083E-2</v>
+      </c>
+      <c r="H22" t="s">
+        <v>30</v>
+      </c>
+      <c r="I22">
+        <v>0.59759799999999996</v>
+      </c>
+      <c r="J22">
+        <v>5.6873E-2</v>
+      </c>
+      <c r="K22">
+        <v>9.6799999999999994E-3</v>
+      </c>
+      <c r="L22">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M22">
+        <v>5.8224999999999999E-2</v>
+      </c>
+      <c r="N22" s="1">
+        <v>1.8073499999999999E-18</v>
+      </c>
+      <c r="O22" s="1">
+        <v>1.8155299999999999E-19</v>
+      </c>
+      <c r="P22" s="1">
+        <v>3.0899100000000001E-20</v>
+      </c>
+      <c r="Q22" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R22" s="1">
+        <v>1.8586699999999999E-19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A23" s="6"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="H23" t="s">
+        <v>31</v>
+      </c>
+      <c r="I23">
+        <v>0.59603399999999995</v>
+      </c>
+      <c r="J23">
+        <v>6.0927000000000002E-2</v>
+      </c>
+      <c r="K23">
+        <v>9.7529999999999995E-3</v>
+      </c>
+      <c r="L23">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M23">
+        <v>6.2202E-2</v>
+      </c>
+      <c r="N23" s="1">
+        <v>1.80236E-18</v>
+      </c>
+      <c r="O23" s="1">
+        <v>1.94493E-19</v>
+      </c>
+      <c r="P23" s="1">
+        <v>3.1134100000000002E-20</v>
+      </c>
+      <c r="Q23" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R23" s="1">
+        <v>1.98564E-19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A24" s="6"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="5"/>
+      <c r="H24" t="s">
+        <v>32</v>
+      </c>
+      <c r="I24">
+        <v>0.59682500000000005</v>
+      </c>
+      <c r="J24">
+        <v>4.1577000000000003E-2</v>
+      </c>
+      <c r="K24">
+        <v>9.6930000000000002E-3</v>
+      </c>
+      <c r="L24">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M24">
+        <v>4.3409999999999997E-2</v>
+      </c>
+      <c r="N24" s="1">
+        <v>1.8048900000000002E-18</v>
+      </c>
+      <c r="O24" s="1">
+        <v>1.32722E-19</v>
+      </c>
+      <c r="P24" s="1">
+        <v>3.0941599999999999E-20</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R24" s="1">
+        <v>1.38575E-19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="C25" s="1"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="1">
+        <f>B3-B21</f>
+        <v>-1.8160492604540383E-25</v>
+      </c>
+      <c r="C26" s="1">
+        <f>C3-C21</f>
+        <v>-6.0268393935454527E-26</v>
+      </c>
+      <c r="D26" s="1">
+        <f>D3-D21</f>
+        <v>7.3240522344635355E-25</v>
+      </c>
+      <c r="E26" s="1">
+        <f>E3-E21</f>
+        <v>-1.7540227036094284E-25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B27" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92994925-A506-0B4B-AB86-443EF5CF787E}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1324,7 +2425,7 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="B16" s="22">
         <f>J6</f>
@@ -1382,7 +2483,7 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="B17" s="24">
         <f>O6</f>
@@ -1440,7 +2541,7 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" s="20" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="B18" s="23">
         <f>B17/B2</f>
@@ -1752,7 +2853,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2695A833-57C4-DC4E-AC5C-0BDB90378BCB}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2799,7 +3900,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2389C22-199B-564C-BB09-6A12BD67C173}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3846,7 +4947,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4100744-860F-4E4F-A67B-4D8310BBC4F7}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4861,7 +5962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C92DCEA-3820-F445-BC5D-3C33E4E08EAD}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5865,7 +6966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A38F9457-2941-A549-82F7-48456C4B3AA6}">
   <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -6287,4 +7388,293 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85FF1E83-BE6E-F145-8ADD-5BBBD8D3B9E8}">
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>1.3716199999999999E-18</v>
+      </c>
+      <c r="C3">
+        <v>1.2505999999999999E-18</v>
+      </c>
+      <c r="D3">
+        <v>2.0878699999999999E-18</v>
+      </c>
+      <c r="E3">
+        <v>1.7157500000000001E-18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3">
+        <v>1.39568E-18</v>
+      </c>
+      <c r="I3">
+        <v>1.2767600000000001E-18</v>
+      </c>
+      <c r="J3">
+        <v>2.1938800000000001E-18</v>
+      </c>
+      <c r="K3">
+        <v>1.8048900000000002E-18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>2.6768599999999998E-19</v>
+      </c>
+      <c r="C4">
+        <v>2.3019399999999998E-19</v>
+      </c>
+      <c r="D4">
+        <v>2.2956400000000002E-19</v>
+      </c>
+      <c r="E4">
+        <v>1.7748999999999999E-19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>2.5917300000000002E-19</v>
+      </c>
+      <c r="I4">
+        <v>2.2214800000000002E-19</v>
+      </c>
+      <c r="J4">
+        <v>1.8957E-19</v>
+      </c>
+      <c r="K4">
+        <v>1.38575E-19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>0.19516046718478877</v>
+      </c>
+      <c r="C5">
+        <v>0.18406684791300176</v>
+      </c>
+      <c r="D5">
+        <v>0.10995129007074196</v>
+      </c>
+      <c r="E5">
+        <v>0.1034474719510418</v>
+      </c>
+      <c r="G5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5">
+        <v>0.18569657801215181</v>
+      </c>
+      <c r="I5">
+        <v>0.17399354616372695</v>
+      </c>
+      <c r="J5">
+        <v>8.6408554706729632E-2</v>
+      </c>
+      <c r="K5">
+        <v>7.67775321487736E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7">
+        <v>7.7165999999999998E-2</v>
+      </c>
+      <c r="C7">
+        <v>6.5948000000000007E-2</v>
+      </c>
+      <c r="D7">
+        <v>5.5322000000000003E-2</v>
+      </c>
+      <c r="E7">
+        <v>3.9819E-2</v>
+      </c>
+      <c r="G7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7">
+        <v>8.0547999999999995E-2</v>
+      </c>
+      <c r="I7">
+        <v>6.8843000000000001E-2</v>
+      </c>
+      <c r="J7">
+        <v>5.7750000000000003E-2</v>
+      </c>
+      <c r="K7">
+        <v>4.1577000000000003E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8">
+        <v>2.4633200000000002E-19</v>
+      </c>
+      <c r="C8">
+        <v>2.1052100000000001E-19</v>
+      </c>
+      <c r="D8">
+        <v>1.76599E-19</v>
+      </c>
+      <c r="E8">
+        <v>1.27111E-19</v>
+      </c>
+      <c r="G8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8">
+        <v>2.5712599999999998E-19</v>
+      </c>
+      <c r="I8">
+        <v>2.1976199999999999E-19</v>
+      </c>
+      <c r="J8">
+        <v>1.8435000000000001E-19</v>
+      </c>
+      <c r="K8">
+        <v>1.32722E-19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9">
+        <v>0.17959201528120036</v>
+      </c>
+      <c r="C9">
+        <v>0.16833599872061414</v>
+      </c>
+      <c r="D9">
+        <v>8.4583331337679077E-2</v>
+      </c>
+      <c r="E9">
+        <v>7.4084802564476179E-2</v>
+      </c>
+      <c r="G9" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9">
+        <v>0.18422990943482745</v>
+      </c>
+      <c r="I9">
+        <v>0.1721247532817444</v>
+      </c>
+      <c r="J9">
+        <v>8.4029208525534665E-2</v>
+      </c>
+      <c r="K9">
+        <v>7.3534675243366626E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B11" s="44" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="44"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B11:C11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
About to modify GetTiltAngle.C as part of data driven acceptance study
</commit_message>
<xml_diff>
--- a/Sheets/ErrorTableRun1.xlsx
+++ b/Sheets/ErrorTableRun1.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B557F89-AE0D-0A48-B0FE-6FC17BE9A720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE15B5FE-3103-BB4F-A051-B54B7EB59444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{C29EF40E-6384-C447-AF4D-92516C1B0710}"/>
+    <workbookView xWindow="440" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{C29EF40E-6384-C447-AF4D-92516C1B0710}"/>
   </bookViews>
   <sheets>
-    <sheet name="Run-1 (v2) (acceptance reweigh)" sheetId="16" r:id="rId1"/>
-    <sheet name="Run-1 (v2) (HS refit)" sheetId="14" r:id="rId2"/>
-    <sheet name="Run-1 (v2) (HS reweight refit)" sheetId="13" r:id="rId3"/>
-    <sheet name="Run-1 (v2) (HS reweight)" sheetId="12" r:id="rId4"/>
-    <sheet name="Run-1 (v2) (HS)" sheetId="11" r:id="rId5"/>
-    <sheet name="Run-1 (v2)" sheetId="6" r:id="rId6"/>
-    <sheet name="Run-1 (v1)" sheetId="1" r:id="rId7"/>
-    <sheet name="Sheet1" sheetId="15" r:id="rId8"/>
+    <sheet name="Run-1 (v2) (accCorr)" sheetId="18" r:id="rId1"/>
+    <sheet name="Run-1 (v2) (noVertCorr_accCorr)" sheetId="17" r:id="rId2"/>
+    <sheet name="Run-1 (v2) (acceptance reweigh)" sheetId="16" r:id="rId3"/>
+    <sheet name="Run-1 (v2) (HS refit)" sheetId="14" r:id="rId4"/>
+    <sheet name="Run-1 (v2) (HS reweight refit)" sheetId="13" r:id="rId5"/>
+    <sheet name="Run-1 (v2) (HS reweight)" sheetId="12" r:id="rId6"/>
+    <sheet name="Run-1 (v2) (HS)" sheetId="11" r:id="rId7"/>
+    <sheet name="Run-1 (v2)" sheetId="6" r:id="rId8"/>
+    <sheet name="Run-1 (v1)" sheetId="1" r:id="rId9"/>
+    <sheet name="Sheet1" sheetId="15" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="55">
   <si>
     <t>Run-1a</t>
   </si>
@@ -760,6 +762,2389 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E09ADE20-C0A3-6B45-A44C-298217AE29F2}">
+  <dimension ref="A1:R29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="22">
+        <f>N6</f>
+        <v>1.31224E-18</v>
+      </c>
+      <c r="C2" s="22">
+        <f>N12</f>
+        <v>1.2245600000000001E-18</v>
+      </c>
+      <c r="D2" s="22">
+        <f>N18</f>
+        <v>2.0725800000000002E-18</v>
+      </c>
+      <c r="E2" s="22">
+        <f>N24</f>
+        <v>1.71814E-18</v>
+      </c>
+      <c r="F2" s="1">
+        <f>SQRT(B2^2+C2^2+D2^2+E2^2)/4</f>
+        <v>8.0890025370870047E-19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="24">
+        <f>R6</f>
+        <v>2.5754199999999999E-19</v>
+      </c>
+      <c r="C3" s="24">
+        <f>R12</f>
+        <v>2.2074800000000002E-19</v>
+      </c>
+      <c r="D3" s="24">
+        <f>R18</f>
+        <v>1.8504799999999999E-19</v>
+      </c>
+      <c r="E3" s="24">
+        <f>R24</f>
+        <v>1.3753199999999999E-19</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F4" si="0">SQRT(B3^2+C3^2+D3^2+E3^2)/4</f>
+        <v>1.0253516914820006E-19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="23">
+        <f>B3/B2</f>
+        <v>0.19626135463025055</v>
+      </c>
+      <c r="C4" s="23">
+        <f t="shared" ref="C4:E4" si="1">C3/C2</f>
+        <v>0.18026719801398053</v>
+      </c>
+      <c r="D4" s="23">
+        <f t="shared" si="1"/>
+        <v>8.9283887714828855E-2</v>
+      </c>
+      <c r="E4" s="28">
+        <f t="shared" si="1"/>
+        <v>8.0047027599613532E-2</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
+        <v>7.3055595796164066E-2</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4">
+        <v>0.619228</v>
+      </c>
+      <c r="J4">
+        <v>0.110584</v>
+      </c>
+      <c r="K4">
+        <v>1.0763999999999999E-2</v>
+      </c>
+      <c r="L4">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M4">
+        <v>0.111307</v>
+      </c>
+      <c r="N4" s="1">
+        <v>1.9118000000000001E-18</v>
+      </c>
+      <c r="O4" s="1">
+        <v>3.5301E-19</v>
+      </c>
+      <c r="P4" s="1">
+        <v>3.4361099999999999E-20</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R4" s="1">
+        <v>3.5531699999999998E-19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" s="37"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="H5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5">
+        <v>0.22257099999999999</v>
+      </c>
+      <c r="J5">
+        <v>0.11607099999999999</v>
+      </c>
+      <c r="K5">
+        <v>3.6329999999999999E-3</v>
+      </c>
+      <c r="L5">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M5">
+        <v>0.11631900000000001</v>
+      </c>
+      <c r="N5" s="1">
+        <v>6.4558700000000005E-19</v>
+      </c>
+      <c r="O5" s="1">
+        <v>3.70525E-19</v>
+      </c>
+      <c r="P5" s="1">
+        <v>1.15966E-20</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R5" s="1">
+        <v>3.7131699999999998E-19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A6" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="38"/>
+      <c r="F6" s="1"/>
+      <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6">
+        <v>0.43140800000000001</v>
+      </c>
+      <c r="J6">
+        <v>8.0069000000000001E-2</v>
+      </c>
+      <c r="K6">
+        <v>7.3080000000000003E-3</v>
+      </c>
+      <c r="L6">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M6">
+        <v>8.0678E-2</v>
+      </c>
+      <c r="N6" s="1">
+        <v>1.31224E-18</v>
+      </c>
+      <c r="O6" s="1">
+        <v>2.5559799999999998E-19</v>
+      </c>
+      <c r="P6" s="1">
+        <v>2.3328799999999999E-20</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R6" s="1">
+        <v>2.5754199999999999E-19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A8" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="22">
+        <f>L4</f>
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="C8" s="22">
+        <f>L12</f>
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="D8" s="22">
+        <f>L18</f>
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="E8" s="22">
+        <f>L24</f>
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="F8" s="1">
+        <f>SQRT(B10^2+C10^2+D10^2+E10^2)/4</f>
+        <v>7.9031718095463367E-3</v>
+      </c>
+      <c r="I8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A9" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="24">
+        <f>Q6</f>
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="C9" s="24">
+        <f>Q12</f>
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="D9" s="24">
+        <f>Q18</f>
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="E9" s="24">
+        <f>Q24</f>
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="F9" s="1">
+        <f>SQRT(B11^2+C11^2+D11^2+E11^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" t="s">
+        <v>25</v>
+      </c>
+      <c r="J9" t="s">
+        <v>26</v>
+      </c>
+      <c r="K9" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" t="s">
+        <v>28</v>
+      </c>
+      <c r="M9" t="s">
+        <v>29</v>
+      </c>
+      <c r="N9" t="s">
+        <v>25</v>
+      </c>
+      <c r="O9" t="s">
+        <v>26</v>
+      </c>
+      <c r="P9" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>28</v>
+      </c>
+      <c r="R9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A10" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="28">
+        <f>B9/B2</f>
+        <v>1.6228814850941901E-2</v>
+      </c>
+      <c r="C10" s="28">
+        <f>C9/C2</f>
+        <v>1.9647791859933362E-2</v>
+      </c>
+      <c r="D10" s="28">
+        <f>D9/D2</f>
+        <v>1.1676702467456021E-2</v>
+      </c>
+      <c r="E10" s="28">
+        <f>E9/E2</f>
+        <v>1.4615281641775408E-2</v>
+      </c>
+      <c r="F10" s="3">
+        <f>SQRT(B12^2+C12^2+D12^2+E12^2)/4</f>
+        <v>4.3503907726777837E-3</v>
+      </c>
+      <c r="H10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10">
+        <v>0.37792999999999999</v>
+      </c>
+      <c r="J10">
+        <v>9.4472E-2</v>
+      </c>
+      <c r="K10">
+        <v>6.1260000000000004E-3</v>
+      </c>
+      <c r="L10">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M10">
+        <v>9.4969999999999999E-2</v>
+      </c>
+      <c r="N10" s="1">
+        <v>1.13939E-18</v>
+      </c>
+      <c r="O10" s="1">
+        <v>3.0157600000000001E-19</v>
+      </c>
+      <c r="P10" s="1">
+        <v>1.9556599999999999E-20</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R10" s="1">
+        <v>3.0316599999999999E-19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A11" s="36"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="H11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11">
+        <v>0.43490600000000001</v>
+      </c>
+      <c r="J11">
+        <v>9.9235000000000004E-2</v>
+      </c>
+      <c r="K11">
+        <v>7.1130000000000004E-3</v>
+      </c>
+      <c r="L11">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M11">
+        <v>9.9774000000000002E-2</v>
+      </c>
+      <c r="N11" s="1">
+        <v>1.3212700000000001E-18</v>
+      </c>
+      <c r="O11" s="1">
+        <v>3.1677900000000002E-19</v>
+      </c>
+      <c r="P11" s="1">
+        <v>2.2705899999999999E-20</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R11" s="1">
+        <v>3.1850200000000002E-19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A12" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="24">
+        <f>K6</f>
+        <v>7.3080000000000003E-3</v>
+      </c>
+      <c r="C12" s="22">
+        <f>K12</f>
+        <v>6.5630000000000003E-3</v>
+      </c>
+      <c r="D12" s="22">
+        <f>K18</f>
+        <v>1.0992999999999999E-2</v>
+      </c>
+      <c r="E12" s="22">
+        <f>K24</f>
+        <v>9.2460000000000007E-3</v>
+      </c>
+      <c r="F12" s="1">
+        <f>SQRT(B14^2+C14^2+D14^2+E14^2)/4</f>
+        <v>8.6262346546329156E-3</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12">
+        <v>0.404611</v>
+      </c>
+      <c r="J12">
+        <v>6.8426000000000001E-2</v>
+      </c>
+      <c r="K12">
+        <v>6.5630000000000003E-3</v>
+      </c>
+      <c r="L12">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M12">
+        <v>6.9152000000000005E-2</v>
+      </c>
+      <c r="N12" s="1">
+        <v>1.2245600000000001E-18</v>
+      </c>
+      <c r="O12" s="1">
+        <v>2.1843100000000001E-19</v>
+      </c>
+      <c r="P12" s="1">
+        <v>2.09508E-20</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R12" s="1">
+        <v>2.2074800000000002E-19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A13" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="24">
+        <f>P6</f>
+        <v>2.3328799999999999E-20</v>
+      </c>
+      <c r="C13" s="24">
+        <f>P12</f>
+        <v>2.09508E-20</v>
+      </c>
+      <c r="D13" s="24">
+        <f>P18</f>
+        <v>3.5093199999999999E-20</v>
+      </c>
+      <c r="E13" s="24">
+        <f>P24</f>
+        <v>2.9516500000000002E-20</v>
+      </c>
+      <c r="F13" s="1">
+        <f>SQRT(B15^2+C15^2+D15^2+E15^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="28">
+        <f>B13/B2</f>
+        <v>1.7777845516064133E-2</v>
+      </c>
+      <c r="C14" s="28">
+        <f>C13/C2</f>
+        <v>1.7108839093225321E-2</v>
+      </c>
+      <c r="D14" s="28">
+        <f>D13/D2</f>
+        <v>1.693213289716199E-2</v>
+      </c>
+      <c r="E14" s="28">
+        <f>E13/E2</f>
+        <v>1.7179333465258944E-2</v>
+      </c>
+      <c r="F14" s="3">
+        <f>SQRT(B16^2+C16^2+D16^2+E16^2)/4</f>
+        <v>3.1606929384630202E-2</v>
+      </c>
+      <c r="I14" t="s">
+        <v>39</v>
+      </c>
+      <c r="J14" t="s">
+        <v>40</v>
+      </c>
+      <c r="K14" t="s">
+        <v>41</v>
+      </c>
+      <c r="L14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A15" s="36"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="H15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" t="s">
+        <v>28</v>
+      </c>
+      <c r="M15" t="s">
+        <v>29</v>
+      </c>
+      <c r="N15" t="s">
+        <v>25</v>
+      </c>
+      <c r="O15" t="s">
+        <v>26</v>
+      </c>
+      <c r="P15" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>28</v>
+      </c>
+      <c r="R15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A16" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="22">
+        <f>J6</f>
+        <v>8.0069000000000001E-2</v>
+      </c>
+      <c r="C16" s="22">
+        <f>J12</f>
+        <v>6.8426000000000001E-2</v>
+      </c>
+      <c r="D16" s="22">
+        <f>J18</f>
+        <v>5.6409000000000001E-2</v>
+      </c>
+      <c r="E16" s="22">
+        <f>J24</f>
+        <v>4.1338E-2</v>
+      </c>
+      <c r="F16" s="1">
+        <f>SQRT(B18^2+C18^2+D18^2+E18^2)/4</f>
+        <v>7.2112857116478371E-2</v>
+      </c>
+      <c r="H16" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16">
+        <v>0.671149</v>
+      </c>
+      <c r="J16">
+        <v>7.7551999999999996E-2</v>
+      </c>
+      <c r="K16">
+        <v>1.0887000000000001E-2</v>
+      </c>
+      <c r="L16">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M16">
+        <v>7.8678999999999999E-2</v>
+      </c>
+      <c r="N16" s="1">
+        <v>2.05507E-18</v>
+      </c>
+      <c r="O16" s="1">
+        <v>2.4756299999999999E-19</v>
+      </c>
+      <c r="P16" s="1">
+        <v>3.4752199999999999E-20</v>
+      </c>
+      <c r="Q16" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R16" s="1">
+        <v>2.51159E-19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A17" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="24">
+        <f>O6</f>
+        <v>2.5559799999999998E-19</v>
+      </c>
+      <c r="C17" s="24">
+        <f>O12</f>
+        <v>2.1843100000000001E-19</v>
+      </c>
+      <c r="D17" s="24">
+        <f>O18</f>
+        <v>1.8007100000000001E-19</v>
+      </c>
+      <c r="E17" s="24">
+        <f>O24</f>
+        <v>1.3195900000000001E-19</v>
+      </c>
+      <c r="F17" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17">
+        <v>0.68295300000000003</v>
+      </c>
+      <c r="J17">
+        <v>8.2196000000000005E-2</v>
+      </c>
+      <c r="K17">
+        <v>1.1122999999999999E-2</v>
+      </c>
+      <c r="L17">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M17">
+        <v>8.3291000000000004E-2</v>
+      </c>
+      <c r="N17" s="1">
+        <v>2.0927499999999999E-18</v>
+      </c>
+      <c r="O17" s="1">
+        <v>2.6238799999999998E-19</v>
+      </c>
+      <c r="P17" s="1">
+        <v>3.5507399999999999E-20</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R17" s="1">
+        <v>2.6588299999999999E-19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A18" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="23">
+        <f>B17/B2</f>
+        <v>0.19477991830762664</v>
+      </c>
+      <c r="C18" s="23">
+        <f>C17/C2</f>
+        <v>0.17837508982818318</v>
+      </c>
+      <c r="D18" s="28">
+        <f>D17/D2</f>
+        <v>8.6882532881722291E-2</v>
+      </c>
+      <c r="E18" s="28">
+        <f>E17/E2</f>
+        <v>7.6803403680724511E-2</v>
+      </c>
+      <c r="F18" s="3">
+        <f>SQRT(B20^2+C20^2+D20^2+E20^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18">
+        <v>0.67663600000000002</v>
+      </c>
+      <c r="J18">
+        <v>5.6409000000000001E-2</v>
+      </c>
+      <c r="K18">
+        <v>1.0992999999999999E-2</v>
+      </c>
+      <c r="L18">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M18">
+        <v>5.7969E-2</v>
+      </c>
+      <c r="N18" s="1">
+        <v>2.0725800000000002E-18</v>
+      </c>
+      <c r="O18" s="1">
+        <v>1.8007100000000001E-19</v>
+      </c>
+      <c r="P18" s="1">
+        <v>3.5093199999999999E-20</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R18" s="1">
+        <v>1.8504799999999999E-19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A19" s="36"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A20" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="I20" t="s">
+        <v>39</v>
+      </c>
+      <c r="J20" t="s">
+        <v>40</v>
+      </c>
+      <c r="K20" t="s">
+        <v>41</v>
+      </c>
+      <c r="L20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A21" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="22">
+        <f>SQRT(B17^2+B13^2+B9^2)</f>
+        <v>2.5754241279573733E-19</v>
+      </c>
+      <c r="C21" s="22">
+        <f>SQRT(C17^2+C13^2+C9^2)</f>
+        <v>2.2074853695925143E-19</v>
+      </c>
+      <c r="D21" s="22">
+        <f>SQRT(D17^2+D13^2+D9^2)</f>
+        <v>1.850480512949272E-19</v>
+      </c>
+      <c r="E21" s="22">
+        <f>SQRT(E17^2+E13^2+E9^2)</f>
+        <v>1.3753170106001018E-19</v>
+      </c>
+      <c r="H21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I21" t="s">
+        <v>25</v>
+      </c>
+      <c r="J21" t="s">
+        <v>26</v>
+      </c>
+      <c r="K21" t="s">
+        <v>27</v>
+      </c>
+      <c r="L21" t="s">
+        <v>28</v>
+      </c>
+      <c r="M21" t="s">
+        <v>29</v>
+      </c>
+      <c r="N21" t="s">
+        <v>25</v>
+      </c>
+      <c r="O21" t="s">
+        <v>26</v>
+      </c>
+      <c r="P21" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>28</v>
+      </c>
+      <c r="R21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A22" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="23">
+        <f>B21/B2</f>
+        <v>0.19626166920360402</v>
+      </c>
+      <c r="C22" s="23">
+        <f>C21/C2</f>
+        <v>0.18026763650556232</v>
+      </c>
+      <c r="D22" s="23">
+        <f>D21/D2</f>
+        <v>8.9283912464139956E-2</v>
+      </c>
+      <c r="E22" s="28">
+        <f>E21/E2</f>
+        <v>8.0046853609141377E-2</v>
+      </c>
+      <c r="H22" t="s">
+        <v>30</v>
+      </c>
+      <c r="I22">
+        <v>0.56718400000000002</v>
+      </c>
+      <c r="J22">
+        <v>5.6556000000000002E-2</v>
+      </c>
+      <c r="K22">
+        <v>9.1900000000000003E-3</v>
+      </c>
+      <c r="L22">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M22">
+        <v>5.7835999999999999E-2</v>
+      </c>
+      <c r="N22" s="1">
+        <v>1.7102700000000001E-18</v>
+      </c>
+      <c r="O22" s="1">
+        <v>1.8054100000000001E-19</v>
+      </c>
+      <c r="P22" s="1">
+        <v>2.9335299999999998E-20</v>
+      </c>
+      <c r="Q22" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R22" s="1">
+        <v>1.84624E-19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A23" s="6"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="H23" t="s">
+        <v>31</v>
+      </c>
+      <c r="I23">
+        <v>0.57199900000000004</v>
+      </c>
+      <c r="J23">
+        <v>6.0567000000000003E-2</v>
+      </c>
+      <c r="K23">
+        <v>9.3209999999999994E-3</v>
+      </c>
+      <c r="L23">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M23">
+        <v>6.1781999999999997E-2</v>
+      </c>
+      <c r="N23" s="1">
+        <v>1.72564E-18</v>
+      </c>
+      <c r="O23" s="1">
+        <v>1.93342E-19</v>
+      </c>
+      <c r="P23" s="1">
+        <v>2.9753100000000003E-20</v>
+      </c>
+      <c r="Q23" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R23" s="1">
+        <v>1.9722299999999999E-19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A24" s="6"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="5"/>
+      <c r="H24" t="s">
+        <v>32</v>
+      </c>
+      <c r="I24">
+        <v>0.56965100000000002</v>
+      </c>
+      <c r="J24">
+        <v>4.1338E-2</v>
+      </c>
+      <c r="K24">
+        <v>9.2460000000000007E-3</v>
+      </c>
+      <c r="L24">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M24">
+        <v>4.3083000000000003E-2</v>
+      </c>
+      <c r="N24" s="1">
+        <v>1.71814E-18</v>
+      </c>
+      <c r="O24" s="1">
+        <v>1.3195900000000001E-19</v>
+      </c>
+      <c r="P24" s="1">
+        <v>2.9516500000000002E-20</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R24" s="1">
+        <v>1.3753199999999999E-19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="C25" s="1"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="1">
+        <f>B3-B21</f>
+        <v>-4.127957373482719E-25</v>
+      </c>
+      <c r="C26" s="1">
+        <f>C3-C21</f>
+        <v>-5.3695925140858334E-25</v>
+      </c>
+      <c r="D26" s="1">
+        <f>D3-D21</f>
+        <v>-5.1294927203017416E-26</v>
+      </c>
+      <c r="E26" s="1">
+        <f>E3-E21</f>
+        <v>2.9893998981367922E-25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B27" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85FF1E83-BE6E-F145-8ADD-5BBBD8D3B9E8}">
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>1.3716199999999999E-18</v>
+      </c>
+      <c r="C3">
+        <v>1.2505999999999999E-18</v>
+      </c>
+      <c r="D3">
+        <v>2.0878699999999999E-18</v>
+      </c>
+      <c r="E3">
+        <v>1.7157500000000001E-18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3">
+        <v>1.39568E-18</v>
+      </c>
+      <c r="I3">
+        <v>1.2767600000000001E-18</v>
+      </c>
+      <c r="J3">
+        <v>2.1938800000000001E-18</v>
+      </c>
+      <c r="K3">
+        <v>1.8048900000000002E-18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>2.6768599999999998E-19</v>
+      </c>
+      <c r="C4">
+        <v>2.3019399999999998E-19</v>
+      </c>
+      <c r="D4">
+        <v>2.2956400000000002E-19</v>
+      </c>
+      <c r="E4">
+        <v>1.7748999999999999E-19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>2.5917300000000002E-19</v>
+      </c>
+      <c r="I4">
+        <v>2.2214800000000002E-19</v>
+      </c>
+      <c r="J4">
+        <v>1.8957E-19</v>
+      </c>
+      <c r="K4">
+        <v>1.38575E-19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>0.19516046718478877</v>
+      </c>
+      <c r="C5">
+        <v>0.18406684791300176</v>
+      </c>
+      <c r="D5">
+        <v>0.10995129007074196</v>
+      </c>
+      <c r="E5">
+        <v>0.1034474719510418</v>
+      </c>
+      <c r="G5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5">
+        <v>0.18569657801215181</v>
+      </c>
+      <c r="I5">
+        <v>0.17399354616372695</v>
+      </c>
+      <c r="J5">
+        <v>8.6408554706729632E-2</v>
+      </c>
+      <c r="K5">
+        <v>7.67775321487736E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7">
+        <v>7.7165999999999998E-2</v>
+      </c>
+      <c r="C7">
+        <v>6.5948000000000007E-2</v>
+      </c>
+      <c r="D7">
+        <v>5.5322000000000003E-2</v>
+      </c>
+      <c r="E7">
+        <v>3.9819E-2</v>
+      </c>
+      <c r="G7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7">
+        <v>8.0547999999999995E-2</v>
+      </c>
+      <c r="I7">
+        <v>6.8843000000000001E-2</v>
+      </c>
+      <c r="J7">
+        <v>5.7750000000000003E-2</v>
+      </c>
+      <c r="K7">
+        <v>4.1577000000000003E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8">
+        <v>2.4633200000000002E-19</v>
+      </c>
+      <c r="C8">
+        <v>2.1052100000000001E-19</v>
+      </c>
+      <c r="D8">
+        <v>1.76599E-19</v>
+      </c>
+      <c r="E8">
+        <v>1.27111E-19</v>
+      </c>
+      <c r="G8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8">
+        <v>2.5712599999999998E-19</v>
+      </c>
+      <c r="I8">
+        <v>2.1976199999999999E-19</v>
+      </c>
+      <c r="J8">
+        <v>1.8435000000000001E-19</v>
+      </c>
+      <c r="K8">
+        <v>1.32722E-19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9">
+        <v>0.17959201528120036</v>
+      </c>
+      <c r="C9">
+        <v>0.16833599872061414</v>
+      </c>
+      <c r="D9">
+        <v>8.4583331337679077E-2</v>
+      </c>
+      <c r="E9">
+        <v>7.4084802564476179E-2</v>
+      </c>
+      <c r="G9" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9">
+        <v>0.18422990943482745</v>
+      </c>
+      <c r="I9">
+        <v>0.1721247532817444</v>
+      </c>
+      <c r="J9">
+        <v>8.4029208525534665E-2</v>
+      </c>
+      <c r="K9">
+        <v>7.3534675243366626E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B11" s="44" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="44"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B11:C11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16B1AD79-A50E-8B49-8C0D-508B6150C41B}">
+  <dimension ref="A1:R29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="22">
+        <f>N6</f>
+        <v>1.34928E-18</v>
+      </c>
+      <c r="C2" s="22">
+        <f>N12</f>
+        <v>1.25323E-18</v>
+      </c>
+      <c r="D2" s="22">
+        <f>N18</f>
+        <v>2.09675E-18</v>
+      </c>
+      <c r="E2" s="22">
+        <f>N24</f>
+        <v>1.7775199999999998E-18</v>
+      </c>
+      <c r="F2" s="1">
+        <f>SQRT(B2^2+C2^2+D2^2+E2^2)/4</f>
+        <v>8.2715929028966363E-19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="24">
+        <f>R6</f>
+        <v>2.5759199999999999E-19</v>
+      </c>
+      <c r="C3" s="24">
+        <f>R12</f>
+        <v>2.20795E-19</v>
+      </c>
+      <c r="D3" s="24">
+        <f>R18</f>
+        <v>1.8512699999999999E-19</v>
+      </c>
+      <c r="E3" s="24">
+        <f>R24</f>
+        <v>1.3774699999999999E-19</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F4" si="0">SQRT(B3^2+C3^2+D3^2+E3^2)/4</f>
+        <v>1.0257628643691239E-19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="23">
+        <f>B3/B2</f>
+        <v>0.19091070793311987</v>
+      </c>
+      <c r="C4" s="23">
+        <f t="shared" ref="C4:E4" si="1">C3/C2</f>
+        <v>0.17618074894472682</v>
+      </c>
+      <c r="D4" s="23">
+        <f t="shared" si="1"/>
+        <v>8.8292357219506373E-2</v>
+      </c>
+      <c r="E4" s="28">
+        <f t="shared" si="1"/>
+        <v>7.7493924118997262E-2</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
+        <v>7.127736462273089E-2</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4">
+        <v>0.63151299999999999</v>
+      </c>
+      <c r="J4">
+        <v>0.110587</v>
+      </c>
+      <c r="K4">
+        <v>1.0942E-2</v>
+      </c>
+      <c r="L4">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M4">
+        <v>0.111327</v>
+      </c>
+      <c r="N4" s="1">
+        <v>1.9510200000000001E-18</v>
+      </c>
+      <c r="O4" s="1">
+        <v>3.5301899999999999E-19</v>
+      </c>
+      <c r="P4" s="1">
+        <v>3.4930200000000003E-20</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R4" s="1">
+        <v>3.5538099999999999E-19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" s="37"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="H5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5">
+        <v>0.23222400000000001</v>
+      </c>
+      <c r="J5">
+        <v>0.11607099999999999</v>
+      </c>
+      <c r="K5">
+        <v>3.777E-3</v>
+      </c>
+      <c r="L5">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M5">
+        <v>0.116323</v>
+      </c>
+      <c r="N5" s="1">
+        <v>6.7640000000000002E-19</v>
+      </c>
+      <c r="O5" s="1">
+        <v>3.7052300000000001E-19</v>
+      </c>
+      <c r="P5" s="1">
+        <v>1.20565E-20</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R5" s="1">
+        <v>3.7132999999999999E-19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A6" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="38"/>
+      <c r="F6" s="1"/>
+      <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6">
+        <v>0.44301000000000001</v>
+      </c>
+      <c r="J6">
+        <v>8.0070000000000002E-2</v>
+      </c>
+      <c r="K6">
+        <v>7.4650000000000003E-3</v>
+      </c>
+      <c r="L6">
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="M6">
+        <v>8.0694000000000002E-2</v>
+      </c>
+      <c r="N6" s="1">
+        <v>1.34928E-18</v>
+      </c>
+      <c r="O6" s="1">
+        <v>2.55602E-19</v>
+      </c>
+      <c r="P6" s="1">
+        <v>2.3830299999999999E-20</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="R6" s="1">
+        <v>2.5759199999999999E-19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A8" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="22">
+        <f>L4</f>
+        <v>6.6709999999999998E-3</v>
+      </c>
+      <c r="C8" s="22">
+        <f>L12</f>
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="D8" s="22">
+        <f>L18</f>
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="E8" s="22">
+        <f>L24</f>
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="F8" s="1">
+        <f>SQRT(B10^2+C10^2+D10^2+E10^2)/4</f>
+        <v>7.7074693834888212E-3</v>
+      </c>
+      <c r="I8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A9" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="24">
+        <f>Q6</f>
+        <v>2.1296100000000001E-20</v>
+      </c>
+      <c r="C9" s="24">
+        <f>Q12</f>
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="D9" s="24">
+        <f>Q18</f>
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="E9" s="24">
+        <f>Q24</f>
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="F9" s="1">
+        <f>SQRT(B11^2+C11^2+D11^2+E11^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" t="s">
+        <v>25</v>
+      </c>
+      <c r="J9" t="s">
+        <v>26</v>
+      </c>
+      <c r="K9" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" t="s">
+        <v>28</v>
+      </c>
+      <c r="M9" t="s">
+        <v>29</v>
+      </c>
+      <c r="N9" t="s">
+        <v>25</v>
+      </c>
+      <c r="O9" t="s">
+        <v>26</v>
+      </c>
+      <c r="P9" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>28</v>
+      </c>
+      <c r="R9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A10" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="28">
+        <f>B9/B2</f>
+        <v>1.5783306652436855E-2</v>
+      </c>
+      <c r="C10" s="28">
+        <f>C9/C2</f>
+        <v>1.919831156292141E-2</v>
+      </c>
+      <c r="D10" s="28">
+        <f>D9/D2</f>
+        <v>1.1542100870394659E-2</v>
+      </c>
+      <c r="E10" s="28">
+        <f>E9/E2</f>
+        <v>1.4127042171114813E-2</v>
+      </c>
+      <c r="F10" s="3">
+        <f>SQRT(B12^2+C12^2+D12^2+E12^2)/4</f>
+        <v>4.4406761731745313E-3</v>
+      </c>
+      <c r="H10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10">
+        <v>0.38904899999999998</v>
+      </c>
+      <c r="J10">
+        <v>9.4473000000000001E-2</v>
+      </c>
+      <c r="K10">
+        <v>6.306E-3</v>
+      </c>
+      <c r="L10">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M10">
+        <v>9.4982999999999998E-2</v>
+      </c>
+      <c r="N10" s="1">
+        <v>1.1748799999999999E-18</v>
+      </c>
+      <c r="O10" s="1">
+        <v>3.0157899999999999E-19</v>
+      </c>
+      <c r="P10" s="1">
+        <v>2.0130199999999999E-20</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R10" s="1">
+        <v>3.0320600000000001E-19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A11" s="36"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="H11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11">
+        <v>0.441579</v>
+      </c>
+      <c r="J11">
+        <v>9.9235000000000004E-2</v>
+      </c>
+      <c r="K11">
+        <v>7.2150000000000001E-3</v>
+      </c>
+      <c r="L11">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M11">
+        <v>9.9781999999999996E-2</v>
+      </c>
+      <c r="N11" s="1">
+        <v>1.3425700000000001E-18</v>
+      </c>
+      <c r="O11" s="1">
+        <v>3.1678000000000001E-19</v>
+      </c>
+      <c r="P11" s="1">
+        <v>2.30311E-20</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R11" s="1">
+        <v>3.18526E-19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A12" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="24">
+        <f>K6</f>
+        <v>7.4650000000000003E-3</v>
+      </c>
+      <c r="C12" s="22">
+        <f>K12</f>
+        <v>6.7080000000000004E-3</v>
+      </c>
+      <c r="D12" s="22">
+        <f>K18</f>
+        <v>1.1117E-2</v>
+      </c>
+      <c r="E12" s="22">
+        <f>K24</f>
+        <v>9.5499999999999995E-3</v>
+      </c>
+      <c r="F12" s="1">
+        <f>SQRT(B14^2+C14^2+D14^2+E14^2)/4</f>
+        <v>8.6039840111839464E-3</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12">
+        <v>0.41359200000000002</v>
+      </c>
+      <c r="J12">
+        <v>6.8427000000000002E-2</v>
+      </c>
+      <c r="K12">
+        <v>6.7080000000000004E-3</v>
+      </c>
+      <c r="L12">
+        <v>7.5370000000000003E-3</v>
+      </c>
+      <c r="M12">
+        <v>6.9166000000000005E-2</v>
+      </c>
+      <c r="N12" s="1">
+        <v>1.25323E-18</v>
+      </c>
+      <c r="O12" s="1">
+        <v>2.18433E-19</v>
+      </c>
+      <c r="P12" s="1">
+        <v>2.14119E-20</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>2.4059899999999999E-20</v>
+      </c>
+      <c r="R12" s="1">
+        <v>2.20795E-19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A13" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="24">
+        <f>P6</f>
+        <v>2.3830299999999999E-20</v>
+      </c>
+      <c r="C13" s="24">
+        <f>P12</f>
+        <v>2.14119E-20</v>
+      </c>
+      <c r="D13" s="24">
+        <f>P18</f>
+        <v>3.5487199999999998E-20</v>
+      </c>
+      <c r="E13" s="24">
+        <f>P24</f>
+        <v>3.0486800000000002E-20</v>
+      </c>
+      <c r="F13" s="1">
+        <f>SQRT(B15^2+C15^2+D15^2+E15^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="28">
+        <f>B13/B2</f>
+        <v>1.7661493537293963E-2</v>
+      </c>
+      <c r="C14" s="28">
+        <f>C13/C2</f>
+        <v>1.708537140030162E-2</v>
+      </c>
+      <c r="D14" s="28">
+        <f>D13/D2</f>
+        <v>1.6924859902229639E-2</v>
+      </c>
+      <c r="E14" s="28">
+        <f>E13/E2</f>
+        <v>1.7151311940231336E-2</v>
+      </c>
+      <c r="F14" s="3">
+        <f>SQRT(B16^2+C16^2+D16^2+E16^2)/4</f>
+        <v>3.1607416307332048E-2</v>
+      </c>
+      <c r="I14" t="s">
+        <v>39</v>
+      </c>
+      <c r="J14" t="s">
+        <v>40</v>
+      </c>
+      <c r="K14" t="s">
+        <v>41</v>
+      </c>
+      <c r="L14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A15" s="36"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="H15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" t="s">
+        <v>28</v>
+      </c>
+      <c r="M15" t="s">
+        <v>29</v>
+      </c>
+      <c r="N15" t="s">
+        <v>25</v>
+      </c>
+      <c r="O15" t="s">
+        <v>26</v>
+      </c>
+      <c r="P15" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>28</v>
+      </c>
+      <c r="R15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A16" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="22">
+        <f>J6</f>
+        <v>8.0070000000000002E-2</v>
+      </c>
+      <c r="C16" s="22">
+        <f>J12</f>
+        <v>6.8427000000000002E-2</v>
+      </c>
+      <c r="D16" s="22">
+        <f>J18</f>
+        <v>5.6410000000000002E-2</v>
+      </c>
+      <c r="E16" s="22">
+        <f>J24</f>
+        <v>4.1339000000000001E-2</v>
+      </c>
+      <c r="F16" s="1">
+        <f>SQRT(B18^2+C18^2+D18^2+E18^2)/4</f>
+        <v>7.0335129886538159E-2</v>
+      </c>
+      <c r="H16" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16">
+        <v>0.68078000000000005</v>
+      </c>
+      <c r="J16">
+        <v>7.7553999999999998E-2</v>
+      </c>
+      <c r="K16">
+        <v>1.1043000000000001E-2</v>
+      </c>
+      <c r="L16">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M16">
+        <v>7.8701999999999994E-2</v>
+      </c>
+      <c r="N16" s="1">
+        <v>2.0858099999999998E-18</v>
+      </c>
+      <c r="O16" s="1">
+        <v>2.4756800000000001E-19</v>
+      </c>
+      <c r="P16" s="1">
+        <v>3.5250499999999999E-20</v>
+      </c>
+      <c r="Q16" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R16" s="1">
+        <v>2.5123299999999998E-19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A17" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="24">
+        <f>O6</f>
+        <v>2.55602E-19</v>
+      </c>
+      <c r="C17" s="24">
+        <f>O12</f>
+        <v>2.18433E-19</v>
+      </c>
+      <c r="D17" s="24">
+        <f>O18</f>
+        <v>1.8007500000000001E-19</v>
+      </c>
+      <c r="E17" s="24">
+        <f>O24</f>
+        <v>1.3196300000000001E-19</v>
+      </c>
+      <c r="F17" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17">
+        <v>0.68842099999999995</v>
+      </c>
+      <c r="J17">
+        <v>8.2197000000000006E-2</v>
+      </c>
+      <c r="K17">
+        <v>1.1214E-2</v>
+      </c>
+      <c r="L17">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M17">
+        <v>8.3304000000000003E-2</v>
+      </c>
+      <c r="N17" s="1">
+        <v>2.1102000000000001E-18</v>
+      </c>
+      <c r="O17" s="1">
+        <v>2.6239000000000002E-19</v>
+      </c>
+      <c r="P17" s="1">
+        <v>3.5796800000000003E-20</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R17" s="1">
+        <v>2.65924E-19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A18" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="23">
+        <f>B17/B2</f>
+        <v>0.18943584726669038</v>
+      </c>
+      <c r="C18" s="23">
+        <f>C17/C2</f>
+        <v>0.17429601908668002</v>
+      </c>
+      <c r="D18" s="28">
+        <f>D17/D2</f>
+        <v>8.588291403362347E-2</v>
+      </c>
+      <c r="E18" s="28">
+        <f>E17/E2</f>
+        <v>7.4239952293082515E-2</v>
+      </c>
+      <c r="F18" s="3">
+        <f>SQRT(B20^2+C20^2+D20^2+E20^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18">
+        <v>0.68420599999999998</v>
+      </c>
+      <c r="J18">
+        <v>5.6410000000000002E-2</v>
+      </c>
+      <c r="K18">
+        <v>1.1117E-2</v>
+      </c>
+      <c r="L18">
+        <v>7.5810000000000001E-3</v>
+      </c>
+      <c r="M18">
+        <v>5.7993000000000003E-2</v>
+      </c>
+      <c r="N18" s="1">
+        <v>2.09675E-18</v>
+      </c>
+      <c r="O18" s="1">
+        <v>1.8007500000000001E-19</v>
+      </c>
+      <c r="P18" s="1">
+        <v>3.5487199999999998E-20</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>2.4200900000000001E-20</v>
+      </c>
+      <c r="R18" s="1">
+        <v>1.8512699999999999E-19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A19" s="36"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A20" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="I20" t="s">
+        <v>39</v>
+      </c>
+      <c r="J20" t="s">
+        <v>40</v>
+      </c>
+      <c r="K20" t="s">
+        <v>41</v>
+      </c>
+      <c r="L20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A21" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="22">
+        <f>SQRT(B17^2+B13^2+B9^2)</f>
+        <v>2.5759229312481382E-19</v>
+      </c>
+      <c r="C21" s="22">
+        <f>SQRT(C17^2+C13^2+C9^2)</f>
+        <v>2.2079475478058801E-19</v>
+      </c>
+      <c r="D21" s="22">
+        <f>SQRT(D17^2+D13^2+D9^2)</f>
+        <v>1.851270659564668E-19</v>
+      </c>
+      <c r="E21" s="22">
+        <f>SQRT(E17^2+E13^2+E9^2)</f>
+        <v>1.3774703512762082E-19</v>
+      </c>
+      <c r="H21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I21" t="s">
+        <v>25</v>
+      </c>
+      <c r="J21" t="s">
+        <v>26</v>
+      </c>
+      <c r="K21" t="s">
+        <v>27</v>
+      </c>
+      <c r="L21" t="s">
+        <v>28</v>
+      </c>
+      <c r="M21" t="s">
+        <v>29</v>
+      </c>
+      <c r="N21" t="s">
+        <v>25</v>
+      </c>
+      <c r="O21" t="s">
+        <v>26</v>
+      </c>
+      <c r="P21" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>28</v>
+      </c>
+      <c r="R21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A22" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="23">
+        <f>B21/B2</f>
+        <v>0.1909109251784758</v>
+      </c>
+      <c r="C22" s="23">
+        <f>C21/C2</f>
+        <v>0.1761805532748083</v>
+      </c>
+      <c r="D22" s="23">
+        <f>D21/D2</f>
+        <v>8.8292388676030426E-2</v>
+      </c>
+      <c r="E22" s="28">
+        <f>E21/E2</f>
+        <v>7.7493943881149482E-2</v>
+      </c>
+      <c r="H22" t="s">
+        <v>30</v>
+      </c>
+      <c r="I22">
+        <v>0.59076399999999996</v>
+      </c>
+      <c r="J22">
+        <v>5.6557999999999997E-2</v>
+      </c>
+      <c r="K22">
+        <v>9.5720000000000006E-3</v>
+      </c>
+      <c r="L22">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M22">
+        <v>5.79E-2</v>
+      </c>
+      <c r="N22" s="1">
+        <v>1.78554E-18</v>
+      </c>
+      <c r="O22" s="1">
+        <v>1.80547E-19</v>
+      </c>
+      <c r="P22" s="1">
+        <v>3.0556699999999998E-20</v>
+      </c>
+      <c r="Q22" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R22" s="1">
+        <v>1.84828E-19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A23" s="6"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="H23" t="s">
+        <v>31</v>
+      </c>
+      <c r="I23">
+        <v>0.58546699999999996</v>
+      </c>
+      <c r="J23">
+        <v>6.0567999999999997E-2</v>
+      </c>
+      <c r="K23">
+        <v>9.5449999999999997E-3</v>
+      </c>
+      <c r="L23">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M23">
+        <v>6.1817999999999998E-2</v>
+      </c>
+      <c r="N23" s="1">
+        <v>1.76863E-18</v>
+      </c>
+      <c r="O23" s="1">
+        <v>1.93345E-19</v>
+      </c>
+      <c r="P23" s="1">
+        <v>3.0469599999999999E-20</v>
+      </c>
+      <c r="Q23" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R23" s="1">
+        <v>1.97336E-19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A24" s="6"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="5"/>
+      <c r="H24" t="s">
+        <v>32</v>
+      </c>
+      <c r="I24">
+        <v>0.58825099999999997</v>
+      </c>
+      <c r="J24">
+        <v>4.1339000000000001E-2</v>
+      </c>
+      <c r="K24">
+        <v>9.5499999999999995E-3</v>
+      </c>
+      <c r="L24">
+        <v>7.8659999999999997E-3</v>
+      </c>
+      <c r="M24">
+        <v>4.3151000000000002E-2</v>
+      </c>
+      <c r="N24" s="1">
+        <v>1.7775199999999998E-18</v>
+      </c>
+      <c r="O24" s="1">
+        <v>1.3196300000000001E-19</v>
+      </c>
+      <c r="P24" s="1">
+        <v>3.0486800000000002E-20</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>2.5111099999999999E-20</v>
+      </c>
+      <c r="R24" s="1">
+        <v>1.3774699999999999E-19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="C25" s="1"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="1">
+        <f>B3-B21</f>
+        <v>-2.9312481382843707E-25</v>
+      </c>
+      <c r="C26" s="1">
+        <f>C3-C21</f>
+        <v>2.4521941198471628E-25</v>
+      </c>
+      <c r="D26" s="1">
+        <f>D3-D21</f>
+        <v>-6.5956466801791759E-26</v>
+      </c>
+      <c r="E26" s="1">
+        <f>E3-E21</f>
+        <v>-3.5127620823565165E-26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B27" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2482EF7A-1157-4D44-B170-DFD4B5A9AC0F}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1806,7 +4191,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92994925-A506-0B4B-AB86-443EF5CF787E}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2853,7 +5238,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2695A833-57C4-DC4E-AC5C-0BDB90378BCB}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3900,7 +6285,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2389C22-199B-564C-BB09-6A12BD67C173}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4947,7 +7332,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4100744-860F-4E4F-A67B-4D8310BBC4F7}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5962,7 +8347,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C92DCEA-3820-F445-BC5D-3C33E4E08EAD}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -6966,7 +9351,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A38F9457-2941-A549-82F7-48456C4B3AA6}">
   <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -7388,293 +9773,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85FF1E83-BE6E-F145-8ADD-5BBBD8D3B9E8}">
-  <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H2" t="s">
-        <v>0</v>
-      </c>
-      <c r="I2" t="s">
-        <v>1</v>
-      </c>
-      <c r="J2" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>1.3716199999999999E-18</v>
-      </c>
-      <c r="C3">
-        <v>1.2505999999999999E-18</v>
-      </c>
-      <c r="D3">
-        <v>2.0878699999999999E-18</v>
-      </c>
-      <c r="E3">
-        <v>1.7157500000000001E-18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3">
-        <v>1.39568E-18</v>
-      </c>
-      <c r="I3">
-        <v>1.2767600000000001E-18</v>
-      </c>
-      <c r="J3">
-        <v>2.1938800000000001E-18</v>
-      </c>
-      <c r="K3">
-        <v>1.8048900000000002E-18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
-        <v>2.6768599999999998E-19</v>
-      </c>
-      <c r="C4">
-        <v>2.3019399999999998E-19</v>
-      </c>
-      <c r="D4">
-        <v>2.2956400000000002E-19</v>
-      </c>
-      <c r="E4">
-        <v>1.7748999999999999E-19</v>
-      </c>
-      <c r="G4" t="s">
-        <v>4</v>
-      </c>
-      <c r="H4">
-        <v>2.5917300000000002E-19</v>
-      </c>
-      <c r="I4">
-        <v>2.2214800000000002E-19</v>
-      </c>
-      <c r="J4">
-        <v>1.8957E-19</v>
-      </c>
-      <c r="K4">
-        <v>1.38575E-19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>0.19516046718478877</v>
-      </c>
-      <c r="C5">
-        <v>0.18406684791300176</v>
-      </c>
-      <c r="D5">
-        <v>0.10995129007074196</v>
-      </c>
-      <c r="E5">
-        <v>0.1034474719510418</v>
-      </c>
-      <c r="G5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5">
-        <v>0.18569657801215181</v>
-      </c>
-      <c r="I5">
-        <v>0.17399354616372695</v>
-      </c>
-      <c r="J5">
-        <v>8.6408554706729632E-2</v>
-      </c>
-      <c r="K5">
-        <v>7.67775321487736E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7">
-        <v>7.7165999999999998E-2</v>
-      </c>
-      <c r="C7">
-        <v>6.5948000000000007E-2</v>
-      </c>
-      <c r="D7">
-        <v>5.5322000000000003E-2</v>
-      </c>
-      <c r="E7">
-        <v>3.9819E-2</v>
-      </c>
-      <c r="G7" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7">
-        <v>8.0547999999999995E-2</v>
-      </c>
-      <c r="I7">
-        <v>6.8843000000000001E-2</v>
-      </c>
-      <c r="J7">
-        <v>5.7750000000000003E-2</v>
-      </c>
-      <c r="K7">
-        <v>4.1577000000000003E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8">
-        <v>2.4633200000000002E-19</v>
-      </c>
-      <c r="C8">
-        <v>2.1052100000000001E-19</v>
-      </c>
-      <c r="D8">
-        <v>1.76599E-19</v>
-      </c>
-      <c r="E8">
-        <v>1.27111E-19</v>
-      </c>
-      <c r="G8" t="s">
-        <v>37</v>
-      </c>
-      <c r="H8">
-        <v>2.5712599999999998E-19</v>
-      </c>
-      <c r="I8">
-        <v>2.1976199999999999E-19</v>
-      </c>
-      <c r="J8">
-        <v>1.8435000000000001E-19</v>
-      </c>
-      <c r="K8">
-        <v>1.32722E-19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9">
-        <v>0.17959201528120036</v>
-      </c>
-      <c r="C9">
-        <v>0.16833599872061414</v>
-      </c>
-      <c r="D9">
-        <v>8.4583331337679077E-2</v>
-      </c>
-      <c r="E9">
-        <v>7.4084802564476179E-2</v>
-      </c>
-      <c r="G9" t="s">
-        <v>38</v>
-      </c>
-      <c r="H9">
-        <v>0.18422990943482745</v>
-      </c>
-      <c r="I9">
-        <v>0.1721247532817444</v>
-      </c>
-      <c r="J9">
-        <v>8.4029208525534665E-2</v>
-      </c>
-      <c r="K9">
-        <v>7.3534675243366626E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B11" s="44" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11" s="44"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>34</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B11:C11"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
First draft of BAM talk
</commit_message>
<xml_diff>
--- a/Sheets/ErrorTableRun1.xlsx
+++ b/Sheets/ErrorTableRun1.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9885965B-6F66-F841-B64F-DA11FE40A57C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F0F29A5D-FB46-7B44-B5D3-A216D1763711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="500" windowWidth="13960" windowHeight="17500" activeTab="1" xr2:uid="{C29EF40E-6384-C447-AF4D-92516C1B0710}"/>
+    <workbookView xWindow="4240" yWindow="-18460" windowWidth="23660" windowHeight="17500" xr2:uid="{C29EF40E-6384-C447-AF4D-92516C1B0710}"/>
   </bookViews>
   <sheets>
-    <sheet name="Run-1 (main)" sheetId="19" r:id="rId1"/>
-    <sheet name="Run-1 (noAccCorr) " sheetId="21" r:id="rId2"/>
-    <sheet name="Run-1 (noDilCorr) " sheetId="22" r:id="rId3"/>
-    <sheet name="Run-1 (noVertCorr)" sheetId="20" r:id="rId4"/>
+    <sheet name="Run-1 (BAM)" sheetId="23" r:id="rId1"/>
+    <sheet name="trackReco" sheetId="24" r:id="rId2"/>
+    <sheet name="Run-1 (main)" sheetId="19" r:id="rId3"/>
+    <sheet name="Run-1 (noAccCorr) " sheetId="21" r:id="rId4"/>
+    <sheet name="Run-1 (noDilCorr) " sheetId="22" r:id="rId5"/>
+    <sheet name="Run-1 (noVertCorr)" sheetId="20" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="65">
   <si>
     <t>Run-1a</t>
   </si>
@@ -142,6 +144,96 @@
   </si>
   <si>
     <t>Raw data</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> acc_error</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> align_error</t>
+  </si>
+  <si>
+    <t>Run-1c</t>
+  </si>
+  <si>
+    <t>Run-1d</t>
+  </si>
+  <si>
+    <t>Acceptance (MC stat) [mrad]</t>
+  </si>
+  <si>
+    <t>Acceptance (MC stat) [ecm]</t>
+  </si>
+  <si>
+    <t>Acceptance (MC stat) [%]</t>
+  </si>
+  <si>
+    <t>stat [mrad]</t>
+  </si>
+  <si>
+    <t>stat [ecm]</t>
+  </si>
+  <si>
+    <t>stat [%]</t>
+  </si>
+  <si>
+    <t>Acceptance (align) [mrad]</t>
+  </si>
+  <si>
+    <t>Acceptance (align) [ecm]</t>
+  </si>
+  <si>
+    <t>Acceptance (align) [%]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fit_err</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> acc_err</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> align_err</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> tot_err</t>
+  </si>
+  <si>
+    <t>S12_</t>
+  </si>
+  <si>
+    <t>S18_</t>
+  </si>
+  <si>
+    <t>S12S18_</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> dMu</t>
+  </si>
+  <si>
+    <t>Tracker</t>
+  </si>
+  <si>
+    <t>Station 12</t>
+  </si>
+  <si>
+    <t>Station 18</t>
+  </si>
+  <si>
+    <t>Combined</t>
+  </si>
+  <si>
+    <t>subli</t>
+  </si>
+  <si>
+    <t>Stat [mrad]</t>
+  </si>
+  <si>
+    <t>Stat [ecm]</t>
+  </si>
+  <si>
+    <t>Stat [%]</t>
   </si>
 </sst>
 </file>
@@ -277,7 +369,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -308,6 +400,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -622,6 +718,1744 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC9B9BC8-8FD6-3A42-BC4B-E358FAE336B5}">
+  <dimension ref="A1:T33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1"/>
+      <c r="H1" s="25" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="12">
+        <f>O6</f>
+        <v>1.12729E-18</v>
+      </c>
+      <c r="C2" s="12">
+        <f>O12</f>
+        <v>1.05287E-18</v>
+      </c>
+      <c r="D2" s="12">
+        <f>O18</f>
+        <v>1.8422999999999998E-18</v>
+      </c>
+      <c r="E2" s="12">
+        <f>O24</f>
+        <v>1.56485E-18</v>
+      </c>
+      <c r="F2" s="1">
+        <f>SQRT(B2^2+C2^2+D2^2+E2^2)/4</f>
+        <v>7.1685697638632916E-19</v>
+      </c>
+      <c r="G2">
+        <f>STDEV(B2:E2)</f>
+        <v>3.7311058882275985E-19</v>
+      </c>
+      <c r="H2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" t="s">
+        <v>30</v>
+      </c>
+      <c r="L2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A3" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="14">
+        <f>T6</f>
+        <v>2.7118699999999999E-19</v>
+      </c>
+      <c r="C3" s="14">
+        <f>T12</f>
+        <v>2.3106199999999998E-19</v>
+      </c>
+      <c r="D3" s="14">
+        <f>T18</f>
+        <v>2.3661900000000002E-19</v>
+      </c>
+      <c r="E3" s="14">
+        <f>T24</f>
+        <v>1.8836200000000001E-19</v>
+      </c>
+      <c r="F3" s="1">
+        <f>SQRT(B3^2+C3^2+D3^2+E3^2)/4</f>
+        <v>1.1683343673206314E-19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" t="s">
+        <v>23</v>
+      </c>
+      <c r="O3" t="s">
+        <v>19</v>
+      </c>
+      <c r="P3" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>35</v>
+      </c>
+      <c r="R3" t="s">
+        <v>36</v>
+      </c>
+      <c r="S3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="13">
+        <f>B3/B2</f>
+        <v>0.2405654268200729</v>
+      </c>
+      <c r="C4" s="13">
+        <f t="shared" ref="C4:E4" si="0">C3/C2</f>
+        <v>0.21945919249290033</v>
+      </c>
+      <c r="D4" s="13">
+        <f t="shared" si="0"/>
+        <v>0.1284367366878359</v>
+      </c>
+      <c r="E4" s="16">
+        <f t="shared" si="0"/>
+        <v>0.12037064255359939</v>
+      </c>
+      <c r="F4" s="2">
+        <f>SQRT(B4^2+C4^2+D4^2+E4^2)/4</f>
+        <v>9.2540244174678737E-2</v>
+      </c>
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4">
+        <v>0.49249700000000002</v>
+      </c>
+      <c r="J4">
+        <v>9.9625000000000005E-2</v>
+      </c>
+      <c r="K4">
+        <v>3.3287999999999998E-2</v>
+      </c>
+      <c r="L4">
+        <v>2.7465E-2</v>
+      </c>
+      <c r="M4">
+        <v>7.2979999999999998E-3</v>
+      </c>
+      <c r="N4">
+        <v>0.108816</v>
+      </c>
+      <c r="O4" s="1">
+        <v>1.50131E-18</v>
+      </c>
+      <c r="P4" s="1">
+        <v>3.1802599999999998E-19</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>1.06261E-19</v>
+      </c>
+      <c r="R4" s="1">
+        <v>8.7672999999999999E-20</v>
+      </c>
+      <c r="S4" s="1">
+        <v>2.32968E-20</v>
+      </c>
+      <c r="T4" s="1">
+        <v>3.4736299999999998E-19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A5" s="21"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5">
+        <v>0.180344</v>
+      </c>
+      <c r="J5">
+        <v>0.119869</v>
+      </c>
+      <c r="K5">
+        <v>2.4185999999999999E-2</v>
+      </c>
+      <c r="L5">
+        <v>1.9296000000000001E-2</v>
+      </c>
+      <c r="M5">
+        <v>7.2979999999999998E-3</v>
+      </c>
+      <c r="N5">
+        <v>0.124012</v>
+      </c>
+      <c r="O5" s="1">
+        <v>5.0484499999999999E-19</v>
+      </c>
+      <c r="P5" s="1">
+        <v>3.8264700000000001E-19</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>7.7208699999999998E-20</v>
+      </c>
+      <c r="R5" s="1">
+        <v>6.1596499999999998E-20</v>
+      </c>
+      <c r="S5" s="1">
+        <v>2.32968E-20</v>
+      </c>
+      <c r="T5" s="1">
+        <v>3.9587500000000002E-19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A6" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="22"/>
+      <c r="F6" s="1"/>
+      <c r="H6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6">
+        <v>0.37533100000000003</v>
+      </c>
+      <c r="J6">
+        <v>7.7410000000000007E-2</v>
+      </c>
+      <c r="K6">
+        <v>1.8971999999999999E-2</v>
+      </c>
+      <c r="L6">
+        <v>2.8486000000000001E-2</v>
+      </c>
+      <c r="M6">
+        <v>7.2979999999999998E-3</v>
+      </c>
+      <c r="N6">
+        <v>8.4952E-2</v>
+      </c>
+      <c r="O6" s="1">
+        <v>1.12729E-18</v>
+      </c>
+      <c r="P6" s="1">
+        <v>2.4710800000000001E-19</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>6.0562399999999996E-20</v>
+      </c>
+      <c r="R6" s="1">
+        <v>9.0934599999999998E-20</v>
+      </c>
+      <c r="S6" s="1">
+        <v>2.32968E-20</v>
+      </c>
+      <c r="T6" s="1">
+        <v>2.7118699999999999E-19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A8" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="12">
+        <f>M6</f>
+        <v>7.2979999999999998E-3</v>
+      </c>
+      <c r="C8" s="12">
+        <f>M12</f>
+        <v>8.1720000000000004E-3</v>
+      </c>
+      <c r="D8" s="12">
+        <f>M18</f>
+        <v>8.2430000000000003E-3</v>
+      </c>
+      <c r="E8" s="12">
+        <f>M24</f>
+        <v>9.1450000000000004E-3</v>
+      </c>
+      <c r="F8" s="1">
+        <f>SQRT(B10^2+C10^2+D10^2+E10^2)/4</f>
+        <v>9.9782343759766672E-3</v>
+      </c>
+      <c r="H8" t="s">
+        <v>1</v>
+      </c>
+      <c r="I8" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" t="s">
+        <v>29</v>
+      </c>
+      <c r="K8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A9" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="14">
+        <f>S6</f>
+        <v>2.32968E-20</v>
+      </c>
+      <c r="C9" s="14">
+        <f>S12</f>
+        <v>2.6087E-20</v>
+      </c>
+      <c r="D9" s="14">
+        <f>S18</f>
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="E9" s="14">
+        <f>S24</f>
+        <v>2.91939E-20</v>
+      </c>
+      <c r="F9" s="1">
+        <f>SQRT(B11^2+C11^2+D11^2+E11^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I9" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9" t="s">
+        <v>35</v>
+      </c>
+      <c r="L9" t="s">
+        <v>36</v>
+      </c>
+      <c r="M9" t="s">
+        <v>22</v>
+      </c>
+      <c r="N9" t="s">
+        <v>23</v>
+      </c>
+      <c r="O9" t="s">
+        <v>19</v>
+      </c>
+      <c r="P9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>35</v>
+      </c>
+      <c r="R9" t="s">
+        <v>36</v>
+      </c>
+      <c r="S9" t="s">
+        <v>22</v>
+      </c>
+      <c r="T9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A10" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="16">
+        <f>B9/B2</f>
+        <v>2.0666199469524256E-2</v>
+      </c>
+      <c r="C10" s="16">
+        <f>C9/C2</f>
+        <v>2.4777038000892797E-2</v>
+      </c>
+      <c r="D10" s="16">
+        <f>D9/D2</f>
+        <v>1.4282907235520817E-2</v>
+      </c>
+      <c r="E10" s="16">
+        <f>E9/E2</f>
+        <v>1.8656037319870915E-2</v>
+      </c>
+      <c r="F10" s="2">
+        <f>SQRT(B12^2+C12^2+D12^2+E12^2)/4</f>
+        <v>1.1501908944823029E-2</v>
+      </c>
+      <c r="H10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10">
+        <v>0.30337399999999998</v>
+      </c>
+      <c r="J10">
+        <v>8.5111000000000006E-2</v>
+      </c>
+      <c r="K10">
+        <v>2.0178999999999999E-2</v>
+      </c>
+      <c r="L10">
+        <v>1.294E-2</v>
+      </c>
+      <c r="M10">
+        <v>8.1720000000000004E-3</v>
+      </c>
+      <c r="N10">
+        <v>8.8799000000000003E-2</v>
+      </c>
+      <c r="O10" s="1">
+        <v>8.9590700000000004E-19</v>
+      </c>
+      <c r="P10" s="1">
+        <v>2.7169200000000002E-19</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>6.4414899999999999E-20</v>
+      </c>
+      <c r="R10" s="1">
+        <v>4.1306000000000001E-20</v>
+      </c>
+      <c r="S10" s="1">
+        <v>2.6087E-20</v>
+      </c>
+      <c r="T10" s="1">
+        <v>2.8346500000000002E-19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A11" s="20"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="H11" t="s">
+        <v>25</v>
+      </c>
+      <c r="I11">
+        <v>0.39422800000000002</v>
+      </c>
+      <c r="J11">
+        <v>0.10247000000000001</v>
+      </c>
+      <c r="K11">
+        <v>3.1690000000000003E-2</v>
+      </c>
+      <c r="L11">
+        <v>2.9930999999999999E-2</v>
+      </c>
+      <c r="M11">
+        <v>8.1720000000000004E-3</v>
+      </c>
+      <c r="N11">
+        <v>0.11165600000000001</v>
+      </c>
+      <c r="O11" s="1">
+        <v>1.18593E-18</v>
+      </c>
+      <c r="P11" s="1">
+        <v>3.2710800000000002E-19</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>1.01163E-19</v>
+      </c>
+      <c r="R11" s="1">
+        <v>9.5546899999999998E-20</v>
+      </c>
+      <c r="S11" s="1">
+        <v>2.6087E-20</v>
+      </c>
+      <c r="T11" s="1">
+        <v>3.5643100000000002E-19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A12" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="14">
+        <f>K6</f>
+        <v>1.8971999999999999E-2</v>
+      </c>
+      <c r="C12" s="12">
+        <f>K12</f>
+        <v>1.8539E-2</v>
+      </c>
+      <c r="D12" s="12">
+        <f>K18</f>
+        <v>2.8611000000000001E-2</v>
+      </c>
+      <c r="E12" s="12">
+        <f>K24</f>
+        <v>2.4382000000000001E-2</v>
+      </c>
+      <c r="F12" s="1">
+        <f>SQRT(B14^2+C14^2+D14^2+E14^2)/4</f>
+        <v>2.6192995387233454E-2</v>
+      </c>
+      <c r="G12" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I12">
+        <v>0.352543</v>
+      </c>
+      <c r="J12">
+        <v>6.6155000000000005E-2</v>
+      </c>
+      <c r="K12">
+        <v>1.8539E-2</v>
+      </c>
+      <c r="L12">
+        <v>2.1269E-2</v>
+      </c>
+      <c r="M12">
+        <v>8.1720000000000004E-3</v>
+      </c>
+      <c r="N12">
+        <v>7.2383000000000003E-2</v>
+      </c>
+      <c r="O12" s="1">
+        <v>1.05287E-18</v>
+      </c>
+      <c r="P12" s="1">
+        <v>2.1118E-19</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>5.91793E-20</v>
+      </c>
+      <c r="R12" s="1">
+        <v>6.7895300000000001E-20</v>
+      </c>
+      <c r="S12" s="1">
+        <v>2.6087E-20</v>
+      </c>
+      <c r="T12" s="1">
+        <v>2.3106199999999998E-19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A13" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="14">
+        <f>Q6</f>
+        <v>6.0562399999999996E-20</v>
+      </c>
+      <c r="C13" s="14">
+        <f>Q12</f>
+        <v>5.91793E-20</v>
+      </c>
+      <c r="D13" s="14">
+        <f>Q18</f>
+        <v>9.1332E-20</v>
+      </c>
+      <c r="E13" s="14">
+        <f>Q24</f>
+        <v>7.7833600000000003E-20</v>
+      </c>
+      <c r="F13" s="1">
+        <f>SQRT(B19^2+C19^2+D19^2+E19^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A14" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="16">
+        <f>B13/B2</f>
+        <v>5.3723886488836053E-2</v>
+      </c>
+      <c r="C14" s="16">
+        <f>C13/C2</f>
+        <v>5.6207603977699049E-2</v>
+      </c>
+      <c r="D14" s="16">
+        <f>D13/D2</f>
+        <v>4.9574987787005378E-2</v>
+      </c>
+      <c r="E14" s="16">
+        <f>E13/E2</f>
+        <v>4.9738696999712437E-2</v>
+      </c>
+      <c r="F14" s="2">
+        <f>SQRT(B20^2+C20^2+D20^2+E20^2)/4</f>
+        <v>3.0555205581455348E-2</v>
+      </c>
+      <c r="H14" t="s">
+        <v>37</v>
+      </c>
+      <c r="I14" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" t="s">
+        <v>29</v>
+      </c>
+      <c r="K14" t="s">
+        <v>30</v>
+      </c>
+      <c r="L14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A15" s="20"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="2"/>
+      <c r="H15" t="s">
+        <v>18</v>
+      </c>
+      <c r="I15" t="s">
+        <v>19</v>
+      </c>
+      <c r="J15" t="s">
+        <v>20</v>
+      </c>
+      <c r="K15" t="s">
+        <v>35</v>
+      </c>
+      <c r="L15" t="s">
+        <v>36</v>
+      </c>
+      <c r="M15" t="s">
+        <v>22</v>
+      </c>
+      <c r="N15" t="s">
+        <v>23</v>
+      </c>
+      <c r="O15" t="s">
+        <v>19</v>
+      </c>
+      <c r="P15" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>35</v>
+      </c>
+      <c r="R15" t="s">
+        <v>36</v>
+      </c>
+      <c r="S15" t="s">
+        <v>22</v>
+      </c>
+      <c r="T15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A16" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="14">
+        <f>L6</f>
+        <v>2.8486000000000001E-2</v>
+      </c>
+      <c r="C16" s="12">
+        <f>L12</f>
+        <v>2.1269E-2</v>
+      </c>
+      <c r="D16" s="12">
+        <f>L18</f>
+        <v>4.0446999999999997E-2</v>
+      </c>
+      <c r="E16" s="12">
+        <f>L24</f>
+        <v>3.4731999999999999E-2</v>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="H16" t="s">
+        <v>24</v>
+      </c>
+      <c r="I16">
+        <v>0.56947300000000001</v>
+      </c>
+      <c r="J16">
+        <v>6.9816000000000003E-2</v>
+      </c>
+      <c r="K16">
+        <v>3.5511000000000001E-2</v>
+      </c>
+      <c r="L16">
+        <v>2.9727E-2</v>
+      </c>
+      <c r="M16">
+        <v>8.2430000000000003E-3</v>
+      </c>
+      <c r="N16">
+        <v>8.4183999999999995E-2</v>
+      </c>
+      <c r="O16" s="1">
+        <v>1.72338E-18</v>
+      </c>
+      <c r="P16" s="1">
+        <v>2.2286700000000001E-19</v>
+      </c>
+      <c r="Q16" s="1">
+        <v>1.13359E-19</v>
+      </c>
+      <c r="R16" s="1">
+        <v>9.4894799999999998E-20</v>
+      </c>
+      <c r="S16" s="1">
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="T16" s="1">
+        <v>2.6873299999999998E-19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A17" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="14">
+        <f>R6</f>
+        <v>9.0934599999999998E-20</v>
+      </c>
+      <c r="C17" s="14">
+        <f>R12</f>
+        <v>6.7895300000000001E-20</v>
+      </c>
+      <c r="D17" s="14">
+        <f>R18</f>
+        <v>1.2911700000000001E-19</v>
+      </c>
+      <c r="E17" s="14">
+        <f>R24</f>
+        <v>1.10871E-19</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="H17" t="s">
+        <v>25</v>
+      </c>
+      <c r="I17">
+        <v>0.61294899999999997</v>
+      </c>
+      <c r="J17">
+        <v>8.4864999999999996E-2</v>
+      </c>
+      <c r="K17">
+        <v>4.3679999999999997E-2</v>
+      </c>
+      <c r="L17">
+        <v>4.8372999999999999E-2</v>
+      </c>
+      <c r="M17">
+        <v>8.2430000000000003E-3</v>
+      </c>
+      <c r="N17">
+        <v>0.107322</v>
+      </c>
+      <c r="O17" s="1">
+        <v>1.86217E-18</v>
+      </c>
+      <c r="P17" s="1">
+        <v>2.7090899999999998E-19</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>1.39436E-19</v>
+      </c>
+      <c r="R17" s="1">
+        <v>1.54418E-19</v>
+      </c>
+      <c r="S17" s="1">
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="T17" s="1">
+        <v>3.42595E-19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A18" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="16">
+        <f>B17/B2</f>
+        <v>8.0666554302796969E-2</v>
+      </c>
+      <c r="C18" s="16">
+        <f t="shared" ref="B18:D18" si="1">C17/C2</f>
+        <v>6.4485928937095746E-2</v>
+      </c>
+      <c r="D18" s="16">
+        <f t="shared" si="1"/>
+        <v>7.0084676762742229E-2</v>
+      </c>
+      <c r="E18" s="16">
+        <f>E17/E2</f>
+        <v>7.0850880276064801E-2</v>
+      </c>
+      <c r="H18" t="s">
+        <v>26</v>
+      </c>
+      <c r="I18">
+        <v>0.60672400000000004</v>
+      </c>
+      <c r="J18">
+        <v>5.4514E-2</v>
+      </c>
+      <c r="K18">
+        <v>2.8611000000000001E-2</v>
+      </c>
+      <c r="L18">
+        <v>4.0446999999999997E-2</v>
+      </c>
+      <c r="M18">
+        <v>8.2430000000000003E-3</v>
+      </c>
+      <c r="N18">
+        <v>7.4123999999999995E-2</v>
+      </c>
+      <c r="O18" s="1">
+        <v>1.8422999999999998E-18</v>
+      </c>
+      <c r="P18" s="1">
+        <v>1.74021E-19</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>9.1332E-20</v>
+      </c>
+      <c r="R18" s="1">
+        <v>1.2911700000000001E-19</v>
+      </c>
+      <c r="S18" s="1">
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="T18" s="1">
+        <v>2.3661900000000002E-19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A19" s="26"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="1">
+        <f>SQRT(B22^2+C22^2+D22^2+E22^2)/4</f>
+        <v>8.0564875314760767E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A20" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="14">
+        <f>J6</f>
+        <v>7.7410000000000007E-2</v>
+      </c>
+      <c r="C20" s="14">
+        <f>J12</f>
+        <v>6.6155000000000005E-2</v>
+      </c>
+      <c r="D20" s="14">
+        <f>J18</f>
+        <v>5.4514E-2</v>
+      </c>
+      <c r="E20" s="14">
+        <f>J24</f>
+        <v>3.9967000000000003E-2</v>
+      </c>
+      <c r="F20" s="1">
+        <f>SQRT(B23^2+C23^2+D23^2+E23^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H20" t="s">
+        <v>38</v>
+      </c>
+      <c r="I20" t="s">
+        <v>28</v>
+      </c>
+      <c r="J20" t="s">
+        <v>29</v>
+      </c>
+      <c r="K20" t="s">
+        <v>30</v>
+      </c>
+      <c r="L20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A21" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" s="14">
+        <f>P6</f>
+        <v>2.4710800000000001E-19</v>
+      </c>
+      <c r="C21" s="14">
+        <f>P12</f>
+        <v>2.1118E-19</v>
+      </c>
+      <c r="D21" s="14">
+        <f>P18</f>
+        <v>1.74021E-19</v>
+      </c>
+      <c r="E21" s="14">
+        <f>P24</f>
+        <v>1.2758299999999999E-19</v>
+      </c>
+      <c r="F21" s="2">
+        <f>SQRT(B24^2+C24^2+D24^2+E24^2)/4</f>
+        <v>0</v>
+      </c>
+      <c r="H21" t="s">
+        <v>18</v>
+      </c>
+      <c r="I21" t="s">
+        <v>19</v>
+      </c>
+      <c r="J21" t="s">
+        <v>20</v>
+      </c>
+      <c r="K21" t="s">
+        <v>35</v>
+      </c>
+      <c r="L21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M21" t="s">
+        <v>22</v>
+      </c>
+      <c r="N21" t="s">
+        <v>23</v>
+      </c>
+      <c r="O21" t="s">
+        <v>19</v>
+      </c>
+      <c r="P21" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>35</v>
+      </c>
+      <c r="R21" t="s">
+        <v>36</v>
+      </c>
+      <c r="S21" t="s">
+        <v>22</v>
+      </c>
+      <c r="T21" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A22" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="13">
+        <f>B21/B2</f>
+        <v>0.21920535088575258</v>
+      </c>
+      <c r="C22" s="13">
+        <f>C21/C2</f>
+        <v>0.200575569633478</v>
+      </c>
+      <c r="D22" s="16">
+        <f>D21/D2</f>
+        <v>9.4458557238234819E-2</v>
+      </c>
+      <c r="E22" s="16">
+        <f>E21/E2</f>
+        <v>8.1530498130811258E-2</v>
+      </c>
+      <c r="H22" t="s">
+        <v>24</v>
+      </c>
+      <c r="I22">
+        <v>0.47294999999999998</v>
+      </c>
+      <c r="J22">
+        <v>5.0963000000000001E-2</v>
+      </c>
+      <c r="K22">
+        <v>2.8503000000000001E-2</v>
+      </c>
+      <c r="L22">
+        <v>2.6859000000000001E-2</v>
+      </c>
+      <c r="M22">
+        <v>9.1450000000000004E-3</v>
+      </c>
+      <c r="N22">
+        <v>6.4920000000000005E-2</v>
+      </c>
+      <c r="O22" s="1">
+        <v>1.40033E-18</v>
+      </c>
+      <c r="P22" s="1">
+        <v>1.62684E-19</v>
+      </c>
+      <c r="Q22" s="1">
+        <v>9.0988299999999996E-20</v>
+      </c>
+      <c r="R22" s="1">
+        <v>8.5739800000000005E-20</v>
+      </c>
+      <c r="S22" s="1">
+        <v>2.91939E-20</v>
+      </c>
+      <c r="T22" s="1">
+        <v>2.0723999999999999E-19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A23" s="20"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="H23" t="s">
+        <v>25</v>
+      </c>
+      <c r="I23">
+        <v>0.57680699999999996</v>
+      </c>
+      <c r="J23">
+        <v>6.2549999999999994E-2</v>
+      </c>
+      <c r="K23">
+        <v>3.9248999999999999E-2</v>
+      </c>
+      <c r="L23">
+        <v>4.3192000000000001E-2</v>
+      </c>
+      <c r="M23">
+        <v>9.1450000000000004E-3</v>
+      </c>
+      <c r="N23">
+        <v>8.6036000000000001E-2</v>
+      </c>
+      <c r="O23" s="1">
+        <v>1.73187E-18</v>
+      </c>
+      <c r="P23" s="1">
+        <v>1.99672E-19</v>
+      </c>
+      <c r="Q23" s="1">
+        <v>1.25292E-19</v>
+      </c>
+      <c r="R23" s="1">
+        <v>1.3787800000000001E-19</v>
+      </c>
+      <c r="S23" s="1">
+        <v>2.91939E-20</v>
+      </c>
+      <c r="T23" s="1">
+        <v>2.74645E-19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A24" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="H24" t="s">
+        <v>26</v>
+      </c>
+      <c r="I24">
+        <v>0.52448600000000001</v>
+      </c>
+      <c r="J24">
+        <v>3.9967000000000003E-2</v>
+      </c>
+      <c r="K24">
+        <v>2.4382000000000001E-2</v>
+      </c>
+      <c r="L24">
+        <v>3.4731999999999999E-2</v>
+      </c>
+      <c r="M24">
+        <v>9.1450000000000004E-3</v>
+      </c>
+      <c r="N24">
+        <v>5.9006999999999997E-2</v>
+      </c>
+      <c r="O24" s="1">
+        <v>1.56485E-18</v>
+      </c>
+      <c r="P24" s="1">
+        <v>1.2758299999999999E-19</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>7.7833600000000003E-20</v>
+      </c>
+      <c r="R24" s="1">
+        <v>1.10871E-19</v>
+      </c>
+      <c r="S24" s="1">
+        <v>2.91939E-20</v>
+      </c>
+      <c r="T24" s="1">
+        <v>1.8836200000000001E-19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A25" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="12">
+        <f>SQRT(B21^2+B13^2+B17^2+B9^2)</f>
+        <v>2.7118630187596129E-19</v>
+      </c>
+      <c r="C25" s="12">
+        <f t="shared" ref="C25:E25" si="2">SQRT(C21^2+C13^2+C17^2+C9^2)</f>
+        <v>2.3106164822310947E-19</v>
+      </c>
+      <c r="D25" s="12">
+        <f t="shared" si="2"/>
+        <v>2.3661875955545029E-19</v>
+      </c>
+      <c r="E25" s="12">
+        <f t="shared" si="2"/>
+        <v>1.8836176261696533E-19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A26" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" s="13">
+        <f>B25/B2</f>
+        <v>0.24056480752597936</v>
+      </c>
+      <c r="C26" s="13">
+        <f>C25/C2</f>
+        <v>0.21945885838053081</v>
+      </c>
+      <c r="D26" s="13">
+        <f>D25/D2</f>
+        <v>0.12843660617459171</v>
+      </c>
+      <c r="E26" s="16">
+        <f>E25/E2</f>
+        <v>0.12037049085660947</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A27" s="5"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A28" s="5"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="C29" s="1"/>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A30" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="1">
+        <f>B3-B25</f>
+        <v>6.9812403869814024E-25</v>
+      </c>
+      <c r="C30" s="1">
+        <f>C3-C25</f>
+        <v>3.5177689050995705E-25</v>
+      </c>
+      <c r="D30" s="1">
+        <f>D3-D25</f>
+        <v>2.4044454973675999E-25</v>
+      </c>
+      <c r="E30" s="1">
+        <f>E3-E25</f>
+        <v>2.3738303468222868E-25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B31" s="1">
+        <f>SQRT(B23^2+C23^2+D23^2+E23^2)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1B35896-C4A9-3544-8AEE-A53C2900D99C}">
+  <dimension ref="A1:Q29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="1"/>
+      <c r="E1" s="25" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="12">
+        <f>K6</f>
+        <v>5.3435399999999998E-18</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" t="e">
+        <f>STDEV(B2:B2)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A3" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="14">
+        <f>O6</f>
+        <v>4.9916800000000003E-19</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K3" t="s">
+        <v>56</v>
+      </c>
+      <c r="L3" t="s">
+        <v>48</v>
+      </c>
+      <c r="M3" t="s">
+        <v>49</v>
+      </c>
+      <c r="N3" t="s">
+        <v>50</v>
+      </c>
+      <c r="O3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="13">
+        <f>B3/B2</f>
+        <v>9.3415226610074981E-2</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="E4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4">
+        <v>1.666417</v>
+      </c>
+      <c r="G4">
+        <v>9.6518999999999994E-2</v>
+      </c>
+      <c r="H4">
+        <v>9.8921999999999996E-2</v>
+      </c>
+      <c r="I4">
+        <v>9.7372E-2</v>
+      </c>
+      <c r="J4">
+        <v>0.16906499999999999</v>
+      </c>
+      <c r="K4" s="1">
+        <v>5.3195699999999998E-18</v>
+      </c>
+      <c r="L4" s="1">
+        <v>3.0810900000000001E-19</v>
+      </c>
+      <c r="M4" s="1">
+        <v>3.1578300000000001E-19</v>
+      </c>
+      <c r="N4" s="1">
+        <v>3.1083399999999998E-19</v>
+      </c>
+      <c r="O4" s="1">
+        <v>5.3969299999999996E-19</v>
+      </c>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A5" s="21"/>
+      <c r="B5" s="6"/>
+      <c r="E5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5">
+        <v>1.68001</v>
+      </c>
+      <c r="G5">
+        <v>0.111913</v>
+      </c>
+      <c r="H5">
+        <v>0.109622</v>
+      </c>
+      <c r="I5">
+        <v>0.13072600000000001</v>
+      </c>
+      <c r="J5">
+        <v>0.204036</v>
+      </c>
+      <c r="K5" s="1">
+        <v>5.3629600000000002E-18</v>
+      </c>
+      <c r="L5" s="1">
+        <v>3.5725000000000002E-19</v>
+      </c>
+      <c r="M5" s="1">
+        <v>3.4993899999999999E-19</v>
+      </c>
+      <c r="N5" s="1">
+        <v>4.1730699999999999E-19</v>
+      </c>
+      <c r="O5" s="1">
+        <v>6.5132899999999995E-19</v>
+      </c>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A6" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="E6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6">
+        <v>1.673926</v>
+      </c>
+      <c r="G6">
+        <v>7.3662000000000005E-2</v>
+      </c>
+      <c r="H6">
+        <v>7.8446000000000002E-2</v>
+      </c>
+      <c r="I6">
+        <v>0.113454</v>
+      </c>
+      <c r="J6">
+        <v>0.15637000000000001</v>
+      </c>
+      <c r="K6" s="1">
+        <v>5.3435399999999998E-18</v>
+      </c>
+      <c r="L6" s="1">
+        <v>2.35144E-19</v>
+      </c>
+      <c r="M6" s="1">
+        <v>2.5041800000000001E-19</v>
+      </c>
+      <c r="N6" s="1">
+        <v>3.6217E-19</v>
+      </c>
+      <c r="O6" s="1">
+        <v>4.9916800000000003E-19</v>
+      </c>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A8" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="14">
+        <f>H6</f>
+        <v>7.8446000000000002E-2</v>
+      </c>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A9" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="14">
+        <f>M6</f>
+        <v>2.5041800000000001E-19</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A10" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="16">
+        <f>B9/B2</f>
+        <v>4.6863689614001211E-2</v>
+      </c>
+      <c r="C10" s="2"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A11" s="27"/>
+      <c r="B11" s="28"/>
+      <c r="E11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" t="s">
+        <v>50</v>
+      </c>
+      <c r="J11" t="s">
+        <v>51</v>
+      </c>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A12" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="14">
+        <f>I6</f>
+        <v>0.113454</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="E12" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="1">
+        <v>5.3195699999999998E-18</v>
+      </c>
+      <c r="G12" s="1">
+        <v>3.0810900000000001E-19</v>
+      </c>
+      <c r="H12" s="1">
+        <v>3.1578300000000001E-19</v>
+      </c>
+      <c r="I12" s="1">
+        <v>3.1083399999999998E-19</v>
+      </c>
+      <c r="J12" s="1">
+        <v>5.3969299999999996E-19</v>
+      </c>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A13" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" s="14">
+        <f>N6</f>
+        <v>3.6217E-19</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="E13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" s="1">
+        <v>5.3629600000000002E-18</v>
+      </c>
+      <c r="G13" s="1">
+        <v>3.5725000000000002E-19</v>
+      </c>
+      <c r="H13" s="1">
+        <v>3.4993899999999999E-19</v>
+      </c>
+      <c r="I13" s="1">
+        <v>4.1730699999999999E-19</v>
+      </c>
+      <c r="J13" s="1">
+        <v>6.5132899999999995E-19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A14" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="16">
+        <f>B13/B2</f>
+        <v>6.7777166447710702E-2</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="E14" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="1">
+        <v>5.3435399999999998E-18</v>
+      </c>
+      <c r="G14" s="1">
+        <v>2.35144E-19</v>
+      </c>
+      <c r="H14" s="1">
+        <v>2.5041800000000001E-19</v>
+      </c>
+      <c r="I14" s="1">
+        <v>3.6217E-19</v>
+      </c>
+      <c r="J14" s="1">
+        <v>4.9916800000000003E-19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A15" s="26"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A16" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="14">
+        <f>G6</f>
+        <v>7.3662000000000005E-2</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A17" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="14">
+        <f>L6</f>
+        <v>2.35144E-19</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A18" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="13">
+        <f>B17/B2</f>
+        <v>4.4005284886049323E-2</v>
+      </c>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+      <c r="Q18" s="1"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A19" s="20"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A20" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="1"/>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A21" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" s="12">
+        <f>SQRT(B17^2+B9^2+B13^2)</f>
+        <v>4.991682926228388E-19</v>
+      </c>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A22" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="13">
+        <f>B21/B2</f>
+        <v>9.34152813720565E-2</v>
+      </c>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A23" s="5"/>
+      <c r="B23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A24" s="5"/>
+      <c r="B24" s="3"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="1">
+        <f>B3-B21</f>
+        <v>-2.926228387736565E-25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="B27" s="1" t="e">
+        <f>SQRT(B19^2+#REF!^2+#REF!^2+#REF!^2)/4</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C3FC9BD-960C-B249-A82F-F026B7E24375}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -630,6 +2464,7 @@
     <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.1640625" customWidth="1"/>
   </cols>
@@ -678,6 +2513,10 @@
       <c r="F2" s="1">
         <f>SQRT(B2^2+C2^2+D2^2+E2^2)/4</f>
         <v>7.7754621637157361E-19</v>
+      </c>
+      <c r="G2">
+        <f>STDEV(B2:E2)</f>
+        <v>3.1780943990332736E-19</v>
       </c>
       <c r="I2" t="s">
         <v>28</v>
@@ -1667,10 +3506,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0226FEE3-3B95-A74A-B9AB-147435730300}">
   <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2735,10 +4575,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{573F644D-04DC-0A40-95E2-DB07317B8B26}">
   <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3803,10 +5644,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59F09356-A4A4-3041-AE57-635F1ED1227C}">
   <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4871,5 +6713,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Applied correct dilution/acceptance scaling to blinding
</commit_message>
<xml_diff>
--- a/Sheets/ErrorTableRun1.xlsx
+++ b/Sheets/ErrorTableRun1.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F0F29A5D-FB46-7B44-B5D3-A216D1763711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758931E2-164D-3F44-B7ED-7BB4C4C2352E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4240" yWindow="-18460" windowWidth="23660" windowHeight="17500" xr2:uid="{C29EF40E-6384-C447-AF4D-92516C1B0710}"/>
+    <workbookView xWindow="-5780" yWindow="-21100" windowWidth="38400" windowHeight="21100" xr2:uid="{C29EF40E-6384-C447-AF4D-92516C1B0710}"/>
   </bookViews>
   <sheets>
     <sheet name="Run-1 (BAM)" sheetId="23" r:id="rId1"/>
-    <sheet name="trackReco" sheetId="24" r:id="rId2"/>
-    <sheet name="Run-1 (main)" sheetId="19" r:id="rId3"/>
-    <sheet name="Run-1 (noAccCorr) " sheetId="21" r:id="rId4"/>
-    <sheet name="Run-1 (noDilCorr) " sheetId="22" r:id="rId5"/>
-    <sheet name="Run-1 (noVertCorr)" sheetId="20" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="25" r:id="rId2"/>
+    <sheet name="trackReco" sheetId="24" r:id="rId3"/>
+    <sheet name="Run-1 (main)" sheetId="19" r:id="rId4"/>
+    <sheet name="Run-1 (noAccCorr) " sheetId="21" r:id="rId5"/>
+    <sheet name="Run-1 (noDilCorr) " sheetId="22" r:id="rId6"/>
+    <sheet name="Run-1 (noVertCorr)" sheetId="20" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="65">
   <si>
     <t>Run-1a</t>
   </si>
@@ -240,10 +241,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="182" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -266,6 +268,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -275,7 +282,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -364,12 +371,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -404,6 +435,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -719,7 +761,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC9B9BC8-8FD6-3A42-BC4B-E358FAE336B5}">
-  <dimension ref="A1:T33"/>
+  <dimension ref="A1:AA33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
@@ -733,7 +775,7 @@
     <col min="9" max="9" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>17</v>
       </c>
@@ -754,7 +796,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>5</v>
       </c>
@@ -798,29 +840,29 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="14">
         <f>T6</f>
-        <v>2.7118699999999999E-19</v>
+        <v>2.6099100000000001E-19</v>
       </c>
       <c r="C3" s="14">
         <f>T12</f>
-        <v>2.3106199999999998E-19</v>
+        <v>2.2436100000000001E-19</v>
       </c>
       <c r="D3" s="14">
         <f>T18</f>
-        <v>2.3661900000000002E-19</v>
+        <v>2.1762600000000002E-19</v>
       </c>
       <c r="E3" s="14">
         <f>T24</f>
-        <v>1.8836200000000001E-19</v>
+        <v>1.78195E-19</v>
       </c>
       <c r="F3" s="1">
         <f>SQRT(B3^2+C3^2+D3^2+E3^2)/4</f>
-        <v>1.1683343673206314E-19</v>
+        <v>1.1112175031890697E-19</v>
       </c>
       <c r="H3" t="s">
         <v>18</v>
@@ -861,30 +903,45 @@
       <c r="T3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="V3" t="s">
+        <v>20</v>
+      </c>
+      <c r="W3" t="s">
+        <v>35</v>
+      </c>
+      <c r="X3" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="13">
         <f>B3/B2</f>
-        <v>0.2405654268200729</v>
+        <v>0.23152072669854251</v>
       </c>
       <c r="C4" s="13">
         <f t="shared" ref="C4:E4" si="0">C3/C2</f>
-        <v>0.21945919249290033</v>
+        <v>0.21309468405406176</v>
       </c>
       <c r="D4" s="13">
         <f t="shared" si="0"/>
-        <v>0.1284367366878359</v>
+        <v>0.11812734082397006</v>
       </c>
       <c r="E4" s="16">
         <f t="shared" si="0"/>
-        <v>0.12037064255359939</v>
+        <v>0.11387353420455634</v>
       </c>
       <c r="F4" s="2">
         <f>SQRT(B4^2+C4^2+D4^2+E4^2)/4</f>
-        <v>9.2540244174678737E-2</v>
+        <v>8.8717403064977995E-2</v>
       </c>
       <c r="H4" t="s">
         <v>24</v>
@@ -899,13 +956,13 @@
         <v>3.3287999999999998E-2</v>
       </c>
       <c r="L4">
-        <v>2.7465E-2</v>
+        <v>2.4493999999999998E-2</v>
       </c>
       <c r="M4">
         <v>7.2979999999999998E-3</v>
       </c>
       <c r="N4">
-        <v>0.108816</v>
+        <v>0.10810400000000001</v>
       </c>
       <c r="O4" s="1">
         <v>1.50131E-18</v>
@@ -917,16 +974,37 @@
         <v>1.06261E-19</v>
       </c>
       <c r="R4" s="1">
-        <v>8.7672999999999999E-20</v>
+        <v>7.8189499999999994E-20</v>
       </c>
       <c r="S4" s="1">
         <v>2.32968E-20</v>
       </c>
       <c r="T4" s="1">
-        <v>3.4736299999999998E-19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+        <v>3.45092E-19</v>
+      </c>
+      <c r="V4" s="3">
+        <f>P4/$O$4</f>
+        <v>0.21183233309576302</v>
+      </c>
+      <c r="W4" s="3">
+        <f t="shared" ref="W4:Z4" si="1">Q4/$O$4</f>
+        <v>7.0778853134928835E-2</v>
+      </c>
+      <c r="X4" s="3">
+        <f t="shared" si="1"/>
+        <v>5.2080849391531389E-2</v>
+      </c>
+      <c r="Y4" s="3">
+        <f t="shared" si="1"/>
+        <v>1.551764792081582E-2</v>
+      </c>
+      <c r="Z4" s="3">
+        <f t="shared" si="1"/>
+        <v>0.22986058841944701</v>
+      </c>
+      <c r="AA4" s="1"/>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" s="21"/>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -945,13 +1023,13 @@
         <v>2.4185999999999999E-2</v>
       </c>
       <c r="L5">
-        <v>1.9296000000000001E-2</v>
+        <v>1.08E-4</v>
       </c>
       <c r="M5">
         <v>7.2979999999999998E-3</v>
       </c>
       <c r="N5">
-        <v>0.124012</v>
+        <v>0.122502</v>
       </c>
       <c r="O5" s="1">
         <v>5.0484499999999999E-19</v>
@@ -963,16 +1041,36 @@
         <v>7.7208699999999998E-20</v>
       </c>
       <c r="R5" s="1">
-        <v>6.1596499999999998E-20</v>
+        <v>3.43429E-22</v>
       </c>
       <c r="S5" s="1">
         <v>2.32968E-20</v>
       </c>
       <c r="T5" s="1">
-        <v>3.9587500000000002E-19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+        <v>3.91054E-19</v>
+      </c>
+      <c r="V5" s="3">
+        <f>P5/$O$5</f>
+        <v>0.75794946963919618</v>
+      </c>
+      <c r="W5" s="3">
+        <f t="shared" ref="W5:Z5" si="2">Q5/$O$5</f>
+        <v>0.15293545543681725</v>
+      </c>
+      <c r="X5" s="31">
+        <f>R5/$O$5</f>
+        <v>6.8026622032505031E-4</v>
+      </c>
+      <c r="Y5" s="3">
+        <f t="shared" si="2"/>
+        <v>4.6146440986837546E-2</v>
+      </c>
+      <c r="Z5" s="3">
+        <f t="shared" si="2"/>
+        <v>0.77460210559676734</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
         <v>15</v>
       </c>
@@ -991,13 +1089,13 @@
         <v>1.8971999999999999E-2</v>
       </c>
       <c r="L6">
-        <v>2.8486000000000001E-2</v>
+        <v>1.6702999999999999E-2</v>
       </c>
       <c r="M6">
         <v>7.2979999999999998E-3</v>
       </c>
       <c r="N6">
-        <v>8.4952E-2</v>
+        <v>8.1757999999999997E-2</v>
       </c>
       <c r="O6" s="1">
         <v>1.12729E-18</v>
@@ -1009,16 +1107,36 @@
         <v>6.0562399999999996E-20</v>
       </c>
       <c r="R6" s="1">
-        <v>9.0934599999999998E-20</v>
+        <v>5.3320400000000003E-20</v>
       </c>
       <c r="S6" s="1">
         <v>2.32968E-20</v>
       </c>
       <c r="T6" s="1">
-        <v>2.7118699999999999E-19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+        <v>2.6099100000000001E-19</v>
+      </c>
+      <c r="V6" s="3">
+        <f>P6/$O$6</f>
+        <v>0.21920535088575258</v>
+      </c>
+      <c r="W6" s="4">
+        <f t="shared" ref="W6:Z6" si="3">Q6/$O$6</f>
+        <v>5.3723886488836053E-2</v>
+      </c>
+      <c r="X6" s="4">
+        <f t="shared" si="3"/>
+        <v>4.7299630086313195E-2</v>
+      </c>
+      <c r="Y6" s="4">
+        <f t="shared" si="3"/>
+        <v>2.0666199469524256E-2</v>
+      </c>
+      <c r="Z6" s="3">
+        <f t="shared" si="3"/>
+        <v>0.23152072669854251</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
@@ -1058,7 +1176,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
         <v>6</v>
       </c>
@@ -1121,8 +1239,23 @@
       <c r="T9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="V9" t="s">
+        <v>20</v>
+      </c>
+      <c r="W9" t="s">
+        <v>35</v>
+      </c>
+      <c r="X9" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
         <v>7</v>
       </c>
@@ -1159,13 +1292,13 @@
         <v>2.0178999999999999E-2</v>
       </c>
       <c r="L10">
-        <v>1.294E-2</v>
+        <v>1.3266E-2</v>
       </c>
       <c r="M10">
         <v>8.1720000000000004E-3</v>
       </c>
       <c r="N10">
-        <v>8.8799000000000003E-2</v>
+        <v>8.8846999999999995E-2</v>
       </c>
       <c r="O10" s="1">
         <v>8.9590700000000004E-19</v>
@@ -1177,16 +1310,36 @@
         <v>6.4414899999999999E-20</v>
       </c>
       <c r="R10" s="1">
-        <v>4.1306000000000001E-20</v>
+        <v>4.2347099999999998E-20</v>
       </c>
       <c r="S10" s="1">
         <v>2.6087E-20</v>
       </c>
       <c r="T10" s="1">
-        <v>2.8346500000000002E-19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+        <v>2.8361899999999999E-19</v>
+      </c>
+      <c r="V10" s="3">
+        <f>P10/$O$10</f>
+        <v>0.30325915524714064</v>
+      </c>
+      <c r="W10" s="3">
+        <f t="shared" ref="W10:Z10" si="4">Q10/$O$10</f>
+        <v>7.1899092204882872E-2</v>
+      </c>
+      <c r="X10" s="3">
+        <f t="shared" si="4"/>
+        <v>4.7267294484807015E-2</v>
+      </c>
+      <c r="Y10" s="3">
+        <f t="shared" si="4"/>
+        <v>2.9117977647233471E-2</v>
+      </c>
+      <c r="Z10" s="3">
+        <f t="shared" si="4"/>
+        <v>0.31657192096947562</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A11" s="20"/>
       <c r="B11" s="24"/>
       <c r="C11" s="18"/>
@@ -1205,13 +1358,13 @@
         <v>3.1690000000000003E-2</v>
       </c>
       <c r="L11">
-        <v>2.9930999999999999E-2</v>
+        <v>8.4229999999999999E-3</v>
       </c>
       <c r="M11">
         <v>8.1720000000000004E-3</v>
       </c>
       <c r="N11">
-        <v>0.11165600000000001</v>
+        <v>0.10789899999999999</v>
       </c>
       <c r="O11" s="1">
         <v>1.18593E-18</v>
@@ -1223,16 +1376,36 @@
         <v>1.01163E-19</v>
       </c>
       <c r="R11" s="1">
-        <v>9.5546899999999998E-20</v>
+        <v>2.68895E-20</v>
       </c>
       <c r="S11" s="1">
         <v>2.6087E-20</v>
       </c>
       <c r="T11" s="1">
-        <v>3.5643100000000002E-19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+        <v>3.4443700000000001E-19</v>
+      </c>
+      <c r="V11" s="3">
+        <f>P11/$O$11</f>
+        <v>0.27582403683185353</v>
+      </c>
+      <c r="W11" s="3">
+        <f t="shared" ref="W11:Z11" si="5">Q11/$O$11</f>
+        <v>8.5302673850901817E-2</v>
+      </c>
+      <c r="X11" s="3">
+        <f t="shared" si="5"/>
+        <v>2.2673766579815E-2</v>
+      </c>
+      <c r="Y11" s="3">
+        <f t="shared" si="5"/>
+        <v>2.1997082458492492E-2</v>
+      </c>
+      <c r="Z11" s="3">
+        <f t="shared" si="5"/>
+        <v>0.29043619775197527</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A12" s="15" t="s">
         <v>39</v>
       </c>
@@ -1272,13 +1445,13 @@
         <v>1.8539E-2</v>
       </c>
       <c r="L12">
-        <v>2.1269E-2</v>
+        <v>1.2364E-2</v>
       </c>
       <c r="M12">
         <v>8.1720000000000004E-3</v>
       </c>
       <c r="N12">
-        <v>7.2383000000000003E-2</v>
+        <v>7.0283999999999999E-2</v>
       </c>
       <c r="O12" s="1">
         <v>1.05287E-18</v>
@@ -1290,16 +1463,36 @@
         <v>5.91793E-20</v>
       </c>
       <c r="R12" s="1">
-        <v>6.7895300000000001E-20</v>
+        <v>3.94701E-20</v>
       </c>
       <c r="S12" s="1">
         <v>2.6087E-20</v>
       </c>
       <c r="T12" s="1">
-        <v>2.3106199999999998E-19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
+        <v>2.2436100000000001E-19</v>
+      </c>
+      <c r="V12" s="3">
+        <f>P12/$O$12</f>
+        <v>0.200575569633478</v>
+      </c>
+      <c r="W12" s="3">
+        <f t="shared" ref="W12:Z12" si="6">Q12/$O$12</f>
+        <v>5.6207603977699049E-2</v>
+      </c>
+      <c r="X12" s="4">
+        <f t="shared" si="6"/>
+        <v>3.7488103944456577E-2</v>
+      </c>
+      <c r="Y12" s="4">
+        <f t="shared" si="6"/>
+        <v>2.4777038000892797E-2</v>
+      </c>
+      <c r="Z12" s="3">
+        <f t="shared" si="6"/>
+        <v>0.21309468405406176</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A13" s="15" t="s">
         <v>40</v>
       </c>
@@ -1324,7 +1517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
         <v>41</v>
       </c>
@@ -1364,7 +1557,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A15" s="20"/>
       <c r="B15" s="29"/>
       <c r="C15" s="28"/>
@@ -1410,26 +1603,41 @@
       <c r="T15" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="V15" t="s">
+        <v>20</v>
+      </c>
+      <c r="W15" t="s">
+        <v>35</v>
+      </c>
+      <c r="X15" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A16" s="15" t="s">
         <v>45</v>
       </c>
       <c r="B16" s="14">
         <f>L6</f>
-        <v>2.8486000000000001E-2</v>
+        <v>1.6702999999999999E-2</v>
       </c>
       <c r="C16" s="12">
         <f>L12</f>
-        <v>2.1269E-2</v>
+        <v>1.2364E-2</v>
       </c>
       <c r="D16" s="12">
         <f>L18</f>
-        <v>4.0446999999999997E-2</v>
+        <v>2.8095999999999999E-2</v>
       </c>
       <c r="E16" s="12">
         <f>L24</f>
-        <v>3.4731999999999999E-2</v>
+        <v>2.8993000000000001E-2</v>
       </c>
       <c r="F16" s="2"/>
       <c r="H16" t="s">
@@ -1445,13 +1653,13 @@
         <v>3.5511000000000001E-2</v>
       </c>
       <c r="L16">
-        <v>2.9727E-2</v>
+        <v>2.9898000000000001E-2</v>
       </c>
       <c r="M16">
         <v>8.2430000000000003E-3</v>
       </c>
       <c r="N16">
-        <v>8.4183999999999995E-2</v>
+        <v>8.4243999999999999E-2</v>
       </c>
       <c r="O16" s="1">
         <v>1.72338E-18</v>
@@ -1463,34 +1671,54 @@
         <v>1.13359E-19</v>
       </c>
       <c r="R16" s="1">
-        <v>9.4894799999999998E-20</v>
+        <v>9.5440700000000003E-20</v>
       </c>
       <c r="S16" s="1">
         <v>2.6313399999999999E-20</v>
       </c>
       <c r="T16" s="1">
-        <v>2.6873299999999998E-19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
+        <v>2.6892699999999998E-19</v>
+      </c>
+      <c r="V16" s="3">
+        <f>P16/$O$16</f>
+        <v>0.12931970894405181</v>
+      </c>
+      <c r="W16" s="3">
+        <f t="shared" ref="W16:Z16" si="7">Q16/$O$16</f>
+        <v>6.5777135628822425E-2</v>
+      </c>
+      <c r="X16" s="3">
+        <f t="shared" si="7"/>
+        <v>5.5379951026471239E-2</v>
+      </c>
+      <c r="Y16" s="3">
+        <f t="shared" si="7"/>
+        <v>1.5268484025577643E-2</v>
+      </c>
+      <c r="Z16" s="3">
+        <f t="shared" si="7"/>
+        <v>0.15604625793498822</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A17" s="15" t="s">
         <v>46</v>
       </c>
       <c r="B17" s="14">
         <f>R6</f>
-        <v>9.0934599999999998E-20</v>
+        <v>5.3320400000000003E-20</v>
       </c>
       <c r="C17" s="14">
         <f>R12</f>
-        <v>6.7895300000000001E-20</v>
+        <v>3.94701E-20</v>
       </c>
       <c r="D17" s="14">
         <f>R18</f>
-        <v>1.2911700000000001E-19</v>
+        <v>8.9688600000000002E-20</v>
       </c>
       <c r="E17" s="14">
         <f>R24</f>
-        <v>1.10871E-19</v>
+        <v>9.2551400000000001E-20</v>
       </c>
       <c r="F17" s="2"/>
       <c r="H17" t="s">
@@ -1506,13 +1734,13 @@
         <v>4.3679999999999997E-2</v>
       </c>
       <c r="L17">
-        <v>4.8372999999999999E-2</v>
+        <v>2.0074999999999999E-2</v>
       </c>
       <c r="M17">
         <v>8.2430000000000003E-3</v>
       </c>
       <c r="N17">
-        <v>0.107322</v>
+        <v>9.7881999999999997E-2</v>
       </c>
       <c r="O17" s="1">
         <v>1.86217E-18</v>
@@ -1524,34 +1752,54 @@
         <v>1.39436E-19</v>
       </c>
       <c r="R17" s="1">
-        <v>1.54418E-19</v>
+        <v>6.4082299999999998E-20</v>
       </c>
       <c r="S17" s="1">
         <v>2.6313399999999999E-20</v>
       </c>
       <c r="T17" s="1">
-        <v>3.42595E-19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
+        <v>3.1246299999999998E-19</v>
+      </c>
+      <c r="V17" s="3">
+        <f>P17/$O$17</f>
+        <v>0.14548027301481603</v>
+      </c>
+      <c r="W17" s="3">
+        <f t="shared" ref="W17:Z17" si="8">Q17/$O$17</f>
+        <v>7.4878233458814183E-2</v>
+      </c>
+      <c r="X17" s="3">
+        <f t="shared" si="8"/>
+        <v>3.4412701310836284E-2</v>
+      </c>
+      <c r="Y17" s="3">
+        <f t="shared" si="8"/>
+        <v>1.4130503659708834E-2</v>
+      </c>
+      <c r="Z17" s="3">
+        <f t="shared" si="8"/>
+        <v>0.16779509926591019</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
         <v>47</v>
       </c>
       <c r="B18" s="16">
         <f>B17/B2</f>
-        <v>8.0666554302796969E-2</v>
+        <v>4.7299630086313195E-2</v>
       </c>
       <c r="C18" s="16">
-        <f t="shared" ref="B18:D18" si="1">C17/C2</f>
-        <v>6.4485928937095746E-2</v>
+        <f t="shared" ref="C18:D18" si="9">C17/C2</f>
+        <v>3.7488103944456577E-2</v>
       </c>
       <c r="D18" s="16">
-        <f t="shared" si="1"/>
-        <v>7.0084676762742229E-2</v>
+        <f t="shared" si="9"/>
+        <v>4.8682950659501713E-2</v>
       </c>
       <c r="E18" s="16">
         <f>E17/E2</f>
-        <v>7.0850880276064801E-2</v>
+        <v>5.9143943508962522E-2</v>
       </c>
       <c r="H18" t="s">
         <v>26</v>
@@ -1566,13 +1814,13 @@
         <v>2.8611000000000001E-2</v>
       </c>
       <c r="L18">
-        <v>4.0446999999999997E-2</v>
+        <v>2.8095999999999999E-2</v>
       </c>
       <c r="M18">
         <v>8.2430000000000003E-3</v>
       </c>
       <c r="N18">
-        <v>7.4123999999999995E-2</v>
+        <v>6.8173999999999998E-2</v>
       </c>
       <c r="O18" s="1">
         <v>1.8422999999999998E-18</v>
@@ -1584,16 +1832,36 @@
         <v>9.1332E-20</v>
       </c>
       <c r="R18" s="1">
-        <v>1.2911700000000001E-19</v>
+        <v>8.9688600000000002E-20</v>
       </c>
       <c r="S18" s="1">
         <v>2.6313399999999999E-20</v>
       </c>
       <c r="T18" s="1">
-        <v>2.3661900000000002E-19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
+        <v>2.1762600000000002E-19</v>
+      </c>
+      <c r="V18" s="3">
+        <f>P18/$O$18</f>
+        <v>9.4458557238234819E-2</v>
+      </c>
+      <c r="W18" s="3">
+        <f t="shared" ref="W18:Z18" si="10">Q18/$O$18</f>
+        <v>4.9574987787005378E-2</v>
+      </c>
+      <c r="X18" s="4">
+        <f t="shared" si="10"/>
+        <v>4.8682950659501713E-2</v>
+      </c>
+      <c r="Y18" s="4">
+        <f t="shared" si="10"/>
+        <v>1.4282907235520817E-2</v>
+      </c>
+      <c r="Z18" s="3">
+        <f t="shared" si="10"/>
+        <v>0.11812734082397006</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A19" s="26"/>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
@@ -1604,7 +1872,7 @@
         <v>8.0564875314760767E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A20" s="15" t="s">
         <v>62</v>
       </c>
@@ -1644,7 +1912,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A21" s="15" t="s">
         <v>63</v>
       </c>
@@ -1707,8 +1975,23 @@
       <c r="T21" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="V21" t="s">
+        <v>20</v>
+      </c>
+      <c r="W21" t="s">
+        <v>35</v>
+      </c>
+      <c r="X21" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A22" s="10" t="s">
         <v>64</v>
       </c>
@@ -1741,13 +2024,13 @@
         <v>2.8503000000000001E-2</v>
       </c>
       <c r="L22">
-        <v>2.6859000000000001E-2</v>
+        <v>2.3647000000000001E-2</v>
       </c>
       <c r="M22">
         <v>9.1450000000000004E-3</v>
       </c>
       <c r="N22">
-        <v>6.4920000000000005E-2</v>
+        <v>6.3658999999999993E-2</v>
       </c>
       <c r="O22" s="1">
         <v>1.40033E-18</v>
@@ -1759,16 +2042,36 @@
         <v>9.0988299999999996E-20</v>
       </c>
       <c r="R22" s="1">
-        <v>8.5739800000000005E-20</v>
+        <v>7.5487099999999998E-20</v>
       </c>
       <c r="S22" s="1">
         <v>2.91939E-20</v>
       </c>
       <c r="T22" s="1">
-        <v>2.0723999999999999E-19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
+        <v>2.0321299999999999E-19</v>
+      </c>
+      <c r="V22" s="3">
+        <f>P22/$O$22</f>
+        <v>0.11617547292423928</v>
+      </c>
+      <c r="W22" s="3">
+        <f t="shared" ref="W22:Z22" si="11">Q22/$O$22</f>
+        <v>6.4976327008633677E-2</v>
+      </c>
+      <c r="X22" s="3">
+        <f t="shared" si="11"/>
+        <v>5.3906650575221551E-2</v>
+      </c>
+      <c r="Y22" s="3">
+        <f t="shared" si="11"/>
+        <v>2.084787157312919E-2</v>
+      </c>
+      <c r="Z22" s="3">
+        <f t="shared" si="11"/>
+        <v>0.14511793648639962</v>
+      </c>
+    </row>
+    <row r="23" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A23" s="20"/>
       <c r="B23" s="17"/>
       <c r="C23" s="17"/>
@@ -1787,13 +2090,13 @@
         <v>3.9248999999999999E-2</v>
       </c>
       <c r="L23">
-        <v>4.3192000000000001E-2</v>
+        <v>3.4178E-2</v>
       </c>
       <c r="M23">
         <v>9.1450000000000004E-3</v>
       </c>
       <c r="N23">
-        <v>8.6036000000000001E-2</v>
+        <v>8.1881999999999996E-2</v>
       </c>
       <c r="O23" s="1">
         <v>1.73187E-18</v>
@@ -1805,16 +2108,36 @@
         <v>1.25292E-19</v>
       </c>
       <c r="R23" s="1">
-        <v>1.3787800000000001E-19</v>
+        <v>1.0910299999999999E-19</v>
       </c>
       <c r="S23" s="1">
         <v>2.91939E-20</v>
       </c>
       <c r="T23" s="1">
-        <v>2.74645E-19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
+        <v>2.6138600000000001E-19</v>
+      </c>
+      <c r="V23" s="3">
+        <f>P23/$O$23</f>
+        <v>0.11529271827562115</v>
+      </c>
+      <c r="W23" s="3">
+        <f t="shared" ref="W23:Z23" si="12">Q23/$O$23</f>
+        <v>7.2344921962964881E-2</v>
+      </c>
+      <c r="X23" s="3">
+        <f t="shared" si="12"/>
+        <v>6.2997222655280127E-2</v>
+      </c>
+      <c r="Y23" s="3">
+        <f t="shared" si="12"/>
+        <v>1.6856865700081415E-2</v>
+      </c>
+      <c r="Z23" s="3">
+        <f t="shared" si="12"/>
+        <v>0.15092703262946988</v>
+      </c>
+    </row>
+    <row r="24" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
         <v>16</v>
       </c>
@@ -1835,13 +2158,13 @@
         <v>2.4382000000000001E-2</v>
       </c>
       <c r="L24">
-        <v>3.4731999999999999E-2</v>
+        <v>2.8993000000000001E-2</v>
       </c>
       <c r="M24">
         <v>9.1450000000000004E-3</v>
       </c>
       <c r="N24">
-        <v>5.9006999999999997E-2</v>
+        <v>5.5821999999999997E-2</v>
       </c>
       <c r="O24" s="1">
         <v>1.56485E-18</v>
@@ -1853,96 +2176,116 @@
         <v>7.7833600000000003E-20</v>
       </c>
       <c r="R24" s="1">
-        <v>1.10871E-19</v>
+        <v>9.2551400000000001E-20</v>
       </c>
       <c r="S24" s="1">
         <v>2.91939E-20</v>
       </c>
       <c r="T24" s="1">
-        <v>1.8836200000000001E-19</v>
-      </c>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
+        <v>1.78195E-19</v>
+      </c>
+      <c r="V24" s="3">
+        <f>P24/$O$24</f>
+        <v>8.1530498130811258E-2</v>
+      </c>
+      <c r="W24" s="3">
+        <f t="shared" ref="W24:Z24" si="13">Q24/$O$24</f>
+        <v>4.9738696999712437E-2</v>
+      </c>
+      <c r="X24" s="4">
+        <f>R24/$O$24</f>
+        <v>5.9143943508962522E-2</v>
+      </c>
+      <c r="Y24" s="4">
+        <f t="shared" si="13"/>
+        <v>1.8656037319870915E-2</v>
+      </c>
+      <c r="Z24" s="3">
+        <f>T24/$O$24</f>
+        <v>0.11387353420455634</v>
+      </c>
+    </row>
+    <row r="25" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>13</v>
       </c>
       <c r="B25" s="12">
         <f>SQRT(B21^2+B13^2+B17^2+B9^2)</f>
-        <v>2.7118630187596129E-19</v>
+        <v>2.6099037128629865E-19</v>
       </c>
       <c r="C25" s="12">
-        <f t="shared" ref="C25:E25" si="2">SQRT(C21^2+C13^2+C17^2+C9^2)</f>
-        <v>2.3106164822310947E-19</v>
+        <f t="shared" ref="C25:E25" si="14">SQRT(C21^2+C13^2+C17^2+C9^2)</f>
+        <v>2.2436042946896852E-19</v>
       </c>
       <c r="D25" s="12">
-        <f t="shared" si="2"/>
-        <v>2.3661875955545029E-19</v>
+        <f t="shared" si="14"/>
+        <v>2.1762647507718358E-19</v>
       </c>
       <c r="E25" s="12">
-        <f t="shared" si="2"/>
-        <v>1.8836176261696533E-19</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
+        <f t="shared" si="14"/>
+        <v>1.7819522052268966E-19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A26" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B26" s="13">
         <f>B25/B2</f>
-        <v>0.24056480752597936</v>
+        <v>0.23152016897719188</v>
       </c>
       <c r="C26" s="13">
         <f>C25/C2</f>
-        <v>0.21945885838053081</v>
+        <v>0.21309414217231806</v>
       </c>
       <c r="D26" s="13">
         <f>D25/D2</f>
-        <v>0.12843660617459171</v>
+        <v>0.11812759869575183</v>
       </c>
       <c r="E26" s="16">
         <f>E25/E2</f>
-        <v>0.12037049085660947</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
+        <v>0.11387367512713018</v>
+      </c>
+    </row>
+    <row r="27" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A27" s="5"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A28" s="5"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="4"/>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.2">
       <c r="C29" s="1"/>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>27</v>
       </c>
       <c r="B30" s="1">
         <f>B3-B25</f>
-        <v>6.9812403869814024E-25</v>
+        <v>6.2871370136205462E-25</v>
       </c>
       <c r="C30" s="1">
         <f>C3-C25</f>
-        <v>3.5177689050995705E-25</v>
+        <v>5.7053103148958365E-25</v>
       </c>
       <c r="D30" s="1">
         <f>D3-D25</f>
-        <v>2.4044454973675999E-25</v>
+        <v>-4.7507718355804294E-25</v>
       </c>
       <c r="E30" s="1">
         <f>E3-E25</f>
-        <v>2.3738303468222868E-25</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
+        <v>-2.205226896586001E-25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B31" s="1">
         <f>SQRT(B23^2+C23^2+D23^2+E23^2)/4</f>
         <v>0</v>
@@ -1959,6 +2302,262 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8329FBAC-DBFC-0E46-9B7C-A44387D01939}">
+  <dimension ref="A1:N18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="17.5" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="12">
+        <v>1.12729E-18</v>
+      </c>
+      <c r="C2" s="12">
+        <v>1.05287E-18</v>
+      </c>
+      <c r="D2" s="12">
+        <v>1.8422999999999998E-18</v>
+      </c>
+      <c r="E2" s="12">
+        <v>1.56485E-18</v>
+      </c>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A3" s="36" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="14">
+        <v>2.7118699999999999E-19</v>
+      </c>
+      <c r="C3" s="14">
+        <v>2.3106199999999998E-19</v>
+      </c>
+      <c r="D3" s="14">
+        <v>2.3661900000000002E-19</v>
+      </c>
+      <c r="E3" s="14">
+        <v>1.8836200000000001E-19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A4" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="13">
+        <v>0.2405654268200729</v>
+      </c>
+      <c r="C4" s="13">
+        <v>0.21945919249290033</v>
+      </c>
+      <c r="D4" s="13">
+        <v>0.1284367366878359</v>
+      </c>
+      <c r="E4" s="13">
+        <v>0.12037064255359939</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A8" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="12">
+        <v>2.32968E-20</v>
+      </c>
+      <c r="C8" s="12">
+        <v>2.6087E-20</v>
+      </c>
+      <c r="D8" s="12">
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="E8" s="12">
+        <v>2.91939E-20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="16">
+        <v>2.0666199469524256E-2</v>
+      </c>
+      <c r="C9" s="16">
+        <v>2.4777038000892797E-2</v>
+      </c>
+      <c r="D9" s="16">
+        <v>1.4282907235520817E-2</v>
+      </c>
+      <c r="E9" s="16">
+        <v>1.8656037319870915E-2</v>
+      </c>
+      <c r="F9" s="33"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="12">
+        <v>6.0562399999999996E-20</v>
+      </c>
+      <c r="C11" s="12">
+        <v>5.91793E-20</v>
+      </c>
+      <c r="D11" s="12">
+        <v>9.1332E-20</v>
+      </c>
+      <c r="E11" s="12">
+        <v>7.7833600000000003E-20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A12" s="34" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="16">
+        <v>5.3723886488836053E-2</v>
+      </c>
+      <c r="C12" s="16">
+        <v>5.6207603977699049E-2</v>
+      </c>
+      <c r="D12" s="16">
+        <v>4.9574987787005378E-2</v>
+      </c>
+      <c r="E12" s="16">
+        <v>4.9738696999712437E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="12">
+        <v>9.0934599999999998E-20</v>
+      </c>
+      <c r="C14" s="12">
+        <v>6.7895300000000001E-20</v>
+      </c>
+      <c r="D14" s="12">
+        <v>1.2911700000000001E-19</v>
+      </c>
+      <c r="E14" s="12">
+        <v>1.10871E-19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A15" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="16">
+        <v>8.0666554302796969E-2</v>
+      </c>
+      <c r="C15" s="16">
+        <v>6.4485928937095746E-2</v>
+      </c>
+      <c r="D15" s="16">
+        <v>7.0084676762742229E-2</v>
+      </c>
+      <c r="E15" s="16">
+        <v>7.0850880276064801E-2</v>
+      </c>
+      <c r="F15" s="33"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="B17" s="12">
+        <v>2.4710800000000001E-19</v>
+      </c>
+      <c r="C17" s="12">
+        <v>2.1118E-19</v>
+      </c>
+      <c r="D17" s="12">
+        <v>1.74021E-19</v>
+      </c>
+      <c r="E17" s="12">
+        <v>1.2758299999999999E-19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18" s="13">
+        <v>0.21920535088575258</v>
+      </c>
+      <c r="C18" s="13">
+        <v>0.200575569633478</v>
+      </c>
+      <c r="D18" s="16">
+        <v>9.4458557238234819E-2</v>
+      </c>
+      <c r="E18" s="16">
+        <v>8.1530498130811258E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1B35896-C4A9-3544-8AEE-A53C2900D99C}">
   <dimension ref="A1:Q29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1969,7 +2568,7 @@
     <col min="5" max="5" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1991,7 +2590,7 @@
       </c>
       <c r="B2" s="12">
         <f>K6</f>
-        <v>5.3435399999999998E-18</v>
+        <v>5.3431799999999999E-18</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" t="e">
@@ -2017,7 +2616,7 @@
       </c>
       <c r="B3" s="14">
         <f>O6</f>
-        <v>4.9916800000000003E-19</v>
+        <v>4.5062399999999997E-19</v>
       </c>
       <c r="C3" s="1"/>
       <c r="E3" t="s">
@@ -2060,41 +2659,41 @@
       </c>
       <c r="B4" s="13">
         <f>B3/B2</f>
-        <v>9.3415226610074981E-2</v>
+        <v>8.433629411698651E-2</v>
       </c>
       <c r="C4" s="2"/>
       <c r="E4" t="s">
         <v>52</v>
       </c>
       <c r="F4">
-        <v>1.666417</v>
+        <v>1.666458</v>
       </c>
       <c r="G4">
         <v>9.6518999999999994E-2</v>
       </c>
       <c r="H4">
-        <v>9.8921999999999996E-2</v>
+        <v>9.8926E-2</v>
       </c>
       <c r="I4">
-        <v>9.7372E-2</v>
+        <v>8.3470000000000003E-2</v>
       </c>
       <c r="J4">
-        <v>0.16906499999999999</v>
+        <v>0.16145999999999999</v>
       </c>
       <c r="K4" s="1">
-        <v>5.3195699999999998E-18</v>
+        <v>5.3197000000000003E-18</v>
       </c>
       <c r="L4" s="1">
-        <v>3.0810900000000001E-19</v>
+        <v>3.08111E-19</v>
       </c>
       <c r="M4" s="1">
-        <v>3.1578300000000001E-19</v>
+        <v>3.1579299999999999E-19</v>
       </c>
       <c r="N4" s="1">
-        <v>3.1083399999999998E-19</v>
+        <v>2.6645400000000001E-19</v>
       </c>
       <c r="O4" s="1">
-        <v>5.3969299999999996E-19</v>
+        <v>5.1541700000000005E-19</v>
       </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
@@ -2106,34 +2705,34 @@
         <v>53</v>
       </c>
       <c r="F5">
-        <v>1.68001</v>
+        <v>1.678785</v>
       </c>
       <c r="G5">
         <v>0.111913</v>
       </c>
       <c r="H5">
-        <v>0.109622</v>
+        <v>0.10954700000000001</v>
       </c>
       <c r="I5">
-        <v>0.13072600000000001</v>
+        <v>9.8524E-2</v>
       </c>
       <c r="J5">
-        <v>0.204036</v>
+        <v>0.18501899999999999</v>
       </c>
       <c r="K5" s="1">
-        <v>5.3629600000000002E-18</v>
+        <v>5.35905E-18</v>
       </c>
       <c r="L5" s="1">
         <v>3.5725000000000002E-19</v>
       </c>
       <c r="M5" s="1">
-        <v>3.4993899999999999E-19</v>
+        <v>3.4969900000000001E-19</v>
       </c>
       <c r="N5" s="1">
-        <v>4.1730699999999999E-19</v>
+        <v>3.1450899999999998E-19</v>
       </c>
       <c r="O5" s="1">
-        <v>6.5132899999999995E-19</v>
+        <v>5.9062100000000001E-19</v>
       </c>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
@@ -2147,34 +2746,34 @@
         <v>54</v>
       </c>
       <c r="F6">
-        <v>1.673926</v>
+        <v>1.673813</v>
       </c>
       <c r="G6">
-        <v>7.3662000000000005E-2</v>
+        <v>7.3661000000000004E-2</v>
       </c>
       <c r="H6">
-        <v>7.8446000000000002E-2</v>
+        <v>7.8441999999999998E-2</v>
       </c>
       <c r="I6">
-        <v>0.113454</v>
+        <v>9.1367000000000004E-2</v>
       </c>
       <c r="J6">
-        <v>0.15637000000000001</v>
+        <v>0.14116300000000001</v>
       </c>
       <c r="K6" s="1">
-        <v>5.3435399999999998E-18</v>
+        <v>5.3431799999999999E-18</v>
       </c>
       <c r="L6" s="1">
         <v>2.35144E-19</v>
       </c>
       <c r="M6" s="1">
-        <v>2.5041800000000001E-19</v>
+        <v>2.5040300000000001E-19</v>
       </c>
       <c r="N6" s="1">
-        <v>3.6217E-19</v>
+        <v>2.9166300000000001E-19</v>
       </c>
       <c r="O6" s="1">
-        <v>4.9916800000000003E-19</v>
+        <v>4.5062399999999997E-19</v>
       </c>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
@@ -2185,7 +2784,7 @@
       </c>
       <c r="B8" s="14">
         <f>H6</f>
-        <v>7.8446000000000002E-2</v>
+        <v>7.8441999999999998E-2</v>
       </c>
       <c r="C8" s="1"/>
     </row>
@@ -2195,7 +2794,7 @@
       </c>
       <c r="B9" s="14">
         <f>M6</f>
-        <v>2.5041800000000001E-19</v>
+        <v>2.5040300000000001E-19</v>
       </c>
       <c r="C9" s="1"/>
     </row>
@@ -2205,7 +2804,7 @@
       </c>
       <c r="B10" s="16">
         <f>B9/B2</f>
-        <v>4.6863689614001211E-2</v>
+        <v>4.6864039766580955E-2</v>
       </c>
       <c r="C10" s="2"/>
       <c r="K10" s="1"/>
@@ -2241,26 +2840,31 @@
       </c>
       <c r="B12" s="14">
         <f>I6</f>
-        <v>0.113454</v>
+        <v>9.1367000000000004E-2</v>
       </c>
       <c r="C12" s="1"/>
       <c r="E12" t="s">
         <v>58</v>
       </c>
       <c r="F12" s="1">
-        <v>5.3195699999999998E-18</v>
+        <f>K4</f>
+        <v>5.3197000000000003E-18</v>
       </c>
       <c r="G12" s="1">
-        <v>3.0810900000000001E-19</v>
+        <f>L4</f>
+        <v>3.08111E-19</v>
       </c>
       <c r="H12" s="1">
-        <v>3.1578300000000001E-19</v>
+        <f>M4</f>
+        <v>3.1579299999999999E-19</v>
       </c>
       <c r="I12" s="1">
-        <v>3.1083399999999998E-19</v>
+        <f>N4</f>
+        <v>2.6645400000000001E-19</v>
       </c>
       <c r="J12" s="1">
-        <v>5.3969299999999996E-19</v>
+        <f>O4</f>
+        <v>5.1541700000000005E-19</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
@@ -2271,26 +2875,31 @@
       </c>
       <c r="B13" s="14">
         <f>N6</f>
-        <v>3.6217E-19</v>
+        <v>2.9166300000000001E-19</v>
       </c>
       <c r="C13" s="1"/>
       <c r="E13" t="s">
         <v>59</v>
       </c>
       <c r="F13" s="1">
-        <v>5.3629600000000002E-18</v>
+        <f>K5</f>
+        <v>5.35905E-18</v>
       </c>
       <c r="G13" s="1">
+        <f t="shared" ref="G13:G14" si="0">L5</f>
         <v>3.5725000000000002E-19</v>
       </c>
       <c r="H13" s="1">
-        <v>3.4993899999999999E-19</v>
+        <f t="shared" ref="H13:J13" si="1">M5</f>
+        <v>3.4969900000000001E-19</v>
       </c>
       <c r="I13" s="1">
-        <v>4.1730699999999999E-19</v>
+        <f t="shared" si="1"/>
+        <v>3.1450899999999998E-19</v>
       </c>
       <c r="J13" s="1">
-        <v>6.5132899999999995E-19</v>
+        <f t="shared" si="1"/>
+        <v>5.9062100000000001E-19</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
@@ -2299,26 +2908,31 @@
       </c>
       <c r="B14" s="16">
         <f>B13/B2</f>
-        <v>6.7777166447710702E-2</v>
+        <v>5.4586033036506353E-2</v>
       </c>
       <c r="C14" s="2"/>
       <c r="E14" t="s">
         <v>60</v>
       </c>
       <c r="F14" s="1">
-        <v>5.3435399999999998E-18</v>
+        <f>K6</f>
+        <v>5.3431799999999999E-18</v>
       </c>
       <c r="G14" s="1">
+        <f t="shared" si="0"/>
         <v>2.35144E-19</v>
       </c>
       <c r="H14" s="1">
-        <v>2.5041800000000001E-19</v>
+        <f>M6</f>
+        <v>2.5040300000000001E-19</v>
       </c>
       <c r="I14" s="1">
-        <v>3.6217E-19</v>
+        <f>N6</f>
+        <v>2.9166300000000001E-19</v>
       </c>
       <c r="J14" s="1">
-        <v>4.9916800000000003E-19</v>
+        <f t="shared" ref="J14" si="2">O6</f>
+        <v>4.5062399999999997E-19</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
@@ -2332,9 +2946,25 @@
       </c>
       <c r="B16" s="14">
         <f>G6</f>
-        <v>7.3662000000000005E-2</v>
+        <v>7.3661000000000004E-2</v>
       </c>
       <c r="C16" s="2"/>
+      <c r="G16" s="4">
+        <f>(G12/$F$12)</f>
+        <v>5.7918867605316088E-2</v>
+      </c>
+      <c r="H16" s="4">
+        <f>(H12/$F$12)</f>
+        <v>5.9362934000037587E-2</v>
+      </c>
+      <c r="I16" s="4">
+        <f t="shared" ref="H16:J16" si="3">(I12/$F$12)</f>
+        <v>5.008816286632705E-2</v>
+      </c>
+      <c r="J16" s="4">
+        <f t="shared" si="3"/>
+        <v>9.6888358366073277E-2</v>
+      </c>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
@@ -2351,6 +2981,22 @@
         <v>2.35144E-19</v>
       </c>
       <c r="C17" s="2"/>
+      <c r="G17" s="4">
+        <f>(G13/$F$13)</f>
+        <v>6.666293466192702E-2</v>
+      </c>
+      <c r="H17" s="4">
+        <f t="shared" ref="H17:J17" si="4">(H13/$F$13)</f>
+        <v>6.5253916272473664E-2</v>
+      </c>
+      <c r="I17" s="4">
+        <f t="shared" si="4"/>
+        <v>5.8687453933066493E-2</v>
+      </c>
+      <c r="J17" s="3">
+        <f t="shared" si="4"/>
+        <v>0.11021001856672358</v>
+      </c>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
@@ -2364,7 +3010,23 @@
       </c>
       <c r="B18" s="13">
         <f>B17/B2</f>
-        <v>4.4005284886049323E-2</v>
+        <v>4.4008249768864235E-2</v>
+      </c>
+      <c r="G18" s="4">
+        <f>(G14/$F$14)</f>
+        <v>4.4008249768864235E-2</v>
+      </c>
+      <c r="H18" s="4">
+        <f t="shared" ref="H18:J18" si="5">(H14/$F$14)</f>
+        <v>4.6864039766580955E-2</v>
+      </c>
+      <c r="I18" s="4">
+        <f t="shared" si="5"/>
+        <v>5.4586033036506353E-2</v>
+      </c>
+      <c r="J18" s="4">
+        <f t="shared" si="5"/>
+        <v>8.433629411698651E-2</v>
       </c>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
@@ -2391,7 +3053,7 @@
       </c>
       <c r="B21" s="12">
         <f>SQRT(B17^2+B9^2+B13^2)</f>
-        <v>4.991682926228388E-19</v>
+        <v>4.5062364420212124E-19</v>
       </c>
       <c r="C21" s="2"/>
     </row>
@@ -2401,7 +3063,7 @@
       </c>
       <c r="B22" s="13">
         <f>B21/B2</f>
-        <v>9.34152813720565E-2</v>
+        <v>8.4336227527824492E-2</v>
       </c>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
@@ -2436,7 +3098,7 @@
       </c>
       <c r="B26" s="1">
         <f>B3-B21</f>
-        <v>-2.926228387736565E-25</v>
+        <v>3.557978787293963E-25</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
@@ -2455,7 +3117,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C3FC9BD-960C-B249-A82F-F026B7E24375}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3510,7 +4172,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0226FEE3-3B95-A74A-B9AB-147435730300}">
   <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4579,7 +5241,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{573F644D-04DC-0A40-95E2-DB07317B8B26}">
   <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5648,7 +6310,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59F09356-A4A4-3041-AE57-635F1ED1227C}">
   <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>